<commit_message>
feat(F-NAR-016): TREE-DIF-056 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-DIF-056.xlsx
+++ b/stories/arbres/TREE-DIF-056.xlsx
@@ -1197,12 +1197,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le gravier du parc est encore chaud. Un pétale de tilleul colle à la chaussure de Nina. Ça sent le miel, et la poussière. Tu as vu le bronze, Nina ? Le petit garçon, avec l'oiseau. Son nez brille encore, tout rond. En ce moment, Nina ouvre le savon, tout doux. Je veux une bulle, sur son nez. La cloche du parc va sonner bientôt. On prend les affaires, alors ? Merci, tu as essuyé le bâton.</t>
+          <t>Sous les tilleuls, le parc retient encore la chaleur. Un pétale jaune se colle au lacet de Nina. Ça sent le miel chaud, et le gravier. Tu as vu le petit bronze, Nina ? Il tient un oiseau, tout près du nez. Le nez est lisse, encore chaud. En ce moment, Nina souffle dans ses mains, vides. Je veux une bulle, collée là. La cloche va fermer le parc. On emporte le savon, alors ? Merci, tu as essuyé le bâton.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le gravier du parc est encore chaud. Un pétale de tilleul colle à la chaussure de Nina. Ça sent le miel, et la poussière. Tu as vu le bronze, Nina ? Le petit garçon, avec l'oiseau. Son nez brille encore, tout rond. En ce moment, Nina ouvre le savon, tout doux. Je veux une bulle, sur son nez. La cloche du parc va sonner bientôt. On prend les affaires, alors ? Merci, tu as essuyé le bâton.</t>
+          <t>Sous les tilleuls, le parc retient encore la chaleur. Un pétale jaune se colle au lacet de Nina. Ça sent le miel chaud, et le gravier. Tu as vu le petit bronze, Nina ? Il tient un oiseau, tout près du nez. Le nez est lisse, encore chaud. En ce moment, Nina souffle dans ses mains, vides. Je veux une bulle, collée là. La cloche va fermer le parc. On emporte le savon, alors ? Merci, tu as essuyé le bâton.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -1337,16 +1337,16 @@
       <c r="AV2" s="2" t="inlineStr"/>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le gravier du parc est encore chaud.
-narrateur|Un pétale de tilleul colle à la chaussure de Nina.
-narrateur|Ça sent le miel, et la poussière.
-papa|Tu as vu le bronze, Nina ?
-enfant-f|Le petit garçon, avec l'oiseau.
-maman|Son nez brille encore, tout rond.
-narrateur|En ce moment, Nina ouvre le savon, tout doux.
-enfant-f|Je veux une bulle, sur son nez.
-papa|La cloche du parc va sonner bientôt.
-maman|On prend les affaires, alors ?
+          <t>narrateur|Sous les tilleuls, le parc retient encore la chaleur.
+narrateur|Un pétale jaune se colle au lacet de Nina.
+narrateur|Ça sent le miel chaud, et le gravier.
+papa|Tu as vu le petit bronze, Nina ?
+enfant-f|Il tient un oiseau, tout près du nez.
+maman|Le nez est lisse, encore chaud.
+narrateur|En ce moment, Nina souffle dans ses mains, vides.
+enfant-f|Je veux une bulle, collée là.
+papa|La cloche va fermer le parc.
+maman|On emporte le savon, alors ?
 papa|Merci, tu as essuyé le bâton.</t>
         </is>
       </c>
@@ -1379,12 +1379,12 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Trois affaires attendent près du gravier. Le bâton, le savon, et la coupelle. Tu prends quoi d'abord, Nina ?</t>
+          <t>Près du lacet, trois affaires attendent. Un bâton, un savon, une coupelle. Par quoi tu commences, Nina ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Trois affaires attendent près du gravier. Le bâton, le savon, et la coupelle. Tu prends quoi d'abord, Nina ?</t>
+          <t>Près du lacet, trois affaires attendent. Un bâton, un savon, une coupelle. Par quoi tu commences, Nina ?</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -1543,9 +1543,9 @@
       <c r="AV3" s="2" t="inlineStr"/>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Trois affaires attendent près du gravier.
-narrateur|Le bâton, le savon, et la coupelle.
-maman|Tu prends quoi d'abord, Nina ?</t>
+          <t>narrateur|Près du lacet, trois affaires attendent.
+narrateur|Un bâton, un savon, une coupelle.
+maman|Par quoi tu commences, Nina ?</t>
         </is>
       </c>
     </row>
@@ -1572,12 +1572,12 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Nina prend d'abord le bâton, encore un peu humide. Il va porter la bulle. Tiens-le droit, tout doux. Un fil de savon tremble au bout, puis tient. Le savon aussi, près de toi. Maman glisse la coupelle contre son coude. Bâton, savon et coupelle avancent avec elle. J'arrive, petit nez. Le bois sent le savon, un peu sucré. Le bâton d'abord, vous l'avez.</t>
+          <t>Nina attrape d'abord le bâton, encore mouillé. La bulle va s'y accrocher. Garde le cercle en l'air. Un film tremble au bout, puis tient. Prends le savon, il est à tes pieds. La coupelle glisse sous son autre bras. Les trois partent, collés à Nina. Nez, j'arrive. Le bois sent le sucre, un peu. Le bâton est à toi, maintenant.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Nina prend d'abord le bâton, encore un peu humide. Il va porter la bulle. Tiens-le droit, tout doux. Un fil de savon tremble au bout, puis tient. Le savon aussi, près de toi. Maman glisse la coupelle contre son coude. Bâton, savon et coupelle avancent avec elle. J'arrive, petit nez. Le bois sent le savon, un peu sucré. Le bâton d'abord, vous l'avez.</t>
+          <t>Nina attrape d'abord le bâton, encore mouillé. La bulle va s'y accrocher. Garde le cercle en l'air. Un film tremble au bout, puis tient. Prends le savon, il est à tes pieds. La coupelle glisse sous son autre bras. Les trois partent, collés à Nina. Nez, j'arrive. Le bois sent le sucre, un peu. Le bâton est à toi, maintenant.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1712,16 +1712,16 @@
       <c r="AV4" s="2" t="inlineStr"/>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Nina prend d'abord le bâton, encore un peu humide.
-enfant-f|Il va porter la bulle.
-maman|Tiens-le droit, tout doux.
-narrateur|Un fil de savon tremble au bout, puis tient.
-papa|Le savon aussi, près de toi.
-narrateur|Maman glisse la coupelle contre son coude.
-narrateur|Bâton, savon et coupelle avancent avec elle.
-enfant-f|J'arrive, petit nez.
-narrateur|Le bois sent le savon, un peu sucré.
-papa|Le bâton d'abord, vous l'avez.</t>
+          <t>narrateur|Nina attrape d'abord le bâton, encore mouillé.
+enfant-f|La bulle va s'y accrocher.
+maman|Garde le cercle en l'air.
+narrateur|Un film tremble au bout, puis tient.
+papa|Prends le savon, il est à tes pieds.
+narrateur|La coupelle glisse sous son autre bras.
+narrateur|Les trois partent, collés à Nina.
+enfant-f|Nez, j'arrive.
+narrateur|Le bois sent le sucre, un peu.
+papa|Le bâton est à toi, maintenant.</t>
         </is>
       </c>
     </row>
@@ -1932,12 +1932,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le bâton tient contre sa poitrine, encore humide. Il va jusqu'au bronze. La cloche n'attendra pas longtemps. On y va, Nina ? Oui, papa. Un fil de savon cherche encore l'air.</t>
+          <t>Le bâton reste contre elle, encore mouillé. On va jusqu'au bronze. La cloche n'est pas loin. Tu tiens bien, Nina ? Oui, papa. Un fil de savon cherche encore l'air.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le bâton tient contre sa poitrine, encore humide. Il va jusqu'au bronze. La cloche n'attendra pas longtemps. On y va, Nina ? Oui, papa. Un fil de savon cherche encore l'air.</t>
+          <t>Le bâton reste contre elle, encore mouillé. On va jusqu'au bronze. La cloche n'est pas loin. Tu tiens bien, Nina ? Oui, papa. Un fil de savon cherche encore l'air.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -2076,10 +2076,10 @@
       </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le bâton tient contre sa poitrine, encore humide.
-enfant-f|Il va jusqu'au bronze.
-maman|La cloche n'attendra pas longtemps.
-papa|On y va, Nina ?
+          <t>narrateur|Le bâton reste contre elle, encore mouillé.
+enfant-f|On va jusqu'au bronze.
+maman|La cloche n'est pas loin.
+papa|Tu tiens bien, Nina ?
 enfant-f|Oui, papa.
 narrateur|Un fil de savon cherche encore l'air.</t>
         </is>
@@ -2108,12 +2108,12 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Le bâton tape sa paume, tout bas. L'allée soulève déjà trop de poussière. Plus loin, le socle brûle encore. Sous le tilleul, les feuilles claquent. Nina, vous partez où ?</t>
+          <t>Le bâton penche vers le bronze, déjà. Devant, l'allée soulève trop de poussière. Le socle, lui, brûle encore au soleil. Sous le tilleul, les feuilles claquent. Nina, tu vas où ?</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Le bâton tape sa paume, tout bas. L'allée soulève déjà trop de poussière. Plus loin, le socle brûle encore. Sous le tilleul, les feuilles claquent. Nina, vous partez où ?</t>
+          <t>Le bâton penche vers le bronze, déjà. Devant, l'allée soulève trop de poussière. Le socle, lui, brûle encore au soleil. Sous le tilleul, les feuilles claquent. Nina, tu vas où ?</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -2272,11 +2272,11 @@
       <c r="AV7" s="2" t="inlineStr"/>
       <c r="AW7" t="inlineStr">
         <is>
-          <t>narrateur|Le bâton tape sa paume, tout bas.
-narrateur|L'allée soulève déjà trop de poussière.
-narrateur|Plus loin, le socle brûle encore.
+          <t>narrateur|Le bâton penche vers le bronze, déjà.
+narrateur|Devant, l'allée soulève trop de poussière.
+narrateur|Le socle, lui, brûle encore au soleil.
 narrateur|Sous le tilleul, les feuilles claquent.
-papa|Nina, vous partez où ?</t>
+papa|Nina, tu vas où ?</t>
         </is>
       </c>
     </row>
@@ -2303,12 +2303,12 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Entre ses doigts, le bois du bâton est tiède. L'allée sent le gravier chaud, trop vif. Le fil se casse, trop vite, trop fort. Ma bulle a sauté ! Un pas soulève la poussière, encore. La bulle n'a plus le temps d'arriver. Ça bouge trop, ici. Elle a besoin de calme. On fait comment, alors ? Tu trouves, Nina ?</t>
+          <t>Entre ses doigts, le bois du bâton est tiède. Le gravier de l'allée saute sous les pas. Le fil se casse, trop vite, trop fort. Ma bulle a crevé ! Encore un pas, encore de la poussière. Le nez reste trop loin, trop gris. Ici, ça n'arrête pas. La bulle a besoin de calme. Alors on fait quoi ? Tu vois comment, Nina ?</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Entre ses doigts, le bois du bâton est tiède. L'allée sent le gravier chaud, trop vif. Le fil se casse, trop vite, trop fort. Ma bulle a sauté ! Un pas soulève la poussière, encore. La bulle n'a plus le temps d'arriver. Ça bouge trop, ici. Elle a besoin de calme. On fait comment, alors ? Tu trouves, Nina ?</t>
+          <t>Entre ses doigts, le bois du bâton est tiède. Le gravier de l'allée saute sous les pas. Le fil se casse, trop vite, trop fort. Ma bulle a crevé ! Encore un pas, encore de la poussière. Le nez reste trop loin, trop gris. Ici, ça n'arrête pas. La bulle a besoin de calme. Alors on fait quoi ? Tu vois comment, Nina ?</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -2444,15 +2444,15 @@
       <c r="AW8" t="inlineStr">
         <is>
           <t>narrateur|Entre ses doigts, le bois du bâton est tiède.
-narrateur|L'allée sent le gravier chaud, trop vif.
+narrateur|Le gravier de l'allée saute sous les pas.
 narrateur|Le fil se casse, trop vite, trop fort.
-enfant-f|Ma bulle a sauté !
-narrateur|Un pas soulève la poussière, encore.
-narrateur|La bulle n'a plus le temps d'arriver.
-papa|Ça bouge trop, ici.
-maman|Elle a besoin de calme.
-enfant-f|On fait comment, alors ?
-papa|Tu trouves, Nina ?</t>
+enfant-f|Ma bulle a crevé !
+narrateur|Encore un pas, encore de la poussière.
+narrateur|Le nez reste trop loin, trop gris.
+papa|Ici, ça n'arrête pas.
+maman|La bulle a besoin de calme.
+enfant-f|Alors on fait quoi ?
+papa|Tu vois comment, Nina ?</t>
         </is>
       </c>
     </row>
@@ -2479,12 +2479,12 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>L'allée soulève encore trop de poussière. Attendre les pas, plus bas, ou le bord ?</t>
+          <t>L'allée n'a pas fini de soulever. Attendre les pas, plus bas, ou le bord ?</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>L'allée soulève encore trop de poussière. Attendre les pas, plus bas, ou le bord ?</t>
+          <t>L'allée n'a pas fini de soulever. Attendre les pas, plus bas, ou le bord ?</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -2647,7 +2647,7 @@
       </c>
       <c r="AW9" t="inlineStr">
         <is>
-          <t>narrateur|L'allée soulève encore trop de poussière.
+          <t>narrateur|L'allée n'a pas fini de soulever.
 papa|Attendre les pas, plus bas, ou le bord ?</t>
         </is>
       </c>
@@ -2675,12 +2675,12 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>On attend les pas. Elle tient le bâton, sans souffler encore. Le gravier se tait, une fois, puis plus. Tu peux partir, maintenant. Pendant ce temps, le bâton reste droit, sage. Les pas se sont tus, maintenant. La bulle part, ronde, tout calme. Tu lui as laissé le temps.</t>
+          <t>On attend les pas. Elle tient le bâton, sans souffler encore. Le gravier se tait, une fois, puis plus. Tu peux partir, maintenant. Pendant ce temps, le bâton reste droit, sans bouger. Les pas se sont tus, maintenant. La bulle part, ronde, tout calme. Tu as attendu, et elle est partie.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>On attend les pas. Elle tient le bâton, sans souffler encore. Le gravier se tait, une fois, puis plus. Tu peux partir, maintenant. Pendant ce temps, le bâton reste droit, sage. Les pas se sont tus, maintenant. La bulle part, ronde, tout calme. Tu lui as laissé le temps.</t>
+          <t>On attend les pas. Elle tient le bâton, sans souffler encore. Le gravier se tait, une fois, puis plus. Tu peux partir, maintenant. Pendant ce temps, le bâton reste droit, sans bouger. Les pas se sont tus, maintenant. La bulle part, ronde, tout calme. Tu as attendu, et elle est partie.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -2819,10 +2819,10 @@
 narrateur|Elle tient le bâton, sans souffler encore.
 narrateur|Le gravier se tait, une fois, puis plus.
 enfant-f|Tu peux partir, maintenant.
-narrateur|Pendant ce temps, le bâton reste droit, sage.
+narrateur|Pendant ce temps, le bâton reste droit, sans bouger.
 papa|Les pas se sont tus, maintenant.
 narrateur|La bulle part, ronde, tout calme.
-maman|Tu lui as laissé le temps.</t>
+maman|Tu as attendu, et elle est partie.</t>
         </is>
       </c>
     </row>
@@ -2849,12 +2849,12 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>La bulle se pose, ronde, sur le nez de bronze. On a attendu les pas. Merci d'avoir laissé le gravier se taire. Rentrez, la cloche n'a pas encore sonné. Le bâton sèche près du savon, un fil encore collant. Une poussière tourne encore, puis s'arrête.</t>
+          <t>La bulle se pose, ronde, sur le nez de bronze. On a attendu les pas. Merci d'avoir laissé le gravier se taire. La cloche n'a pas encore sonné. Le bâton sèche près du savon, un fil encore collant. Un grain de poussière retombe, puis plus rien.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>La bulle se pose, ronde, sur le nez de bronze. On a attendu les pas. Merci d'avoir laissé le gravier se taire. Rentrez, la cloche n'a pas encore sonné. Le bâton sèche près du savon, un fil encore collant. Une poussière tourne encore, puis s'arrête.</t>
+          <t>La bulle se pose, ronde, sur le nez de bronze. On a attendu les pas. Merci d'avoir laissé le gravier se taire. La cloche n'a pas encore sonné. Le bâton sèche près du savon, un fil encore collant. Un grain de poussière retombe, puis plus rien.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -2992,9 +2992,9 @@
           <t>narrateur|La bulle se pose, ronde, sur le nez de bronze.
 enfant-f|On a attendu les pas.
 papa|Merci d'avoir laissé le gravier se taire.
-maman|Rentrez, la cloche n'a pas encore sonné.
+maman|La cloche n'a pas encore sonné.
 narrateur|Le bâton sèche près du savon, un fil encore collant.
-narrateur|Une poussière tourne encore, puis s'arrête.</t>
+narrateur|Un grain de poussière retombe, puis plus rien.</t>
         </is>
       </c>
     </row>
@@ -3021,12 +3021,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Plus bas, d'abord. Elle baisse le bâton, loin de la poussière. Nina s'accroupit, les genoux au gravier. L'air est plus doux, près de l'herbe. Un fil de savon cherche encore l'air. Tu as regardé d'abord. Ici, tu ne sautes plus. Le bas était plus calme.</t>
+          <t>Plus bas, d'abord. Elle baisse le bâton, loin de la poussière. Nina s'accroupit, les genoux au gravier. L'air est plus doux, près de l'herbe. Un fil de savon cherche encore l'air. Tu as vu l'herbe, avant. Ici, tu ne crèves plus. Près du sol, ça tenait mieux.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Plus bas, d'abord. Elle baisse le bâton, loin de la poussière. Nina s'accroupit, les genoux au gravier. L'air est plus doux, près de l'herbe. Un fil de savon cherche encore l'air. Tu as regardé d'abord. Ici, tu ne sautes plus. Le bas était plus calme.</t>
+          <t>Plus bas, d'abord. Elle baisse le bâton, loin de la poussière. Nina s'accroupit, les genoux au gravier. L'air est plus doux, près de l'herbe. Un fil de savon cherche encore l'air. Tu as vu l'herbe, avant. Ici, tu ne crèves plus. Près du sol, ça tenait mieux.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -3166,9 +3166,9 @@
 narrateur|Nina s'accroupit, les genoux au gravier.
 narrateur|L'air est plus doux, près de l'herbe.
 narrateur|Un fil de savon cherche encore l'air.
-papa|Tu as regardé d'abord.
-enfant-f|Ici, tu ne sautes plus.
-maman|Le bas était plus calme.</t>
+papa|Tu as vu l'herbe, avant.
+enfant-f|Ici, tu ne crèves plus.
+maman|Près du sol, ça tenait mieux.</t>
         </is>
       </c>
     </row>
@@ -3195,12 +3195,12 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Plus bas, la bulle monte jusqu'au nez. On s'est baissées, d'abord. Tu as regardé avant de souffler. Essuie tes genoux, sur le paillasson. Le bâton sèche près du savon, un fil encore collant. Un rond d'ombre reste au bas du bronze.</t>
+          <t>Plus bas, la bulle monte jusqu'au nez. On s'est baissées, d'abord. Tu as vu l'herbe avant de souffler. Essuie tes genoux, on rentre. Le bâton sèche près du savon, un fil encore collant. Un rond d'ombre reste au bas du bronze.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Plus bas, la bulle monte jusqu'au nez. On s'est baissées, d'abord. Tu as regardé avant de souffler. Essuie tes genoux, sur le paillasson. Le bâton sèche près du savon, un fil encore collant. Un rond d'ombre reste au bas du bronze.</t>
+          <t>Plus bas, la bulle monte jusqu'au nez. On s'est baissées, d'abord. Tu as vu l'herbe avant de souffler. Essuie tes genoux, on rentre. Le bâton sèche près du savon, un fil encore collant. Un rond d'ombre reste au bas du bronze.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -3337,8 +3337,8 @@
         <is>
           <t>narrateur|Plus bas, la bulle monte jusqu'au nez.
 enfant-f|On s'est baissées, d'abord.
-papa|Tu as regardé avant de souffler.
-maman|Essuie tes genoux, sur le paillasson.
+papa|Tu as vu l'herbe avant de souffler.
+maman|Essuie tes genoux, on rentre.
 narrateur|Le bâton sèche près du savon, un fil encore collant.
 narrateur|Un rond d'ombre reste au bas du bronze.</t>
         </is>
@@ -3367,12 +3367,12 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Au bord, tout petit. Elle glisse le bâton vers le bord d'herbe. L'herbe tient, sans laisser la poussière. Nina répète, tout bas, encore une fois. Pendant ce temps, le bâton reste droit, sage. Le bord n'a pas soulevé. Tu es à l'abri. Tu as parlé lentement.</t>
+          <t>Au bord, tout petit. Elle glisse le bâton vers le bord d'herbe. L'herbe tient, sans laisser la poussière. Nina répète, tout bas, encore une fois. Pendant ce temps, le bâton reste droit, sans bouger. Le bord n'a pas soulevé. Tu es à l'abri. Tu as dit ça tout bas.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Au bord, tout petit. Elle glisse le bâton vers le bord d'herbe. L'herbe tient, sans laisser la poussière. Nina répète, tout bas, encore une fois. Pendant ce temps, le bâton reste droit, sage. Le bord n'a pas soulevé. Tu es à l'abri. Tu as parlé lentement.</t>
+          <t>Au bord, tout petit. Elle glisse le bâton vers le bord d'herbe. L'herbe tient, sans laisser la poussière. Nina répète, tout bas, encore une fois. Pendant ce temps, le bâton reste droit, sans bouger. Le bord n'a pas soulevé. Tu es à l'abri. Tu as dit ça tout bas.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -3511,10 +3511,10 @@
 narrateur|Elle glisse le bâton vers le bord d'herbe.
 narrateur|L'herbe tient, sans laisser la poussière.
 narrateur|Nina répète, tout bas, encore une fois.
-narrateur|Pendant ce temps, le bâton reste droit, sage.
+narrateur|Pendant ce temps, le bâton reste droit, sans bouger.
 papa|Le bord n'a pas soulevé.
 enfant-f|Tu es à l'abri.
-maman|Tu as parlé lentement.</t>
+maman|Tu as dit ça tout bas.</t>
         </is>
       </c>
     </row>
@@ -3713,12 +3713,12 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Entre ses doigts, le bois du bâton est tiède. Le bronze sent le soleil, encore trop fort. Le fil fond, trop chaud, trop mince. Le nez est trop chaud ! Une bulle touche, puis crève, trop vite. Le nez n'a plus de rond, trop nu. Ça brûle trop, ici. Elle n'avance plus. On fait comment, alors ? Tu trouves, Nina ?</t>
+          <t>Entre ses doigts, le bois du bâton est tiède. Le bronze tient encore tout le soleil. Le fil fond, trop chaud, trop mince. Le nez brûle trop ! La bulle touche, puis crève tout de suite. Il ne reste rien sur le bronze. Ici, c'est trop chaud. La bulle n'arrive pas. Alors on fait quoi ? Tu vois comment, Nina ?</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Entre ses doigts, le bois du bâton est tiède. Le bronze sent le soleil, encore trop fort. Le fil fond, trop chaud, trop mince. Le nez est trop chaud ! Une bulle touche, puis crève, trop vite. Le nez n'a plus de rond, trop nu. Ça brûle trop, ici. Elle n'avance plus. On fait comment, alors ? Tu trouves, Nina ?</t>
+          <t>Entre ses doigts, le bois du bâton est tiède. Le bronze tient encore tout le soleil. Le fil fond, trop chaud, trop mince. Le nez brûle trop ! La bulle touche, puis crève tout de suite. Il ne reste rien sur le bronze. Ici, c'est trop chaud. La bulle n'arrive pas. Alors on fait quoi ? Tu vois comment, Nina ?</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -3854,15 +3854,15 @@
       <c r="AW16" t="inlineStr">
         <is>
           <t>narrateur|Entre ses doigts, le bois du bâton est tiède.
-narrateur|Le bronze sent le soleil, encore trop fort.
+narrateur|Le bronze tient encore tout le soleil.
 narrateur|Le fil fond, trop chaud, trop mince.
-enfant-f|Le nez est trop chaud !
-narrateur|Une bulle touche, puis crève, trop vite.
-narrateur|Le nez n'a plus de rond, trop nu.
-papa|Ça brûle trop, ici.
-maman|Elle n'avance plus.
-enfant-f|On fait comment, alors ?
-maman|Tu trouves, Nina ?</t>
+enfant-f|Le nez brûle trop !
+narrateur|La bulle touche, puis crève tout de suite.
+narrateur|Il ne reste rien sur le bronze.
+papa|Ici, c'est trop chaud.
+maman|La bulle n'arrive pas.
+enfant-f|Alors on fait quoi ?
+maman|Tu vois comment, Nina ?</t>
         </is>
       </c>
     </row>
@@ -3889,12 +3889,12 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Le bronze brûle encore, trop fort. Attendre l'ombre, l'oiseau, ou tout près ?</t>
+          <t>Le bronze n'a pas fini de brûler. Attendre l'ombre, l'oiseau, ou tout près ?</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Le bronze brûle encore, trop fort. Attendre l'ombre, l'oiseau, ou tout près ?</t>
+          <t>Le bronze n'a pas fini de brûler. Attendre l'ombre, l'oiseau, ou tout près ?</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -4057,7 +4057,7 @@
       </c>
       <c r="AW17" t="inlineStr">
         <is>
-          <t>narrateur|Le bronze brûle encore, trop fort.
+          <t>narrateur|Le bronze n'a pas fini de brûler.
 maman|Attendre l'ombre, l'oiseau, ou tout près ?</t>
         </is>
       </c>
@@ -4085,12 +4085,12 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>On attend l'ombre. Une ombre de tilleul glisse sur le nez. Sous l'ombre, le bâton ne fond plus. Le bronze se tait, puis se refroidit. Pendant ce temps, le bâton reste droit, sage. Le nez est redevenu doux. Maintenant, tu me vois. Tu as attendu le silence.</t>
+          <t>On attend l'ombre. Une ombre de tilleul glisse sur le nez. Sous l'ombre, le bâton ne fond plus. Le bronze se tait, puis se refroidit. Pendant ce temps, le bâton reste droit, sans bouger. Le nez est redevenu doux. Maintenant, tu me vois. Tu as laissé l'ombre arriver.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>On attend l'ombre. Une ombre de tilleul glisse sur le nez. Sous l'ombre, le bâton ne fond plus. Le bronze se tait, puis se refroidit. Pendant ce temps, le bâton reste droit, sage. Le nez est redevenu doux. Maintenant, tu me vois. Tu as attendu le silence.</t>
+          <t>On attend l'ombre. Une ombre de tilleul glisse sur le nez. Sous l'ombre, le bâton ne fond plus. Le bronze se tait, puis se refroidit. Pendant ce temps, le bâton reste droit, sans bouger. Le nez est redevenu doux. Maintenant, tu me vois. Tu as laissé l'ombre arriver.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -4229,10 +4229,10 @@
 narrateur|Une ombre de tilleul glisse sur le nez.
 narrateur|Sous l'ombre, le bâton ne fond plus.
 narrateur|Le bronze se tait, puis se refroidit.
-narrateur|Pendant ce temps, le bâton reste droit, sage.
+narrateur|Pendant ce temps, le bâton reste droit, sans bouger.
 maman|Le nez est redevenu doux.
 enfant-f|Maintenant, tu me vois.
-papa|Tu as attendu le silence.</t>
+papa|Tu as laissé l'ombre arriver.</t>
         </is>
       </c>
     </row>
@@ -4259,12 +4259,12 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Quand l'ombre a touché, la bulle a tenu. On a attendu le tilleul. Le silence vous a aidées. Le bronze sent encore le soleil, moins fort. Le bâton sèche près du savon, un fil encore collant. Un pli d'ombre se recouche, tout lent.</t>
+          <t>Quand l'ombre a touché, la bulle a tenu. On a attendu le tilleul. L'ombre vous a aidées. Le bronze sent encore le soleil, moins fort. Le bâton sèche près du savon, un fil encore collant. L'ombre reste un moment, puis glisse.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Quand l'ombre a touché, la bulle a tenu. On a attendu le tilleul. Le silence vous a aidées. Le bronze sent encore le soleil, moins fort. Le bâton sèche près du savon, un fil encore collant. Un pli d'ombre se recouche, tout lent.</t>
+          <t>Quand l'ombre a touché, la bulle a tenu. On a attendu le tilleul. L'ombre vous a aidées. Le bronze sent encore le soleil, moins fort. Le bâton sèche près du savon, un fil encore collant. L'ombre reste un moment, puis glisse.</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -4401,10 +4401,10 @@
         <is>
           <t>narrateur|Quand l'ombre a touché, la bulle a tenu.
 enfant-f|On a attendu le tilleul.
-papa|Le silence vous a aidées.
+papa|L'ombre vous a aidées.
 maman|Le bronze sent encore le soleil, moins fort.
 narrateur|Le bâton sèche près du savon, un fil encore collant.
-narrateur|Un pli d'ombre se recouche, tout lent.</t>
+narrateur|L'ombre reste un moment, puis glisse.</t>
         </is>
       </c>
     </row>
@@ -4431,12 +4431,12 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>L'oiseau, d'abord, il est plus frais. Elle pose d'abord le fil sur l'oiseau. L'oiseau de bronze est à l'ombre, déjà. Le nez reçoit ensuite un rond tout calme. Un fil de savon cherche encore l'air. Tu n'as pas soufflé trop fort. C'est pour toi. Tu as laissé le bronze parler.</t>
+          <t>L'oiseau, d'abord, il est plus frais. Elle pose d'abord le fil sur l'oiseau. L'oiseau de bronze est à l'ombre, déjà. Le nez reçoit ensuite un rond tout calme. Un fil de savon cherche encore l'air. Tu n'as pas soufflé trop fort. C'est pour toi. L'oiseau était plus frais, tu as vu.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>L'oiseau, d'abord, il est plus frais. Elle pose d'abord le fil sur l'oiseau. L'oiseau de bronze est à l'ombre, déjà. Le nez reçoit ensuite un rond tout calme. Un fil de savon cherche encore l'air. Tu n'as pas soufflé trop fort. C'est pour toi. Tu as laissé le bronze parler.</t>
+          <t>L'oiseau, d'abord, il est plus frais. Elle pose d'abord le fil sur l'oiseau. L'oiseau de bronze est à l'ombre, déjà. Le nez reçoit ensuite un rond tout calme. Un fil de savon cherche encore l'air. Tu n'as pas soufflé trop fort. C'est pour toi. L'oiseau était plus frais, tu as vu.</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -4578,7 +4578,7 @@
 narrateur|Un fil de savon cherche encore l'air.
 papa|Tu n'as pas soufflé trop fort.
 enfant-f|C'est pour toi.
-maman|Tu as laissé le bronze parler.</t>
+maman|L'oiseau était plus frais, tu as vu.</t>
         </is>
       </c>
     </row>
@@ -4605,12 +4605,12 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>De l'oiseau au nez, la bulle a glissé. On a commencé par l'oiseau. Tu n'as pas soufflé trop fort. Le bronze a parlé tout seul. Le bâton sèche près du savon, un fil encore collant. Un rond net reste sur le nez, puis pâlit.</t>
+          <t>De l'oiseau au nez, la bulle a glissé. On a commencé par l'oiseau. Tu n'as pas soufflé trop fort. L'oiseau était plus frais, d'abord. Le bâton sèche près du savon, un fil encore collant. Un rond net reste sur le nez, puis pâlit.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>De l'oiseau au nez, la bulle a glissé. On a commencé par l'oiseau. Tu n'as pas soufflé trop fort. Le bronze a parlé tout seul. Le bâton sèche près du savon, un fil encore collant. Un rond net reste sur le nez, puis pâlit.</t>
+          <t>De l'oiseau au nez, la bulle a glissé. On a commencé par l'oiseau. Tu n'as pas soufflé trop fort. L'oiseau était plus frais, d'abord. Le bâton sèche près du savon, un fil encore collant. Un rond net reste sur le nez, puis pâlit.</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -4748,7 +4748,7 @@
           <t>narrateur|De l'oiseau au nez, la bulle a glissé.
 enfant-f|On a commencé par l'oiseau.
 papa|Tu n'as pas soufflé trop fort.
-maman|Le bronze a parlé tout seul.
+maman|L'oiseau était plus frais, d'abord.
 narrateur|Le bâton sèche près du savon, un fil encore collant.
 narrateur|Un rond net reste sur le nez, puis pâlit.</t>
         </is>
@@ -4777,12 +4777,12 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Tout près, contre le bronze. Nina se glisse contre le socle, tout doux. Tout près, le bâton n'a plus d'air chaud. La bulle n'a plus à voyager trop loin. Pendant ce temps, le bâton reste droit, sage. Tu t'es mise tout près, contre le nez. Le nez est là. Tu as observé d'abord.</t>
+          <t>Tout près, contre le bronze. Nina se glisse contre le socle, tout doux. Tout près, le bâton n'a plus d'air chaud. La bulle n'a plus à voyager trop loin. Pendant ce temps, le bâton reste droit, sans bouger. Tu t'es mise tout près, contre le nez. Le nez est là. Tu t'es mise tout contre.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Tout près, contre le bronze. Nina se glisse contre le socle, tout doux. Tout près, le bâton n'a plus d'air chaud. La bulle n'a plus à voyager trop loin. Pendant ce temps, le bâton reste droit, sage. Tu t'es mise tout près, contre le nez. Le nez est là. Tu as observé d'abord.</t>
+          <t>Tout près, contre le bronze. Nina se glisse contre le socle, tout doux. Tout près, le bâton n'a plus d'air chaud. La bulle n'a plus à voyager trop loin. Pendant ce temps, le bâton reste droit, sans bouger. Tu t'es mise tout près, contre le nez. Le nez est là. Tu t'es mise tout contre.</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -4921,10 +4921,10 @@
 narrateur|Nina se glisse contre le socle, tout doux.
 narrateur|Tout près, le bâton n'a plus d'air chaud.
 narrateur|La bulle n'a plus à voyager trop loin.
-narrateur|Pendant ce temps, le bâton reste droit, sage.
+narrateur|Pendant ce temps, le bâton reste droit, sans bouger.
 papa|Tu t'es mise tout près, contre le nez.
 enfant-f|Le nez est là.
-maman|Tu as observé d'abord.</t>
+maman|Tu t'es mise tout contre.</t>
         </is>
       </c>
     </row>
@@ -4951,12 +4951,12 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Tout près, la bulle touche le nez, déjà. Je me suis mise tout près. Tu t'es glissée, comme l'ombre. Vous rentrez, les mains pleines de savon. Le bâton sèche près du savon, un fil encore collant. Le socle reste derrière, sans brûler.</t>
+          <t>Tout près, la bulle touche le nez, déjà. Je me suis mise tout près. Tu t'es glissée, comme l'ombre. Vos mains sentent encore le savon. Le bâton sèche près du savon, un fil encore collant. Le socle reste derrière, sans brûler.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Tout près, la bulle touche le nez, déjà. Je me suis mise tout près. Tu t'es glissée, comme l'ombre. Vous rentrez, les mains pleines de savon. Le bâton sèche près du savon, un fil encore collant. Le socle reste derrière, sans brûler.</t>
+          <t>Tout près, la bulle touche le nez, déjà. Je me suis mise tout près. Tu t'es glissée, comme l'ombre. Vos mains sentent encore le savon. Le bâton sèche près du savon, un fil encore collant. Le socle reste derrière, sans brûler.</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -5094,7 +5094,7 @@
           <t>narrateur|Tout près, la bulle touche le nez, déjà.
 enfant-f|Je me suis mise tout près.
 papa|Tu t'es glissée, comme l'ombre.
-maman|Vous rentrez, les mains pleines de savon.
+maman|Vos mains sentent encore le savon.
 narrateur|Le bâton sèche près du savon, un fil encore collant.
 narrateur|Le socle reste derrière, sans brûler.</t>
         </is>
@@ -5123,12 +5123,12 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Entre ses doigts, le bois du bâton est tiède. Le tilleul sent le miel, trop vif. Le fil claque, trop léger dans l'air. Le vent prend tout ! Une feuille claque, puis une autre. La bulle part de travers, trop loin. Ça souffle trop, ici. Elle a besoin de temps. On fait comment, alors ? Tu trouves, Nina ?</t>
+          <t>Entre ses doigts, le bois du bâton est tiède. Le tilleul agite ses feuilles, trop vite. Le fil claque, trop léger dans l'air. Le vent prend tout ! Une feuille claque, puis une autre. La bulle part de travers, trop loin. Ici, ça souffle trop. Il lui faut du temps. Alors on fait quoi ? Tu vois comment, Nina ?</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Entre ses doigts, le bois du bâton est tiède. Le tilleul sent le miel, trop vif. Le fil claque, trop léger dans l'air. Le vent prend tout ! Une feuille claque, puis une autre. La bulle part de travers, trop loin. Ça souffle trop, ici. Elle a besoin de temps. On fait comment, alors ? Tu trouves, Nina ?</t>
+          <t>Entre ses doigts, le bois du bâton est tiède. Le tilleul agite ses feuilles, trop vite. Le fil claque, trop léger dans l'air. Le vent prend tout ! Une feuille claque, puis une autre. La bulle part de travers, trop loin. Ici, ça souffle trop. Il lui faut du temps. Alors on fait quoi ? Tu vois comment, Nina ?</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -5264,15 +5264,15 @@
       <c r="AW24" t="inlineStr">
         <is>
           <t>narrateur|Entre ses doigts, le bois du bâton est tiède.
-narrateur|Le tilleul sent le miel, trop vif.
+narrateur|Le tilleul agite ses feuilles, trop vite.
 narrateur|Le fil claque, trop léger dans l'air.
 enfant-f|Le vent prend tout !
 narrateur|Une feuille claque, puis une autre.
 narrateur|La bulle part de travers, trop loin.
-papa|Ça souffle trop, ici.
-maman|Elle a besoin de temps.
-enfant-f|On fait comment, alors ?
-papa|Tu trouves, Nina ?</t>
+papa|Ici, ça souffle trop.
+maman|Il lui faut du temps.
+enfant-f|Alors on fait quoi ?
+papa|Tu vois comment, Nina ?</t>
         </is>
       </c>
     </row>
@@ -5299,12 +5299,12 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Les feuilles claquent encore, trop fort. Attendre les feuilles, derrière, ou tout petit ?</t>
+          <t>Les feuilles n'ont pas fini de claquer. Attendre les feuilles, derrière, ou tout petit ?</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Les feuilles claquent encore, trop fort. Attendre les feuilles, derrière, ou tout petit ?</t>
+          <t>Les feuilles n'ont pas fini de claquer. Attendre les feuilles, derrière, ou tout petit ?</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -5467,7 +5467,7 @@
       </c>
       <c r="AW25" t="inlineStr">
         <is>
-          <t>narrateur|Les feuilles claquent encore, trop fort.
+          <t>narrateur|Les feuilles n'ont pas fini de claquer.
 papa|Attendre les feuilles, derrière, ou tout petit ?</t>
         </is>
       </c>
@@ -5495,12 +5495,12 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>On attend les feuilles, d'abord. Elle tient le bâton, puis attend les feuilles. Les feuilles vont, reviennent, puis se taisent. L'air redevient un seul souffle, net. Pendant ce temps, le bâton reste droit, sage. Le tilleul n'a plus claqué. Maintenant, tu peux rester. Tu as attendu le calme.</t>
+          <t>On attend les feuilles, d'abord. Elle tient le bâton, puis attend les feuilles. Les feuilles vont, reviennent, puis se taisent. L'air redevient un seul souffle, net. Pendant ce temps, le bâton reste droit, sans bouger. Le tilleul n'a plus claqué. Maintenant, tu peux rester. Tu as laissé les feuilles finir.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>On attend les feuilles, d'abord. Elle tient le bâton, puis attend les feuilles. Les feuilles vont, reviennent, puis se taisent. L'air redevient un seul souffle, net. Pendant ce temps, le bâton reste droit, sage. Le tilleul n'a plus claqué. Maintenant, tu peux rester. Tu as attendu le calme.</t>
+          <t>On attend les feuilles, d'abord. Elle tient le bâton, puis attend les feuilles. Les feuilles vont, reviennent, puis se taisent. L'air redevient un seul souffle, net. Pendant ce temps, le bâton reste droit, sans bouger. Le tilleul n'a plus claqué. Maintenant, tu peux rester. Tu as laissé les feuilles finir.</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -5639,10 +5639,10 @@
 narrateur|Elle tient le bâton, puis attend les feuilles.
 narrateur|Les feuilles vont, reviennent, puis se taisent.
 narrateur|L'air redevient un seul souffle, net.
-narrateur|Pendant ce temps, le bâton reste droit, sage.
+narrateur|Pendant ce temps, le bâton reste droit, sans bouger.
 papa|Le tilleul n'a plus claqué.
 enfant-f|Maintenant, tu peux rester.
-maman|Tu as attendu le calme.</t>
+maman|Tu as laissé les feuilles finir.</t>
         </is>
       </c>
     </row>
@@ -5841,12 +5841,12 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Derrière, pas trop près du vent. Derrière le tronc, le bâton ne claque plus. Nina se glisse derrière le tronc, tout bas. Rien ne claque, rien ne pousse plus. Un fil de savon cherche encore l'air. Tu n'as pas couru. Tu es ronde, maintenant. Tu as préparé le chemin.</t>
+          <t>Derrière, pas trop près du vent. Derrière le tronc, le bâton ne claque plus. Nina se glisse derrière le tronc, tout bas. Rien ne claque, rien ne pousse plus. Un fil de savon cherche encore l'air. Tu n'as pas couru. Tu es ronde, maintenant. Derrière, l'air était plus doux.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Derrière, pas trop près du vent. Derrière le tronc, le bâton ne claque plus. Nina se glisse derrière le tronc, tout bas. Rien ne claque, rien ne pousse plus. Un fil de savon cherche encore l'air. Tu n'as pas couru. Tu es ronde, maintenant. Tu as préparé le chemin.</t>
+          <t>Derrière, pas trop près du vent. Derrière le tronc, le bâton ne claque plus. Nina se glisse derrière le tronc, tout bas. Rien ne claque, rien ne pousse plus. Un fil de savon cherche encore l'air. Tu n'as pas couru. Tu es ronde, maintenant. Derrière, l'air était plus doux.</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -5988,7 +5988,7 @@
 narrateur|Un fil de savon cherche encore l'air.
 papa|Tu n'as pas couru.
 enfant-f|Tu es ronde, maintenant.
-maman|Tu as préparé le chemin.</t>
+maman|Derrière, l'air était plus doux.</t>
         </is>
       </c>
     </row>
@@ -6187,12 +6187,12 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Tout petit, tout serré. Une toute petite bulle quitte le bâton. Nina souffle à peine, sans prendre le vent. Le tilleul se tait, plus loin, tout seul. Pendant ce temps, le bâton reste droit, sage. Le petit rond n'a pas volé. Tu restes, bulle. Le petit tenait assez.</t>
+          <t>Tout petit, tout serré. Une toute petite bulle quitte le bâton. Nina souffle à peine, sans prendre le vent. Le tilleul se tait, plus loin, tout seul. Un fil de savon cherche encore l'air. Le petit rond n'a pas volé. Tu restes, bulle. Le petit rond a suffi.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Tout petit, tout serré. Une toute petite bulle quitte le bâton. Nina souffle à peine, sans prendre le vent. Le tilleul se tait, plus loin, tout seul. Pendant ce temps, le bâton reste droit, sage. Le petit rond n'a pas volé. Tu restes, bulle. Le petit tenait assez.</t>
+          <t>Tout petit, tout serré. Une toute petite bulle quitte le bâton. Nina souffle à peine, sans prendre le vent. Le tilleul se tait, plus loin, tout seul. Un fil de savon cherche encore l'air. Le petit rond n'a pas volé. Tu restes, bulle. Le petit rond a suffi.</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -6331,10 +6331,10 @@
 narrateur|Une toute petite bulle quitte le bâton.
 narrateur|Nina souffle à peine, sans prendre le vent.
 narrateur|Le tilleul se tait, plus loin, tout seul.
-narrateur|Pendant ce temps, le bâton reste droit, sage.
+narrateur|Un fil de savon cherche encore l'air.
 papa|Le petit rond n'a pas volé.
 enfant-f|Tu restes, bulle.
-maman|Le petit tenait assez.</t>
+maman|Le petit rond a suffi.</t>
         </is>
       </c>
     </row>
@@ -6361,12 +6361,12 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Tout petit, le rond tient sur le nez, tout calme. On a soufflé à peine. Le petit rond n'a pas volé. Rentrez, le savon est déjà sec. Le bâton sèche près du savon, un fil encore collant. Le tilleul se tait, plus loin, tout seul.</t>
+          <t>Tout petit, le rond tient sur le nez, tout calme. On a soufflé à peine. Le petit rond n'a pas volé. Le savon est déjà sec, on rentre. Le bâton sèche près du savon, un fil encore collant. Le tilleul se tait, plus loin, tout seul.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Tout petit, le rond tient sur le nez, tout calme. On a soufflé à peine. Le petit rond n'a pas volé. Rentrez, le savon est déjà sec. Le bâton sèche près du savon, un fil encore collant. Le tilleul se tait, plus loin, tout seul.</t>
+          <t>Tout petit, le rond tient sur le nez, tout calme. On a soufflé à peine. Le petit rond n'a pas volé. Le savon est déjà sec, on rentre. Le bâton sèche près du savon, un fil encore collant. Le tilleul se tait, plus loin, tout seul.</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -6504,7 +6504,7 @@
           <t>narrateur|Tout petit, le rond tient sur le nez, tout calme.
 enfant-f|On a soufflé à peine.
 papa|Le petit rond n'a pas volé.
-maman|Rentrez, le savon est déjà sec.
+maman|Le savon est déjà sec, on rentre.
 narrateur|Le bâton sèche près du savon, un fil encore collant.
 narrateur|Le tilleul se tait, plus loin, tout seul.</t>
         </is>
@@ -6533,12 +6533,12 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Nina prend d'abord le savon, encore un peu collant. Il va faire la bulle. Ouvre tout doux, pas trop vite. Une goutte reste au pouce, puis glisse. Le bâton, ensuite, près de toi. Papa pose la coupelle contre le gravier. Elle emporte les trois, contre elle. Tu vas m'aider, savon. Le flacon frotte sa manche, un peu. Le savon d'abord, il est prêt.</t>
+          <t>Nina dévisse d'abord le savon, tout lentement. Il va donner la bulle. Une goutte, pas tout le flacon. La goutte reste au pouce, puis tombe. Le bâton t'attend, près du lacet. Papa pose la coupelle contre le gravier chaud. Nina serre les trois contre son ventre. Savon, tu restes avec moi. Le flacon colle un peu sa manche. Le savon est ouvert, tu peux y aller.</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Nina prend d'abord le savon, encore un peu collant. Il va faire la bulle. Ouvre tout doux, pas trop vite. Une goutte reste au pouce, puis glisse. Le bâton, ensuite, près de toi. Papa pose la coupelle contre le gravier. Elle emporte les trois, contre elle. Tu vas m'aider, savon. Le flacon frotte sa manche, un peu. Le savon d'abord, il est prêt.</t>
+          <t>Nina dévisse d'abord le savon, tout lentement. Il va donner la bulle. Une goutte, pas tout le flacon. La goutte reste au pouce, puis tombe. Le bâton t'attend, près du lacet. Papa pose la coupelle contre le gravier chaud. Nina serre les trois contre son ventre. Savon, tu restes avec moi. Le flacon colle un peu sa manche. Le savon est ouvert, tu peux y aller.</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -6673,16 +6673,16 @@
       <c r="AV32" s="2" t="inlineStr"/>
       <c r="AW32" t="inlineStr">
         <is>
-          <t>narrateur|Nina prend d'abord le savon, encore un peu collant.
-enfant-f|Il va faire la bulle.
-papa|Ouvre tout doux, pas trop vite.
-narrateur|Une goutte reste au pouce, puis glisse.
-maman|Le bâton, ensuite, près de toi.
-narrateur|Papa pose la coupelle contre le gravier.
-narrateur|Elle emporte les trois, contre elle.
-enfant-f|Tu vas m'aider, savon.
-narrateur|Le flacon frotte sa manche, un peu.
-maman|Le savon d'abord, il est prêt.</t>
+          <t>narrateur|Nina dévisse d'abord le savon, tout lentement.
+enfant-f|Il va donner la bulle.
+papa|Une goutte, pas tout le flacon.
+narrateur|La goutte reste au pouce, puis tombe.
+maman|Le bâton t'attend, près du lacet.
+narrateur|Papa pose la coupelle contre le gravier chaud.
+narrateur|Nina serre les trois contre son ventre.
+enfant-f|Savon, tu restes avec moi.
+narrateur|Le flacon colle un peu sa manche.
+maman|Le savon est ouvert, tu peux y aller.</t>
         </is>
       </c>
     </row>
@@ -6893,12 +6893,12 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Le savon fait un rond lâche, au poignet. Il va filer la bulle. Le flacon sent encore le sucre. Vos mains sont prêtes ? Oui, maman. Une goutte se tait, puis plus rien.</t>
+          <t>Le savon pend au poignet, un peu lâche. Il va filer la bulle. Ça sent encore le sucre, toi. Tes mains sont prêtes ? Oui, maman. Une goutte se tait, puis plus rien.</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Le savon fait un rond lâche, au poignet. Il va filer la bulle. Le flacon sent encore le sucre. Vos mains sont prêtes ? Oui, maman. Une goutte se tait, puis plus rien.</t>
+          <t>Le savon pend au poignet, un peu lâche. Il va filer la bulle. Ça sent encore le sucre, toi. Tes mains sont prêtes ? Oui, maman. Une goutte se tait, puis plus rien.</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -7037,10 +7037,10 @@
       </c>
       <c r="AW34" t="inlineStr">
         <is>
-          <t>narrateur|Le savon fait un rond lâche, au poignet.
+          <t>narrateur|Le savon pend au poignet, un peu lâche.
 enfant-f|Il va filer la bulle.
-papa|Le flacon sent encore le sucre.
-maman|Vos mains sont prêtes ?
+papa|Ça sent encore le sucre, toi.
+maman|Tes mains sont prêtes ?
 enfant-f|Oui, maman.
 narrateur|Une goutte se tait, puis plus rien.</t>
         </is>
@@ -7069,12 +7069,12 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Le savon frotte sa manche, un peu collant. L'allée soulève déjà trop de poussière. Plus loin, le socle brûle encore. Sous le tilleul, les feuilles claquent. Nina, vous partez où ?</t>
+          <t>Le savon colle encore à sa manche. Devant, l'allée soulève trop de poussière. Le socle, lui, brûle encore au soleil. Sous le tilleul, les feuilles claquent. Nina, tu vas où ?</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Le savon frotte sa manche, un peu collant. L'allée soulève déjà trop de poussière. Plus loin, le socle brûle encore. Sous le tilleul, les feuilles claquent. Nina, vous partez où ?</t>
+          <t>Le savon colle encore à sa manche. Devant, l'allée soulève trop de poussière. Le socle, lui, brûle encore au soleil. Sous le tilleul, les feuilles claquent. Nina, tu vas où ?</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -7233,11 +7233,11 @@
       <c r="AV35" s="2" t="inlineStr"/>
       <c r="AW35" t="inlineStr">
         <is>
-          <t>narrateur|Le savon frotte sa manche, un peu collant.
-narrateur|L'allée soulève déjà trop de poussière.
-narrateur|Plus loin, le socle brûle encore.
+          <t>narrateur|Le savon colle encore à sa manche.
+narrateur|Devant, l'allée soulève trop de poussière.
+narrateur|Le socle, lui, brûle encore au soleil.
 narrateur|Sous le tilleul, les feuilles claquent.
-papa|Nina, vous partez où ?</t>
+papa|Nina, tu vas où ?</t>
         </is>
       </c>
     </row>
@@ -7264,12 +7264,12 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Dans sa paume, le flacon de savon est tiède. L'allée sent le gravier chaud, trop vif. La goutte saute, trop sèche, trop vite. Ma bulle a sauté ! Un pas soulève la poussière, encore. La bulle n'a plus le temps d'arriver. Ça bouge trop, ici. Elle a besoin de calme. On fait comment, alors ? Tu trouves, Nina ?</t>
+          <t>Dans sa paume, le flacon de savon est tiède. Le gravier de l'allée saute sous les pas. La goutte saute, trop sèche, trop vite. Ma bulle a crevé ! Encore un pas, encore de la poussière. Le nez reste trop loin, trop gris. Ici, ça n'arrête pas. La bulle a besoin de calme. Alors on fait quoi ? Tu vois comment, Nina ?</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Dans sa paume, le flacon de savon est tiède. L'allée sent le gravier chaud, trop vif. La goutte saute, trop sèche, trop vite. Ma bulle a sauté ! Un pas soulève la poussière, encore. La bulle n'a plus le temps d'arriver. Ça bouge trop, ici. Elle a besoin de calme. On fait comment, alors ? Tu trouves, Nina ?</t>
+          <t>Dans sa paume, le flacon de savon est tiède. Le gravier de l'allée saute sous les pas. La goutte saute, trop sèche, trop vite. Ma bulle a crevé ! Encore un pas, encore de la poussière. Le nez reste trop loin, trop gris. Ici, ça n'arrête pas. La bulle a besoin de calme. Alors on fait quoi ? Tu vois comment, Nina ?</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -7405,15 +7405,15 @@
       <c r="AW36" t="inlineStr">
         <is>
           <t>narrateur|Dans sa paume, le flacon de savon est tiède.
-narrateur|L'allée sent le gravier chaud, trop vif.
+narrateur|Le gravier de l'allée saute sous les pas.
 narrateur|La goutte saute, trop sèche, trop vite.
-enfant-f|Ma bulle a sauté !
-narrateur|Un pas soulève la poussière, encore.
-narrateur|La bulle n'a plus le temps d'arriver.
-papa|Ça bouge trop, ici.
-maman|Elle a besoin de calme.
-enfant-f|On fait comment, alors ?
-papa|Tu trouves, Nina ?</t>
+enfant-f|Ma bulle a crevé !
+narrateur|Encore un pas, encore de la poussière.
+narrateur|Le nez reste trop loin, trop gris.
+papa|Ici, ça n'arrête pas.
+maman|La bulle a besoin de calme.
+enfant-f|Alors on fait quoi ?
+papa|Tu vois comment, Nina ?</t>
         </is>
       </c>
     </row>
@@ -7440,12 +7440,12 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>L'allée soulève encore trop de poussière. Attendre les pas, plus bas, ou le bord ?</t>
+          <t>L'allée n'a pas fini de soulever. Attendre les pas, plus bas, ou le bord ?</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>L'allée soulève encore trop de poussière. Attendre les pas, plus bas, ou le bord ?</t>
+          <t>L'allée n'a pas fini de soulever. Attendre les pas, plus bas, ou le bord ?</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -7608,7 +7608,7 @@
       </c>
       <c r="AW37" t="inlineStr">
         <is>
-          <t>narrateur|L'allée soulève encore trop de poussière.
+          <t>narrateur|L'allée n'a pas fini de soulever.
 papa|Attendre les pas, plus bas, ou le bord ?</t>
         </is>
       </c>
@@ -7636,12 +7636,12 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>On attend les pas. Elle tient le savon, sans ouvrir encore. Le gravier se tait, une fois, puis plus. Tu peux partir, maintenant. Fermé, le savon attend contre son pouce. Les pas se sont tus, maintenant. La bulle part, ronde, tout calme. Tu lui as laissé le temps.</t>
+          <t>On attend les pas. Elle tient le savon, sans ouvrir encore. Le gravier se tait, une fois, puis plus. Tu peux partir, maintenant. Fermé, le savon attend contre son pouce. Les pas se sont tus, maintenant. La bulle part, ronde, tout calme. Tu as attendu, et elle est partie.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>On attend les pas. Elle tient le savon, sans ouvrir encore. Le gravier se tait, une fois, puis plus. Tu peux partir, maintenant. Fermé, le savon attend contre son pouce. Les pas se sont tus, maintenant. La bulle part, ronde, tout calme. Tu lui as laissé le temps.</t>
+          <t>On attend les pas. Elle tient le savon, sans ouvrir encore. Le gravier se tait, une fois, puis plus. Tu peux partir, maintenant. Fermé, le savon attend contre son pouce. Les pas se sont tus, maintenant. La bulle part, ronde, tout calme. Tu as attendu, et elle est partie.</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -7783,7 +7783,7 @@
 narrateur|Fermé, le savon attend contre son pouce.
 papa|Les pas se sont tus, maintenant.
 narrateur|La bulle part, ronde, tout calme.
-maman|Tu lui as laissé le temps.</t>
+maman|Tu as attendu, et elle est partie.</t>
         </is>
       </c>
     </row>
@@ -7810,12 +7810,12 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>La bulle se pose, ronde, sur le nez de bronze. On a attendu les pas. Merci d'avoir laissé le gravier se taire. Rentrez, la cloche n'a pas encore sonné. Le flacon reste fermé, une goutte au bouchon. Une poussière tourne encore, puis s'arrête.</t>
+          <t>La bulle se pose, ronde, sur le nez de bronze. On a attendu les pas. Merci d'avoir laissé le gravier se taire. La cloche n'a pas encore sonné. Le flacon reste fermé, une goutte au bouchon. Un grain de poussière retombe, puis plus rien.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>La bulle se pose, ronde, sur le nez de bronze. On a attendu les pas. Merci d'avoir laissé le gravier se taire. Rentrez, la cloche n'a pas encore sonné. Le flacon reste fermé, une goutte au bouchon. Une poussière tourne encore, puis s'arrête.</t>
+          <t>La bulle se pose, ronde, sur le nez de bronze. On a attendu les pas. Merci d'avoir laissé le gravier se taire. La cloche n'a pas encore sonné. Le flacon reste fermé, une goutte au bouchon. Un grain de poussière retombe, puis plus rien.</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -7953,9 +7953,9 @@
           <t>narrateur|La bulle se pose, ronde, sur le nez de bronze.
 enfant-f|On a attendu les pas.
 papa|Merci d'avoir laissé le gravier se taire.
-maman|Rentrez, la cloche n'a pas encore sonné.
+maman|La cloche n'a pas encore sonné.
 narrateur|Le flacon reste fermé, une goutte au bouchon.
-narrateur|Une poussière tourne encore, puis s'arrête.</t>
+narrateur|Un grain de poussière retombe, puis plus rien.</t>
         </is>
       </c>
     </row>
@@ -7982,12 +7982,12 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Plus bas, d'abord. Elle baisse le savon, loin de la poussière. Nina s'accroupit, les genoux au gravier. L'air est plus doux, près de l'herbe. Une goutte de savon brille, prête à filer. Tu as regardé d'abord. Ici, tu ne sautes plus. Le bas était plus calme.</t>
+          <t>Plus bas, d'abord. Elle baisse le savon, loin de la poussière. Nina s'accroupit, les genoux au gravier. L'air est plus doux, près de l'herbe. Une goutte de savon brille, prête à filer. Tu as vu l'herbe, avant. Ici, tu ne crèves plus. Près du sol, ça tenait mieux.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Plus bas, d'abord. Elle baisse le savon, loin de la poussière. Nina s'accroupit, les genoux au gravier. L'air est plus doux, près de l'herbe. Une goutte de savon brille, prête à filer. Tu as regardé d'abord. Ici, tu ne sautes plus. Le bas était plus calme.</t>
+          <t>Plus bas, d'abord. Elle baisse le savon, loin de la poussière. Nina s'accroupit, les genoux au gravier. L'air est plus doux, près de l'herbe. Une goutte de savon brille, prête à filer. Tu as vu l'herbe, avant. Ici, tu ne crèves plus. Près du sol, ça tenait mieux.</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -8127,9 +8127,9 @@
 narrateur|Nina s'accroupit, les genoux au gravier.
 narrateur|L'air est plus doux, près de l'herbe.
 narrateur|Une goutte de savon brille, prête à filer.
-papa|Tu as regardé d'abord.
-enfant-f|Ici, tu ne sautes plus.
-maman|Le bas était plus calme.</t>
+papa|Tu as vu l'herbe, avant.
+enfant-f|Ici, tu ne crèves plus.
+maman|Près du sol, ça tenait mieux.</t>
         </is>
       </c>
     </row>
@@ -8156,12 +8156,12 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Plus bas, la bulle monte jusqu'au nez. On s'est baissées, d'abord. Tu as regardé avant de souffler. Essuie tes genoux, sur le paillasson. Le flacon reste fermé, une goutte au bouchon. Un rond d'ombre reste au bas du bronze.</t>
+          <t>Plus bas, la bulle monte jusqu'au nez. On s'est baissées, d'abord. Tu as vu l'herbe avant de souffler. Essuie tes genoux, on rentre. Le flacon reste fermé, une goutte au bouchon. Un rond d'ombre reste au bas du bronze.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Plus bas, la bulle monte jusqu'au nez. On s'est baissées, d'abord. Tu as regardé avant de souffler. Essuie tes genoux, sur le paillasson. Le flacon reste fermé, une goutte au bouchon. Un rond d'ombre reste au bas du bronze.</t>
+          <t>Plus bas, la bulle monte jusqu'au nez. On s'est baissées, d'abord. Tu as vu l'herbe avant de souffler. Essuie tes genoux, on rentre. Le flacon reste fermé, une goutte au bouchon. Un rond d'ombre reste au bas du bronze.</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -8298,8 +8298,8 @@
         <is>
           <t>narrateur|Plus bas, la bulle monte jusqu'au nez.
 enfant-f|On s'est baissées, d'abord.
-papa|Tu as regardé avant de souffler.
-maman|Essuie tes genoux, sur le paillasson.
+papa|Tu as vu l'herbe avant de souffler.
+maman|Essuie tes genoux, on rentre.
 narrateur|Le flacon reste fermé, une goutte au bouchon.
 narrateur|Un rond d'ombre reste au bas du bronze.</t>
         </is>
@@ -8328,12 +8328,12 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Au bord, tout petit. Elle glisse le savon vers le bord d'herbe. L'herbe tient, sans laisser la poussière. Nina répète, tout bas, encore une fois. Fermé, le savon attend contre son pouce. Le bord n'a pas soulevé. Tu es à l'abri. Tu as parlé lentement.</t>
+          <t>Au bord, tout petit. Elle glisse le savon vers le bord d'herbe. L'herbe tient, sans laisser la poussière. Nina répète, tout bas, encore une fois. Fermé, le savon attend contre son pouce. Le bord n'a pas soulevé. Tu es à l'abri. Tu as dit ça tout bas.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Au bord, tout petit. Elle glisse le savon vers le bord d'herbe. L'herbe tient, sans laisser la poussière. Nina répète, tout bas, encore une fois. Fermé, le savon attend contre son pouce. Le bord n'a pas soulevé. Tu es à l'abri. Tu as parlé lentement.</t>
+          <t>Au bord, tout petit. Elle glisse le savon vers le bord d'herbe. L'herbe tient, sans laisser la poussière. Nina répète, tout bas, encore une fois. Fermé, le savon attend contre son pouce. Le bord n'a pas soulevé. Tu es à l'abri. Tu as dit ça tout bas.</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -8475,7 +8475,7 @@
 narrateur|Fermé, le savon attend contre son pouce.
 papa|Le bord n'a pas soulevé.
 enfant-f|Tu es à l'abri.
-maman|Tu as parlé lentement.</t>
+maman|Tu as dit ça tout bas.</t>
         </is>
       </c>
     </row>
@@ -8674,12 +8674,12 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Dans sa paume, le flacon de savon est tiède. Le bronze sent le soleil, encore trop fort. La goutte sèche, trop vite, trop chaude. Le nez est trop chaud ! Une bulle touche, puis crève, trop vite. Le nez n'a plus de rond, trop nu. Ça brûle trop, ici. Elle n'avance plus. On fait comment, alors ? Tu trouves, Nina ?</t>
+          <t>Dans sa paume, le flacon de savon est tiède. Le bronze tient encore tout le soleil. La goutte sèche, trop vite, trop chaude. Le nez brûle trop ! La bulle touche, puis crève tout de suite. Il ne reste rien sur le bronze. Ici, c'est trop chaud. La bulle n'arrive pas. Alors on fait quoi ? Tu vois comment, Nina ?</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Dans sa paume, le flacon de savon est tiède. Le bronze sent le soleil, encore trop fort. La goutte sèche, trop vite, trop chaude. Le nez est trop chaud ! Une bulle touche, puis crève, trop vite. Le nez n'a plus de rond, trop nu. Ça brûle trop, ici. Elle n'avance plus. On fait comment, alors ? Tu trouves, Nina ?</t>
+          <t>Dans sa paume, le flacon de savon est tiède. Le bronze tient encore tout le soleil. La goutte sèche, trop vite, trop chaude. Le nez brûle trop ! La bulle touche, puis crève tout de suite. Il ne reste rien sur le bronze. Ici, c'est trop chaud. La bulle n'arrive pas. Alors on fait quoi ? Tu vois comment, Nina ?</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -8815,15 +8815,15 @@
       <c r="AW44" t="inlineStr">
         <is>
           <t>narrateur|Dans sa paume, le flacon de savon est tiède.
-narrateur|Le bronze sent le soleil, encore trop fort.
+narrateur|Le bronze tient encore tout le soleil.
 narrateur|La goutte sèche, trop vite, trop chaude.
-enfant-f|Le nez est trop chaud !
-narrateur|Une bulle touche, puis crève, trop vite.
-narrateur|Le nez n'a plus de rond, trop nu.
-papa|Ça brûle trop, ici.
-maman|Elle n'avance plus.
-enfant-f|On fait comment, alors ?
-maman|Tu trouves, Nina ?</t>
+enfant-f|Le nez brûle trop !
+narrateur|La bulle touche, puis crève tout de suite.
+narrateur|Il ne reste rien sur le bronze.
+papa|Ici, c'est trop chaud.
+maman|La bulle n'arrive pas.
+enfant-f|Alors on fait quoi ?
+maman|Tu vois comment, Nina ?</t>
         </is>
       </c>
     </row>
@@ -8850,12 +8850,12 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Le bronze brûle encore, trop fort. Attendre l'ombre, l'oiseau, ou tout près ?</t>
+          <t>Le bronze n'a pas fini de brûler. Attendre l'ombre, l'oiseau, ou tout près ?</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Le bronze brûle encore, trop fort. Attendre l'ombre, l'oiseau, ou tout près ?</t>
+          <t>Le bronze n'a pas fini de brûler. Attendre l'ombre, l'oiseau, ou tout près ?</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -9018,7 +9018,7 @@
       </c>
       <c r="AW45" t="inlineStr">
         <is>
-          <t>narrateur|Le bronze brûle encore, trop fort.
+          <t>narrateur|Le bronze n'a pas fini de brûler.
 maman|Attendre l'ombre, l'oiseau, ou tout près ?</t>
         </is>
       </c>
@@ -9046,12 +9046,12 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>On attend l'ombre. Une ombre de tilleul glisse sur le nez. Sous l'ombre, le savon ne sèche plus. Le bronze se tait, puis se refroidit. Fermé, le savon attend contre son pouce. Le nez est redevenu doux. Maintenant, tu me vois. Tu as attendu le silence.</t>
+          <t>On attend l'ombre. Une ombre de tilleul glisse sur le nez. Sous l'ombre, le savon ne sèche plus. Le bronze se tait, puis se refroidit. Fermé, le savon attend contre son pouce. Le nez est redevenu doux. Maintenant, tu me vois. Tu as laissé l'ombre arriver.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>On attend l'ombre. Une ombre de tilleul glisse sur le nez. Sous l'ombre, le savon ne sèche plus. Le bronze se tait, puis se refroidit. Fermé, le savon attend contre son pouce. Le nez est redevenu doux. Maintenant, tu me vois. Tu as attendu le silence.</t>
+          <t>On attend l'ombre. Une ombre de tilleul glisse sur le nez. Sous l'ombre, le savon ne sèche plus. Le bronze se tait, puis se refroidit. Fermé, le savon attend contre son pouce. Le nez est redevenu doux. Maintenant, tu me vois. Tu as laissé l'ombre arriver.</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -9193,7 +9193,7 @@
 narrateur|Fermé, le savon attend contre son pouce.
 maman|Le nez est redevenu doux.
 enfant-f|Maintenant, tu me vois.
-papa|Tu as attendu le silence.</t>
+papa|Tu as laissé l'ombre arriver.</t>
         </is>
       </c>
     </row>
@@ -9220,12 +9220,12 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Quand l'ombre a touché, la bulle a tenu. On a attendu le tilleul. Le silence vous a aidées. Le bronze sent encore le soleil, moins fort. Le flacon reste fermé, une goutte au bouchon. Un pli d'ombre se recouche, tout lent.</t>
+          <t>Quand l'ombre a touché, la bulle a tenu. On a attendu le tilleul. L'ombre vous a aidées. Le bronze sent encore le soleil, moins fort. Le flacon reste fermé, une goutte au bouchon. L'ombre reste un moment, puis glisse.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Quand l'ombre a touché, la bulle a tenu. On a attendu le tilleul. Le silence vous a aidées. Le bronze sent encore le soleil, moins fort. Le flacon reste fermé, une goutte au bouchon. Un pli d'ombre se recouche, tout lent.</t>
+          <t>Quand l'ombre a touché, la bulle a tenu. On a attendu le tilleul. L'ombre vous a aidées. Le bronze sent encore le soleil, moins fort. Le flacon reste fermé, une goutte au bouchon. L'ombre reste un moment, puis glisse.</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -9362,10 +9362,10 @@
         <is>
           <t>narrateur|Quand l'ombre a touché, la bulle a tenu.
 enfant-f|On a attendu le tilleul.
-papa|Le silence vous a aidées.
+papa|L'ombre vous a aidées.
 maman|Le bronze sent encore le soleil, moins fort.
 narrateur|Le flacon reste fermé, une goutte au bouchon.
-narrateur|Un pli d'ombre se recouche, tout lent.</t>
+narrateur|L'ombre reste un moment, puis glisse.</t>
         </is>
       </c>
     </row>
@@ -9392,12 +9392,12 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>L'oiseau, d'abord, il est plus frais. Elle pose d'abord la goutte sur l'oiseau. L'oiseau de bronze est à l'ombre, déjà. Le nez reçoit ensuite un rond tout calme. Une goutte de savon brille, prête à filer. Tu n'as pas soufflé trop fort. C'est pour toi. Tu as laissé le bronze parler.</t>
+          <t>L'oiseau, d'abord, il est plus frais. Elle pose d'abord la goutte sur l'oiseau. L'oiseau de bronze est à l'ombre, déjà. Le nez reçoit ensuite un rond tout calme. Une goutte de savon brille, prête à filer. Tu n'as pas soufflé trop fort. C'est pour toi. L'oiseau était plus frais, tu as vu.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>L'oiseau, d'abord, il est plus frais. Elle pose d'abord la goutte sur l'oiseau. L'oiseau de bronze est à l'ombre, déjà. Le nez reçoit ensuite un rond tout calme. Une goutte de savon brille, prête à filer. Tu n'as pas soufflé trop fort. C'est pour toi. Tu as laissé le bronze parler.</t>
+          <t>L'oiseau, d'abord, il est plus frais. Elle pose d'abord la goutte sur l'oiseau. L'oiseau de bronze est à l'ombre, déjà. Le nez reçoit ensuite un rond tout calme. Une goutte de savon brille, prête à filer. Tu n'as pas soufflé trop fort. C'est pour toi. L'oiseau était plus frais, tu as vu.</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -9539,7 +9539,7 @@
 narrateur|Une goutte de savon brille, prête à filer.
 papa|Tu n'as pas soufflé trop fort.
 enfant-f|C'est pour toi.
-maman|Tu as laissé le bronze parler.</t>
+maman|L'oiseau était plus frais, tu as vu.</t>
         </is>
       </c>
     </row>
@@ -9566,12 +9566,12 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>De l'oiseau au nez, la bulle a glissé. On a commencé par l'oiseau. Tu n'as pas soufflé trop fort. Le bronze a parlé tout seul. Le flacon reste fermé, une goutte au bouchon. Un rond net reste sur le nez, puis pâlit.</t>
+          <t>De l'oiseau au nez, la bulle a glissé. On a commencé par l'oiseau. Tu n'as pas soufflé trop fort. L'oiseau était plus frais, d'abord. Le flacon reste fermé, une goutte au bouchon. Un rond net reste sur le nez, puis pâlit.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>De l'oiseau au nez, la bulle a glissé. On a commencé par l'oiseau. Tu n'as pas soufflé trop fort. Le bronze a parlé tout seul. Le flacon reste fermé, une goutte au bouchon. Un rond net reste sur le nez, puis pâlit.</t>
+          <t>De l'oiseau au nez, la bulle a glissé. On a commencé par l'oiseau. Tu n'as pas soufflé trop fort. L'oiseau était plus frais, d'abord. Le flacon reste fermé, une goutte au bouchon. Un rond net reste sur le nez, puis pâlit.</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -9709,7 +9709,7 @@
           <t>narrateur|De l'oiseau au nez, la bulle a glissé.
 enfant-f|On a commencé par l'oiseau.
 papa|Tu n'as pas soufflé trop fort.
-maman|Le bronze a parlé tout seul.
+maman|L'oiseau était plus frais, d'abord.
 narrateur|Le flacon reste fermé, une goutte au bouchon.
 narrateur|Un rond net reste sur le nez, puis pâlit.</t>
         </is>
@@ -9738,12 +9738,12 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Tout près, contre le bronze. Nina se glisse contre le socle, tout doux. Tout près, le savon n'a plus d'air chaud. La bulle n'a plus à voyager trop loin. Fermé, le savon attend contre son pouce. Tu t'es mise tout près, contre le nez. Le nez est là. Tu as observé d'abord.</t>
+          <t>Tout près, contre le bronze. Nina se glisse contre le socle, tout doux. Tout près, le savon n'a plus d'air chaud. La bulle n'a plus à voyager trop loin. Fermé, le savon attend contre son pouce. Tu t'es mise tout près, contre le nez. Le nez est là. Tu t'es mise tout contre.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>Tout près, contre le bronze. Nina se glisse contre le socle, tout doux. Tout près, le savon n'a plus d'air chaud. La bulle n'a plus à voyager trop loin. Fermé, le savon attend contre son pouce. Tu t'es mise tout près, contre le nez. Le nez est là. Tu as observé d'abord.</t>
+          <t>Tout près, contre le bronze. Nina se glisse contre le socle, tout doux. Tout près, le savon n'a plus d'air chaud. La bulle n'a plus à voyager trop loin. Fermé, le savon attend contre son pouce. Tu t'es mise tout près, contre le nez. Le nez est là. Tu t'es mise tout contre.</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -9885,7 +9885,7 @@
 narrateur|Fermé, le savon attend contre son pouce.
 papa|Tu t'es mise tout près, contre le nez.
 enfant-f|Le nez est là.
-maman|Tu as observé d'abord.</t>
+maman|Tu t'es mise tout contre.</t>
         </is>
       </c>
     </row>
@@ -9912,12 +9912,12 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Tout près, la bulle touche le nez, déjà. Je me suis mise tout près. Tu t'es glissée, comme l'ombre. Vous rentrez, les mains pleines de savon. Le flacon reste fermé, une goutte au bouchon. Le socle reste derrière, sans brûler.</t>
+          <t>Tout près, la bulle touche le nez, déjà. Je me suis mise tout près. Tu t'es glissée, comme l'ombre. Vos mains sentent encore le savon. Le flacon reste fermé, une goutte au bouchon. Le socle reste derrière, sans brûler.</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Tout près, la bulle touche le nez, déjà. Je me suis mise tout près. Tu t'es glissée, comme l'ombre. Vous rentrez, les mains pleines de savon. Le flacon reste fermé, une goutte au bouchon. Le socle reste derrière, sans brûler.</t>
+          <t>Tout près, la bulle touche le nez, déjà. Je me suis mise tout près. Tu t'es glissée, comme l'ombre. Vos mains sentent encore le savon. Le flacon reste fermé, une goutte au bouchon. Le socle reste derrière, sans brûler.</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -10055,7 +10055,7 @@
           <t>narrateur|Tout près, la bulle touche le nez, déjà.
 enfant-f|Je me suis mise tout près.
 papa|Tu t'es glissée, comme l'ombre.
-maman|Vous rentrez, les mains pleines de savon.
+maman|Vos mains sentent encore le savon.
 narrateur|Le flacon reste fermé, une goutte au bouchon.
 narrateur|Le socle reste derrière, sans brûler.</t>
         </is>
@@ -10084,12 +10084,12 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Dans sa paume, le flacon de savon est tiède. Le tilleul sent le miel, trop vif. La goutte s'envole, trop prise par le vent. Le vent prend tout ! Une feuille claque, puis une autre. La bulle part de travers, trop loin. Ça souffle trop, ici. Elle a besoin de temps. On fait comment, alors ? Tu trouves, Nina ?</t>
+          <t>Dans sa paume, le flacon de savon est tiède. Le tilleul agite ses feuilles, trop vite. La goutte s'envole, trop prise par le vent. Le vent prend tout ! Une feuille claque, puis une autre. La bulle part de travers, trop loin. Ici, ça souffle trop. Il lui faut du temps. Alors on fait quoi ? Tu vois comment, Nina ?</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Dans sa paume, le flacon de savon est tiède. Le tilleul sent le miel, trop vif. La goutte s'envole, trop prise par le vent. Le vent prend tout ! Une feuille claque, puis une autre. La bulle part de travers, trop loin. Ça souffle trop, ici. Elle a besoin de temps. On fait comment, alors ? Tu trouves, Nina ?</t>
+          <t>Dans sa paume, le flacon de savon est tiède. Le tilleul agite ses feuilles, trop vite. La goutte s'envole, trop prise par le vent. Le vent prend tout ! Une feuille claque, puis une autre. La bulle part de travers, trop loin. Ici, ça souffle trop. Il lui faut du temps. Alors on fait quoi ? Tu vois comment, Nina ?</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -10225,15 +10225,15 @@
       <c r="AW52" t="inlineStr">
         <is>
           <t>narrateur|Dans sa paume, le flacon de savon est tiède.
-narrateur|Le tilleul sent le miel, trop vif.
+narrateur|Le tilleul agite ses feuilles, trop vite.
 narrateur|La goutte s'envole, trop prise par le vent.
 enfant-f|Le vent prend tout !
 narrateur|Une feuille claque, puis une autre.
 narrateur|La bulle part de travers, trop loin.
-papa|Ça souffle trop, ici.
-maman|Elle a besoin de temps.
-enfant-f|On fait comment, alors ?
-papa|Tu trouves, Nina ?</t>
+papa|Ici, ça souffle trop.
+maman|Il lui faut du temps.
+enfant-f|Alors on fait quoi ?
+papa|Tu vois comment, Nina ?</t>
         </is>
       </c>
     </row>
@@ -10260,12 +10260,12 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>Les feuilles claquent encore, trop fort. Attendre les feuilles, derrière, ou tout petit ?</t>
+          <t>Les feuilles n'ont pas fini de claquer. Attendre les feuilles, derrière, ou tout petit ?</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>Les feuilles claquent encore, trop fort. Attendre les feuilles, derrière, ou tout petit ?</t>
+          <t>Les feuilles n'ont pas fini de claquer. Attendre les feuilles, derrière, ou tout petit ?</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -10428,7 +10428,7 @@
       </c>
       <c r="AW53" t="inlineStr">
         <is>
-          <t>narrateur|Les feuilles claquent encore, trop fort.
+          <t>narrateur|Les feuilles n'ont pas fini de claquer.
 papa|Attendre les feuilles, derrière, ou tout petit ?</t>
         </is>
       </c>
@@ -10456,12 +10456,12 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>On attend les feuilles, d'abord. Elle tient le savon, puis attend les feuilles. Les feuilles vont, reviennent, puis se taisent. L'air redevient un seul souffle, net. Fermé, le savon attend contre son pouce. Le tilleul n'a plus claqué. Maintenant, tu peux rester. Tu as attendu le calme.</t>
+          <t>On attend les feuilles, d'abord. Elle tient le savon, puis attend les feuilles. Les feuilles vont, reviennent, puis se taisent. L'air redevient un seul souffle, net. Fermé, le savon attend contre son pouce. Le tilleul n'a plus claqué. Maintenant, tu peux rester. Tu as laissé les feuilles finir.</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>On attend les feuilles, d'abord. Elle tient le savon, puis attend les feuilles. Les feuilles vont, reviennent, puis se taisent. L'air redevient un seul souffle, net. Fermé, le savon attend contre son pouce. Le tilleul n'a plus claqué. Maintenant, tu peux rester. Tu as attendu le calme.</t>
+          <t>On attend les feuilles, d'abord. Elle tient le savon, puis attend les feuilles. Les feuilles vont, reviennent, puis se taisent. L'air redevient un seul souffle, net. Fermé, le savon attend contre son pouce. Le tilleul n'a plus claqué. Maintenant, tu peux rester. Tu as laissé les feuilles finir.</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -10603,7 +10603,7 @@
 narrateur|Fermé, le savon attend contre son pouce.
 papa|Le tilleul n'a plus claqué.
 enfant-f|Maintenant, tu peux rester.
-maman|Tu as attendu le calme.</t>
+maman|Tu as laissé les feuilles finir.</t>
         </is>
       </c>
     </row>
@@ -10802,12 +10802,12 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Derrière, pas trop près du vent. Derrière le tronc, le savon ne s'envole plus. Nina se glisse derrière le tronc, tout bas. Rien ne claque, rien ne pousse plus. Une goutte de savon brille, prête à filer. Tu n'as pas couru. Tu es ronde, maintenant. Tu as préparé le chemin.</t>
+          <t>Derrière, pas trop près du vent. Derrière le tronc, le savon ne s'envole plus. Nina se glisse derrière le tronc, tout bas. Rien ne claque, rien ne pousse plus. Une goutte de savon brille, prête à filer. Tu n'as pas couru. Tu es ronde, maintenant. Derrière, l'air était plus doux.</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Derrière, pas trop près du vent. Derrière le tronc, le savon ne s'envole plus. Nina se glisse derrière le tronc, tout bas. Rien ne claque, rien ne pousse plus. Une goutte de savon brille, prête à filer. Tu n'as pas couru. Tu es ronde, maintenant. Tu as préparé le chemin.</t>
+          <t>Derrière, pas trop près du vent. Derrière le tronc, le savon ne s'envole plus. Nina se glisse derrière le tronc, tout bas. Rien ne claque, rien ne pousse plus. Une goutte de savon brille, prête à filer. Tu n'as pas couru. Tu es ronde, maintenant. Derrière, l'air était plus doux.</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -10949,7 +10949,7 @@
 narrateur|Une goutte de savon brille, prête à filer.
 papa|Tu n'as pas couru.
 enfant-f|Tu es ronde, maintenant.
-maman|Tu as préparé le chemin.</t>
+maman|Derrière, l'air était plus doux.</t>
         </is>
       </c>
     </row>
@@ -11148,12 +11148,12 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Tout petit, tout serré. Une toute petite bulle quitte le savon. Nina souffle à peine, sans prendre le vent. Le tilleul se tait, plus loin, tout seul. Fermé, le savon attend contre son pouce. Le petit rond n'a pas volé. Tu restes, bulle. Le petit tenait assez.</t>
+          <t>Tout petit, tout serré. Une toute petite bulle quitte le savon. Nina souffle à peine, sans prendre le vent. Le tilleul se tait, plus loin, tout seul. Une goutte de savon brille, prête à filer. Le petit rond n'a pas volé. Tu restes, bulle. Le petit rond a suffi.</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Tout petit, tout serré. Une toute petite bulle quitte le savon. Nina souffle à peine, sans prendre le vent. Le tilleul se tait, plus loin, tout seul. Fermé, le savon attend contre son pouce. Le petit rond n'a pas volé. Tu restes, bulle. Le petit tenait assez.</t>
+          <t>Tout petit, tout serré. Une toute petite bulle quitte le savon. Nina souffle à peine, sans prendre le vent. Le tilleul se tait, plus loin, tout seul. Une goutte de savon brille, prête à filer. Le petit rond n'a pas volé. Tu restes, bulle. Le petit rond a suffi.</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -11292,10 +11292,10 @@
 narrateur|Une toute petite bulle quitte le savon.
 narrateur|Nina souffle à peine, sans prendre le vent.
 narrateur|Le tilleul se tait, plus loin, tout seul.
-narrateur|Fermé, le savon attend contre son pouce.
+narrateur|Une goutte de savon brille, prête à filer.
 papa|Le petit rond n'a pas volé.
 enfant-f|Tu restes, bulle.
-maman|Le petit tenait assez.</t>
+maman|Le petit rond a suffi.</t>
         </is>
       </c>
     </row>
@@ -11322,12 +11322,12 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Tout petit, le rond tient sur le nez, tout calme. On a soufflé à peine. Le petit rond n'a pas volé. Rentrez, le savon est déjà sec. Le flacon reste fermé, une goutte au bouchon. Le tilleul se tait, plus loin, tout seul.</t>
+          <t>Tout petit, le rond tient sur le nez, tout calme. On a soufflé à peine. Le petit rond n'a pas volé. Le savon est déjà sec, on rentre. Le flacon reste fermé, une goutte au bouchon. Le tilleul se tait, plus loin, tout seul.</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Tout petit, le rond tient sur le nez, tout calme. On a soufflé à peine. Le petit rond n'a pas volé. Rentrez, le savon est déjà sec. Le flacon reste fermé, une goutte au bouchon. Le tilleul se tait, plus loin, tout seul.</t>
+          <t>Tout petit, le rond tient sur le nez, tout calme. On a soufflé à peine. Le petit rond n'a pas volé. Le savon est déjà sec, on rentre. Le flacon reste fermé, une goutte au bouchon. Le tilleul se tait, plus loin, tout seul.</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -11465,7 +11465,7 @@
           <t>narrateur|Tout petit, le rond tient sur le nez, tout calme.
 enfant-f|On a soufflé à peine.
 papa|Le petit rond n'a pas volé.
-maman|Rentrez, le savon est déjà sec.
+maman|Le savon est déjà sec, on rentre.
 narrateur|Le flacon reste fermé, une goutte au bouchon.
 narrateur|Le tilleul se tait, plus loin, tout seul.</t>
         </is>
@@ -11494,12 +11494,12 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Nina prend d'abord la coupelle, encore un peu tiède. Elle va garder le savon. Tiens-la plate, tout doux. Le rond d'eau tremble, puis se tait. Le bâton et le savon, avec vous. Il les pose près de son genou. Rien ne reste près du banc. Je te porte, coupelle. Un cercle de savon brille au fond. La coupelle d'abord, elle est prête.</t>
+          <t>Nina lève d'abord la coupelle, bien à plat. Le savon va dormir dedans. Pas trop d'eau, juste un miroir. Le rond tremble, puis s'arrête. Voici le bâton, et le savon. Il les glisse contre son genou. Le gravier reste vide, derrière eux. Coupelle, je te porte. Un cercle de savon brille au fond. La coupelle est prête, on avance.</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>Nina prend d'abord la coupelle, encore un peu tiède. Elle va garder le savon. Tiens-la plate, tout doux. Le rond d'eau tremble, puis se tait. Le bâton et le savon, avec vous. Il les pose près de son genou. Rien ne reste près du banc. Je te porte, coupelle. Un cercle de savon brille au fond. La coupelle d'abord, elle est prête.</t>
+          <t>Nina lève d'abord la coupelle, bien à plat. Le savon va dormir dedans. Pas trop d'eau, juste un miroir. Le rond tremble, puis s'arrête. Voici le bâton, et le savon. Il les glisse contre son genou. Le gravier reste vide, derrière eux. Coupelle, je te porte. Un cercle de savon brille au fond. La coupelle est prête, on avance.</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -11634,16 +11634,16 @@
       <c r="AV60" s="2" t="inlineStr"/>
       <c r="AW60" t="inlineStr">
         <is>
-          <t>narrateur|Nina prend d'abord la coupelle, encore un peu tiède.
-enfant-f|Elle va garder le savon.
-maman|Tiens-la plate, tout doux.
-narrateur|Le rond d'eau tremble, puis se tait.
-papa|Le bâton et le savon, avec vous.
-narrateur|Il les pose près de son genou.
-narrateur|Rien ne reste près du banc.
-enfant-f|Je te porte, coupelle.
+          <t>narrateur|Nina lève d'abord la coupelle, bien à plat.
+enfant-f|Le savon va dormir dedans.
+maman|Pas trop d'eau, juste un miroir.
+narrateur|Le rond tremble, puis s'arrête.
+papa|Voici le bâton, et le savon.
+narrateur|Il les glisse contre son genou.
+narrateur|Le gravier reste vide, derrière eux.
+enfant-f|Coupelle, je te porte.
 narrateur|Un cercle de savon brille au fond.
-papa|La coupelle d'abord, elle est prête.</t>
+papa|La coupelle est prête, on avance.</t>
         </is>
       </c>
     </row>
@@ -11854,12 +11854,12 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>La coupelle reste plate, contre son ventre. Elle va porter le savon. Le rond sent encore le miel. On y va, tous les trois ? Oui. Le rond de savon attend, tout calme.</t>
+          <t>La coupelle reste plate, contre son ventre. Le savon ne verse pas. Le rond sent encore le miel. On avance, tous les trois ? Oui. Le rond de savon attend, tout calme.</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>La coupelle reste plate, contre son ventre. Elle va porter le savon. Le rond sent encore le miel. On y va, tous les trois ? Oui. Le rond de savon attend, tout calme.</t>
+          <t>La coupelle reste plate, contre son ventre. Le savon ne verse pas. Le rond sent encore le miel. On avance, tous les trois ? Oui. Le rond de savon attend, tout calme.</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -11999,9 +11999,9 @@
       <c r="AW62" t="inlineStr">
         <is>
           <t>narrateur|La coupelle reste plate, contre son ventre.
-enfant-f|Elle va porter le savon.
+enfant-f|Le savon ne verse pas.
 maman|Le rond sent encore le miel.
-papa|On y va, tous les trois ?
+papa|On avance, tous les trois ?
 enfant-f|Oui.
 narrateur|Le rond de savon attend, tout calme.</t>
         </is>
@@ -12030,12 +12030,12 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>La coupelle tape le ventre, tout doux. L'allée soulève déjà trop de poussière. Plus loin, le socle brûle encore. Sous le tilleul, les feuilles claquent. Nina, vous partez où ?</t>
+          <t>La coupelle appuie contre son ventre. Devant, l'allée soulève trop de poussière. Le socle, lui, brûle encore au soleil. Sous le tilleul, les feuilles claquent. Nina, tu vas où ?</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>La coupelle tape le ventre, tout doux. L'allée soulève déjà trop de poussière. Plus loin, le socle brûle encore. Sous le tilleul, les feuilles claquent. Nina, vous partez où ?</t>
+          <t>La coupelle appuie contre son ventre. Devant, l'allée soulève trop de poussière. Le socle, lui, brûle encore au soleil. Sous le tilleul, les feuilles claquent. Nina, tu vas où ?</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -12194,11 +12194,11 @@
       <c r="AV63" s="2" t="inlineStr"/>
       <c r="AW63" t="inlineStr">
         <is>
-          <t>narrateur|La coupelle tape le ventre, tout doux.
-narrateur|L'allée soulève déjà trop de poussière.
-narrateur|Plus loin, le socle brûle encore.
+          <t>narrateur|La coupelle appuie contre son ventre.
+narrateur|Devant, l'allée soulève trop de poussière.
+narrateur|Le socle, lui, brûle encore au soleil.
 narrateur|Sous le tilleul, les feuilles claquent.
-papa|Nina, vous partez où ?</t>
+papa|Nina, tu vas où ?</t>
         </is>
       </c>
     </row>
@@ -12225,12 +12225,12 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Contre son ventre, la coupelle reste bien plate. L'allée sent le gravier chaud, trop vif. Le rond se plisse, trop agité, trop gris. Ma bulle a sauté ! Un pas soulève la poussière, encore. La bulle n'a plus le temps d'arriver. Ça bouge trop, ici. Elle a besoin de calme. On fait comment, alors ? Tu trouves, Nina ?</t>
+          <t>Contre son ventre, la coupelle reste bien plate. Le gravier de l'allée saute sous les pas. Le rond se plisse, trop agité, trop gris. Ma bulle a crevé ! Encore un pas, encore de la poussière. Le nez reste trop loin, trop gris. Ici, ça n'arrête pas. La bulle a besoin de calme. Alors on fait quoi ? Tu vois comment, Nina ?</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Contre son ventre, la coupelle reste bien plate. L'allée sent le gravier chaud, trop vif. Le rond se plisse, trop agité, trop gris. Ma bulle a sauté ! Un pas soulève la poussière, encore. La bulle n'a plus le temps d'arriver. Ça bouge trop, ici. Elle a besoin de calme. On fait comment, alors ? Tu trouves, Nina ?</t>
+          <t>Contre son ventre, la coupelle reste bien plate. Le gravier de l'allée saute sous les pas. Le rond se plisse, trop agité, trop gris. Ma bulle a crevé ! Encore un pas, encore de la poussière. Le nez reste trop loin, trop gris. Ici, ça n'arrête pas. La bulle a besoin de calme. Alors on fait quoi ? Tu vois comment, Nina ?</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -12366,15 +12366,15 @@
       <c r="AW64" t="inlineStr">
         <is>
           <t>narrateur|Contre son ventre, la coupelle reste bien plate.
-narrateur|L'allée sent le gravier chaud, trop vif.
+narrateur|Le gravier de l'allée saute sous les pas.
 narrateur|Le rond se plisse, trop agité, trop gris.
-enfant-f|Ma bulle a sauté !
-narrateur|Un pas soulève la poussière, encore.
-narrateur|La bulle n'a plus le temps d'arriver.
-papa|Ça bouge trop, ici.
-maman|Elle a besoin de calme.
-enfant-f|On fait comment, alors ?
-papa|Tu trouves, Nina ?</t>
+enfant-f|Ma bulle a crevé !
+narrateur|Encore un pas, encore de la poussière.
+narrateur|Le nez reste trop loin, trop gris.
+papa|Ici, ça n'arrête pas.
+maman|La bulle a besoin de calme.
+enfant-f|Alors on fait quoi ?
+papa|Tu vois comment, Nina ?</t>
         </is>
       </c>
     </row>
@@ -12401,12 +12401,12 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>L'allée soulève encore trop de poussière. Attendre les pas, plus bas, ou le bord ?</t>
+          <t>L'allée n'a pas fini de soulever. Attendre les pas, plus bas, ou le bord ?</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>L'allée soulève encore trop de poussière. Attendre les pas, plus bas, ou le bord ?</t>
+          <t>L'allée n'a pas fini de soulever. Attendre les pas, plus bas, ou le bord ?</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -12569,7 +12569,7 @@
       </c>
       <c r="AW65" t="inlineStr">
         <is>
-          <t>narrateur|L'allée soulève encore trop de poussière.
+          <t>narrateur|L'allée n'a pas fini de soulever.
 papa|Attendre les pas, plus bas, ou le bord ?</t>
         </is>
       </c>
@@ -12597,12 +12597,12 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>On attend les pas. Elle tient la coupelle, sans verser encore. Le gravier se tait, une fois, puis plus. Tu peux partir, maintenant. Plate, la coupelle attend, sans verser. Les pas se sont tus, maintenant. La bulle part, ronde, tout calme. Tu lui as laissé le temps.</t>
+          <t>On attend les pas. Elle tient la coupelle, sans verser encore. Le gravier se tait, une fois, puis plus. Tu peux partir, maintenant. Plate, la coupelle attend, sans verser. Les pas se sont tus, maintenant. La bulle part, ronde, tout calme. Tu as attendu, et elle est partie.</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>On attend les pas. Elle tient la coupelle, sans verser encore. Le gravier se tait, une fois, puis plus. Tu peux partir, maintenant. Plate, la coupelle attend, sans verser. Les pas se sont tus, maintenant. La bulle part, ronde, tout calme. Tu lui as laissé le temps.</t>
+          <t>On attend les pas. Elle tient la coupelle, sans verser encore. Le gravier se tait, une fois, puis plus. Tu peux partir, maintenant. Plate, la coupelle attend, sans verser. Les pas se sont tus, maintenant. La bulle part, ronde, tout calme. Tu as attendu, et elle est partie.</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -12744,7 +12744,7 @@
 narrateur|Plate, la coupelle attend, sans verser.
 papa|Les pas se sont tus, maintenant.
 narrateur|La bulle part, ronde, tout calme.
-maman|Tu lui as laissé le temps.</t>
+maman|Tu as attendu, et elle est partie.</t>
         </is>
       </c>
     </row>
@@ -12771,12 +12771,12 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>La bulle se pose, ronde, sur le nez de bronze. On a attendu les pas. Merci d'avoir laissé le gravier se taire. Rentrez, la cloche n'a pas encore sonné. La coupelle sèche près du gravier, un cercle de savon. Une poussière tourne encore, puis s'arrête.</t>
+          <t>La bulle se pose, ronde, sur le nez de bronze. On a attendu les pas. Merci d'avoir laissé le gravier se taire. La cloche n'a pas encore sonné. La coupelle sèche près du gravier, un cercle de savon. Un grain de poussière retombe, puis plus rien.</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>La bulle se pose, ronde, sur le nez de bronze. On a attendu les pas. Merci d'avoir laissé le gravier se taire. Rentrez, la cloche n'a pas encore sonné. La coupelle sèche près du gravier, un cercle de savon. Une poussière tourne encore, puis s'arrête.</t>
+          <t>La bulle se pose, ronde, sur le nez de bronze. On a attendu les pas. Merci d'avoir laissé le gravier se taire. La cloche n'a pas encore sonné. La coupelle sèche près du gravier, un cercle de savon. Un grain de poussière retombe, puis plus rien.</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -12914,9 +12914,9 @@
           <t>narrateur|La bulle se pose, ronde, sur le nez de bronze.
 enfant-f|On a attendu les pas.
 papa|Merci d'avoir laissé le gravier se taire.
-maman|Rentrez, la cloche n'a pas encore sonné.
+maman|La cloche n'a pas encore sonné.
 narrateur|La coupelle sèche près du gravier, un cercle de savon.
-narrateur|Une poussière tourne encore, puis s'arrête.</t>
+narrateur|Un grain de poussière retombe, puis plus rien.</t>
         </is>
       </c>
     </row>
@@ -12943,12 +12943,12 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Plus bas, d'abord. Elle baisse la coupelle, loin de la poussière. Nina s'accroupit, les genoux au gravier. L'air est plus doux, près de l'herbe. Le rond de savon attend, tout calme. Tu as regardé d'abord. Ici, tu ne sautes plus. Le bas était plus calme.</t>
+          <t>Plus bas, d'abord. Elle baisse la coupelle, loin de la poussière. Nina s'accroupit, les genoux au gravier. L'air est plus doux, près de l'herbe. Le rond de savon attend, tout calme. Tu as vu l'herbe, avant. Ici, tu ne crèves plus. Près du sol, ça tenait mieux.</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>Plus bas, d'abord. Elle baisse la coupelle, loin de la poussière. Nina s'accroupit, les genoux au gravier. L'air est plus doux, près de l'herbe. Le rond de savon attend, tout calme. Tu as regardé d'abord. Ici, tu ne sautes plus. Le bas était plus calme.</t>
+          <t>Plus bas, d'abord. Elle baisse la coupelle, loin de la poussière. Nina s'accroupit, les genoux au gravier. L'air est plus doux, près de l'herbe. Le rond de savon attend, tout calme. Tu as vu l'herbe, avant. Ici, tu ne crèves plus. Près du sol, ça tenait mieux.</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -13088,9 +13088,9 @@
 narrateur|Nina s'accroupit, les genoux au gravier.
 narrateur|L'air est plus doux, près de l'herbe.
 narrateur|Le rond de savon attend, tout calme.
-papa|Tu as regardé d'abord.
-enfant-f|Ici, tu ne sautes plus.
-maman|Le bas était plus calme.</t>
+papa|Tu as vu l'herbe, avant.
+enfant-f|Ici, tu ne crèves plus.
+maman|Près du sol, ça tenait mieux.</t>
         </is>
       </c>
     </row>
@@ -13117,12 +13117,12 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Plus bas, la bulle monte jusqu'au nez. On s'est baissées, d'abord. Tu as regardé avant de souffler. Essuie tes genoux, sur le paillasson. La coupelle sèche près du gravier, un cercle de savon. Un rond d'ombre reste au bas du bronze.</t>
+          <t>Plus bas, la bulle monte jusqu'au nez. On s'est baissées, d'abord. Tu as vu l'herbe avant de souffler. Essuie tes genoux, on rentre. La coupelle sèche près du gravier, un cercle de savon. Un rond d'ombre reste au bas du bronze.</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>Plus bas, la bulle monte jusqu'au nez. On s'est baissées, d'abord. Tu as regardé avant de souffler. Essuie tes genoux, sur le paillasson. La coupelle sèche près du gravier, un cercle de savon. Un rond d'ombre reste au bas du bronze.</t>
+          <t>Plus bas, la bulle monte jusqu'au nez. On s'est baissées, d'abord. Tu as vu l'herbe avant de souffler. Essuie tes genoux, on rentre. La coupelle sèche près du gravier, un cercle de savon. Un rond d'ombre reste au bas du bronze.</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -13259,8 +13259,8 @@
         <is>
           <t>narrateur|Plus bas, la bulle monte jusqu'au nez.
 enfant-f|On s'est baissées, d'abord.
-papa|Tu as regardé avant de souffler.
-maman|Essuie tes genoux, sur le paillasson.
+papa|Tu as vu l'herbe avant de souffler.
+maman|Essuie tes genoux, on rentre.
 narrateur|La coupelle sèche près du gravier, un cercle de savon.
 narrateur|Un rond d'ombre reste au bas du bronze.</t>
         </is>
@@ -13289,12 +13289,12 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Au bord, tout petit. Elle glisse la coupelle vers le bord d'herbe. L'herbe tient, sans laisser la poussière. Nina répète, tout bas, encore une fois. Plate, la coupelle attend, sans verser. Le bord n'a pas soulevé. Tu es à l'abri. Tu as parlé lentement.</t>
+          <t>Au bord, tout petit. Elle glisse la coupelle vers le bord d'herbe. L'herbe tient, sans laisser la poussière. Nina répète, tout bas, encore une fois. Plate, la coupelle attend, sans verser. Le bord n'a pas soulevé. Tu es à l'abri. Tu as dit ça tout bas.</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>Au bord, tout petit. Elle glisse la coupelle vers le bord d'herbe. L'herbe tient, sans laisser la poussière. Nina répète, tout bas, encore une fois. Plate, la coupelle attend, sans verser. Le bord n'a pas soulevé. Tu es à l'abri. Tu as parlé lentement.</t>
+          <t>Au bord, tout petit. Elle glisse la coupelle vers le bord d'herbe. L'herbe tient, sans laisser la poussière. Nina répète, tout bas, encore une fois. Plate, la coupelle attend, sans verser. Le bord n'a pas soulevé. Tu es à l'abri. Tu as dit ça tout bas.</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -13436,7 +13436,7 @@
 narrateur|Plate, la coupelle attend, sans verser.
 papa|Le bord n'a pas soulevé.
 enfant-f|Tu es à l'abri.
-maman|Tu as parlé lentement.</t>
+maman|Tu as dit ça tout bas.</t>
         </is>
       </c>
     </row>
@@ -13635,12 +13635,12 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Contre son ventre, la coupelle reste bien plate. Le bronze sent le soleil, encore trop fort. Le rond fume un peu, trop chaud. Le nez est trop chaud ! Une bulle touche, puis crève, trop vite. Le nez n'a plus de rond, trop nu. Ça brûle trop, ici. Elle n'avance plus. On fait comment, alors ? Tu trouves, Nina ?</t>
+          <t>Contre son ventre, la coupelle reste bien plate. Le bronze tient encore tout le soleil. Le rond tremble, trop chaud, trop mince. Le nez brûle trop ! La bulle touche, puis crève tout de suite. Il ne reste rien sur le bronze. Ici, c'est trop chaud. La bulle n'arrive pas. Alors on fait quoi ? Tu vois comment, Nina ?</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>Contre son ventre, la coupelle reste bien plate. Le bronze sent le soleil, encore trop fort. Le rond fume un peu, trop chaud. Le nez est trop chaud ! Une bulle touche, puis crève, trop vite. Le nez n'a plus de rond, trop nu. Ça brûle trop, ici. Elle n'avance plus. On fait comment, alors ? Tu trouves, Nina ?</t>
+          <t>Contre son ventre, la coupelle reste bien plate. Le bronze tient encore tout le soleil. Le rond tremble, trop chaud, trop mince. Le nez brûle trop ! La bulle touche, puis crève tout de suite. Il ne reste rien sur le bronze. Ici, c'est trop chaud. La bulle n'arrive pas. Alors on fait quoi ? Tu vois comment, Nina ?</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -13776,15 +13776,15 @@
       <c r="AW72" t="inlineStr">
         <is>
           <t>narrateur|Contre son ventre, la coupelle reste bien plate.
-narrateur|Le bronze sent le soleil, encore trop fort.
-narrateur|Le rond fume un peu, trop chaud.
-enfant-f|Le nez est trop chaud !
-narrateur|Une bulle touche, puis crève, trop vite.
-narrateur|Le nez n'a plus de rond, trop nu.
-papa|Ça brûle trop, ici.
-maman|Elle n'avance plus.
-enfant-f|On fait comment, alors ?
-maman|Tu trouves, Nina ?</t>
+narrateur|Le bronze tient encore tout le soleil.
+narrateur|Le rond tremble, trop chaud, trop mince.
+enfant-f|Le nez brûle trop !
+narrateur|La bulle touche, puis crève tout de suite.
+narrateur|Il ne reste rien sur le bronze.
+papa|Ici, c'est trop chaud.
+maman|La bulle n'arrive pas.
+enfant-f|Alors on fait quoi ?
+maman|Tu vois comment, Nina ?</t>
         </is>
       </c>
     </row>
@@ -13811,12 +13811,12 @@
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>Le bronze brûle encore, trop fort. Attendre l'ombre, l'oiseau, ou tout près ?</t>
+          <t>Le bronze n'a pas fini de brûler. Attendre l'ombre, l'oiseau, ou tout près ?</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>Le bronze brûle encore, trop fort. Attendre l'ombre, l'oiseau, ou tout près ?</t>
+          <t>Le bronze n'a pas fini de brûler. Attendre l'ombre, l'oiseau, ou tout près ?</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -13979,7 +13979,7 @@
       </c>
       <c r="AW73" t="inlineStr">
         <is>
-          <t>narrateur|Le bronze brûle encore, trop fort.
+          <t>narrateur|Le bronze n'a pas fini de brûler.
 maman|Attendre l'ombre, l'oiseau, ou tout près ?</t>
         </is>
       </c>
@@ -14007,12 +14007,12 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>On attend l'ombre. Une ombre de tilleul glisse sur le nez. Sous l'ombre, la coupelle ne fume plus. Le bronze se tait, puis se refroidit. Plate, la coupelle attend, sans verser. Le nez est redevenu doux. Maintenant, tu me vois. Tu as attendu le silence.</t>
+          <t>On attend l'ombre. Une ombre de tilleul glisse sur le nez. Sous l'ombre, la coupelle ne fume plus. Le bronze se tait, puis se refroidit. Plate, la coupelle attend, sans verser. Le nez est redevenu doux. Maintenant, tu me vois. Tu as laissé l'ombre arriver.</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>On attend l'ombre. Une ombre de tilleul glisse sur le nez. Sous l'ombre, la coupelle ne fume plus. Le bronze se tait, puis se refroidit. Plate, la coupelle attend, sans verser. Le nez est redevenu doux. Maintenant, tu me vois. Tu as attendu le silence.</t>
+          <t>On attend l'ombre. Une ombre de tilleul glisse sur le nez. Sous l'ombre, la coupelle ne fume plus. Le bronze se tait, puis se refroidit. Plate, la coupelle attend, sans verser. Le nez est redevenu doux. Maintenant, tu me vois. Tu as laissé l'ombre arriver.</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -14154,7 +14154,7 @@
 narrateur|Plate, la coupelle attend, sans verser.
 maman|Le nez est redevenu doux.
 enfant-f|Maintenant, tu me vois.
-papa|Tu as attendu le silence.</t>
+papa|Tu as laissé l'ombre arriver.</t>
         </is>
       </c>
     </row>
@@ -14181,12 +14181,12 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Quand l'ombre a touché, la bulle a tenu. On a attendu le tilleul. Le silence vous a aidées. Le bronze sent encore le soleil, moins fort. La coupelle sèche près du gravier, un cercle de savon. Un pli d'ombre se recouche, tout lent.</t>
+          <t>Quand l'ombre a touché, la bulle a tenu. On a attendu le tilleul. L'ombre vous a aidées. Le bronze sent encore le soleil, moins fort. La coupelle sèche près du gravier, un cercle de savon. L'ombre reste un moment, puis glisse.</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>Quand l'ombre a touché, la bulle a tenu. On a attendu le tilleul. Le silence vous a aidées. Le bronze sent encore le soleil, moins fort. La coupelle sèche près du gravier, un cercle de savon. Un pli d'ombre se recouche, tout lent.</t>
+          <t>Quand l'ombre a touché, la bulle a tenu. On a attendu le tilleul. L'ombre vous a aidées. Le bronze sent encore le soleil, moins fort. La coupelle sèche près du gravier, un cercle de savon. L'ombre reste un moment, puis glisse.</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -14323,10 +14323,10 @@
         <is>
           <t>narrateur|Quand l'ombre a touché, la bulle a tenu.
 enfant-f|On a attendu le tilleul.
-papa|Le silence vous a aidées.
+papa|L'ombre vous a aidées.
 maman|Le bronze sent encore le soleil, moins fort.
 narrateur|La coupelle sèche près du gravier, un cercle de savon.
-narrateur|Un pli d'ombre se recouche, tout lent.</t>
+narrateur|L'ombre reste un moment, puis glisse.</t>
         </is>
       </c>
     </row>
@@ -14353,12 +14353,12 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>L'oiseau, d'abord, il est plus frais. Elle pose d'abord le rond sur l'oiseau. L'oiseau de bronze est à l'ombre, déjà. Le nez reçoit ensuite un rond tout calme. Le rond de savon attend, tout calme. Tu n'as pas soufflé trop fort. C'est pour toi. Tu as laissé le bronze parler.</t>
+          <t>L'oiseau, d'abord, il est plus frais. Elle pose d'abord le rond sur l'oiseau. L'oiseau de bronze est à l'ombre, déjà. Le nez reçoit ensuite un rond tout calme. Le rond de savon attend, tout calme. Tu n'as pas soufflé trop fort. C'est pour toi. L'oiseau était plus frais, tu as vu.</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>L'oiseau, d'abord, il est plus frais. Elle pose d'abord le rond sur l'oiseau. L'oiseau de bronze est à l'ombre, déjà. Le nez reçoit ensuite un rond tout calme. Le rond de savon attend, tout calme. Tu n'as pas soufflé trop fort. C'est pour toi. Tu as laissé le bronze parler.</t>
+          <t>L'oiseau, d'abord, il est plus frais. Elle pose d'abord le rond sur l'oiseau. L'oiseau de bronze est à l'ombre, déjà. Le nez reçoit ensuite un rond tout calme. Le rond de savon attend, tout calme. Tu n'as pas soufflé trop fort. C'est pour toi. L'oiseau était plus frais, tu as vu.</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -14500,7 +14500,7 @@
 narrateur|Le rond de savon attend, tout calme.
 papa|Tu n'as pas soufflé trop fort.
 enfant-f|C'est pour toi.
-maman|Tu as laissé le bronze parler.</t>
+maman|L'oiseau était plus frais, tu as vu.</t>
         </is>
       </c>
     </row>
@@ -14527,12 +14527,12 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>De l'oiseau au nez, la bulle a glissé. On a commencé par l'oiseau. Tu n'as pas soufflé trop fort. Le bronze a parlé tout seul. La coupelle sèche près du gravier, un cercle de savon. Un rond net reste sur le nez, puis pâlit.</t>
+          <t>De l'oiseau au nez, la bulle a glissé. On a commencé par l'oiseau. Tu n'as pas soufflé trop fort. L'oiseau était plus frais, d'abord. La coupelle sèche près du gravier, un cercle de savon. Un rond net reste sur le nez, puis pâlit.</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>De l'oiseau au nez, la bulle a glissé. On a commencé par l'oiseau. Tu n'as pas soufflé trop fort. Le bronze a parlé tout seul. La coupelle sèche près du gravier, un cercle de savon. Un rond net reste sur le nez, puis pâlit.</t>
+          <t>De l'oiseau au nez, la bulle a glissé. On a commencé par l'oiseau. Tu n'as pas soufflé trop fort. L'oiseau était plus frais, d'abord. La coupelle sèche près du gravier, un cercle de savon. Un rond net reste sur le nez, puis pâlit.</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -14670,7 +14670,7 @@
           <t>narrateur|De l'oiseau au nez, la bulle a glissé.
 enfant-f|On a commencé par l'oiseau.
 papa|Tu n'as pas soufflé trop fort.
-maman|Le bronze a parlé tout seul.
+maman|L'oiseau était plus frais, d'abord.
 narrateur|La coupelle sèche près du gravier, un cercle de savon.
 narrateur|Un rond net reste sur le nez, puis pâlit.</t>
         </is>
@@ -14699,12 +14699,12 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Tout près, contre le bronze. Nina se glisse contre le socle, tout doux. Tout près, la coupelle n'a plus d'air chaud. La bulle n'a plus à voyager trop loin. Plate, la coupelle attend, sans verser. Tu t'es mise tout près, contre le nez. Le nez est là. Tu as observé d'abord.</t>
+          <t>Tout près, contre le bronze. Nina se glisse contre le socle, tout doux. Tout près, la coupelle n'a plus d'air chaud. La bulle n'a plus à voyager trop loin. Plate, la coupelle attend, sans verser. Tu t'es mise tout près, contre le nez. Le nez est là. Tu t'es mise tout contre.</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>Tout près, contre le bronze. Nina se glisse contre le socle, tout doux. Tout près, la coupelle n'a plus d'air chaud. La bulle n'a plus à voyager trop loin. Plate, la coupelle attend, sans verser. Tu t'es mise tout près, contre le nez. Le nez est là. Tu as observé d'abord.</t>
+          <t>Tout près, contre le bronze. Nina se glisse contre le socle, tout doux. Tout près, la coupelle n'a plus d'air chaud. La bulle n'a plus à voyager trop loin. Plate, la coupelle attend, sans verser. Tu t'es mise tout près, contre le nez. Le nez est là. Tu t'es mise tout contre.</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -14846,7 +14846,7 @@
 narrateur|Plate, la coupelle attend, sans verser.
 papa|Tu t'es mise tout près, contre le nez.
 enfant-f|Le nez est là.
-maman|Tu as observé d'abord.</t>
+maman|Tu t'es mise tout contre.</t>
         </is>
       </c>
     </row>
@@ -14873,12 +14873,12 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>Tout près, la bulle touche le nez, déjà. Je me suis mise tout près. Tu t'es glissée, comme l'ombre. Vous rentrez, les mains pleines de savon. La coupelle sèche près du gravier, un cercle de savon. Le socle reste derrière, sans brûler.</t>
+          <t>Tout près, la bulle touche le nez, déjà. Je me suis mise tout près. Tu t'es glissée, comme l'ombre. Vos mains sentent encore le savon. La coupelle sèche près du gravier, un cercle de savon. Le socle reste derrière, sans brûler.</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>Tout près, la bulle touche le nez, déjà. Je me suis mise tout près. Tu t'es glissée, comme l'ombre. Vous rentrez, les mains pleines de savon. La coupelle sèche près du gravier, un cercle de savon. Le socle reste derrière, sans brûler.</t>
+          <t>Tout près, la bulle touche le nez, déjà. Je me suis mise tout près. Tu t'es glissée, comme l'ombre. Vos mains sentent encore le savon. La coupelle sèche près du gravier, un cercle de savon. Le socle reste derrière, sans brûler.</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -15016,7 +15016,7 @@
           <t>narrateur|Tout près, la bulle touche le nez, déjà.
 enfant-f|Je me suis mise tout près.
 papa|Tu t'es glissée, comme l'ombre.
-maman|Vous rentrez, les mains pleines de savon.
+maman|Vos mains sentent encore le savon.
 narrateur|La coupelle sèche près du gravier, un cercle de savon.
 narrateur|Le socle reste derrière, sans brûler.</t>
         </is>
@@ -15045,12 +15045,12 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Contre son ventre, la coupelle reste bien plate. Le tilleul sent le miel, trop vif. Le rond se plie, trop poussé par les feuilles. Le vent prend tout ! Une feuille claque, puis une autre. La bulle part de travers, trop loin. Ça souffle trop, ici. Elle a besoin de temps. On fait comment, alors ? Tu trouves, Nina ?</t>
+          <t>Contre son ventre, la coupelle reste bien plate. Le tilleul agite ses feuilles, trop vite. Le rond se plie, trop poussé par les feuilles. Le vent prend tout ! Une feuille claque, puis une autre. La bulle part de travers, trop loin. Ici, ça souffle trop. Il lui faut du temps. Alors on fait quoi ? Tu vois comment, Nina ?</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>Contre son ventre, la coupelle reste bien plate. Le tilleul sent le miel, trop vif. Le rond se plie, trop poussé par les feuilles. Le vent prend tout ! Une feuille claque, puis une autre. La bulle part de travers, trop loin. Ça souffle trop, ici. Elle a besoin de temps. On fait comment, alors ? Tu trouves, Nina ?</t>
+          <t>Contre son ventre, la coupelle reste bien plate. Le tilleul agite ses feuilles, trop vite. Le rond se plie, trop poussé par les feuilles. Le vent prend tout ! Une feuille claque, puis une autre. La bulle part de travers, trop loin. Ici, ça souffle trop. Il lui faut du temps. Alors on fait quoi ? Tu vois comment, Nina ?</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -15186,15 +15186,15 @@
       <c r="AW80" t="inlineStr">
         <is>
           <t>narrateur|Contre son ventre, la coupelle reste bien plate.
-narrateur|Le tilleul sent le miel, trop vif.
+narrateur|Le tilleul agite ses feuilles, trop vite.
 narrateur|Le rond se plie, trop poussé par les feuilles.
 enfant-f|Le vent prend tout !
 narrateur|Une feuille claque, puis une autre.
 narrateur|La bulle part de travers, trop loin.
-papa|Ça souffle trop, ici.
-maman|Elle a besoin de temps.
-enfant-f|On fait comment, alors ?
-papa|Tu trouves, Nina ?</t>
+papa|Ici, ça souffle trop.
+maman|Il lui faut du temps.
+enfant-f|Alors on fait quoi ?
+papa|Tu vois comment, Nina ?</t>
         </is>
       </c>
     </row>
@@ -15221,12 +15221,12 @@
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>Les feuilles claquent encore, trop fort. Attendre les feuilles, derrière, ou tout petit ?</t>
+          <t>Les feuilles n'ont pas fini de claquer. Attendre les feuilles, derrière, ou tout petit ?</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>Les feuilles claquent encore, trop fort. Attendre les feuilles, derrière, ou tout petit ?</t>
+          <t>Les feuilles n'ont pas fini de claquer. Attendre les feuilles, derrière, ou tout petit ?</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -15389,7 +15389,7 @@
       </c>
       <c r="AW81" t="inlineStr">
         <is>
-          <t>narrateur|Les feuilles claquent encore, trop fort.
+          <t>narrateur|Les feuilles n'ont pas fini de claquer.
 papa|Attendre les feuilles, derrière, ou tout petit ?</t>
         </is>
       </c>
@@ -15417,12 +15417,12 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>On attend les feuilles, d'abord. Elle tient la coupelle, puis attend les feuilles. Les feuilles vont, reviennent, puis se taisent. L'air redevient un seul souffle, net. Plate, la coupelle attend, sans verser. Le tilleul n'a plus claqué. Maintenant, tu peux rester. Tu as attendu le calme.</t>
+          <t>On attend les feuilles, d'abord. Elle tient la coupelle, puis attend les feuilles. Les feuilles vont, reviennent, puis se taisent. L'air redevient un seul souffle, net. Plate, la coupelle attend, sans verser. Le tilleul n'a plus claqué. Maintenant, tu peux rester. Tu as laissé les feuilles finir.</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>On attend les feuilles, d'abord. Elle tient la coupelle, puis attend les feuilles. Les feuilles vont, reviennent, puis se taisent. L'air redevient un seul souffle, net. Plate, la coupelle attend, sans verser. Le tilleul n'a plus claqué. Maintenant, tu peux rester. Tu as attendu le calme.</t>
+          <t>On attend les feuilles, d'abord. Elle tient la coupelle, puis attend les feuilles. Les feuilles vont, reviennent, puis se taisent. L'air redevient un seul souffle, net. Plate, la coupelle attend, sans verser. Le tilleul n'a plus claqué. Maintenant, tu peux rester. Tu as laissé les feuilles finir.</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -15564,7 +15564,7 @@
 narrateur|Plate, la coupelle attend, sans verser.
 papa|Le tilleul n'a plus claqué.
 enfant-f|Maintenant, tu peux rester.
-maman|Tu as attendu le calme.</t>
+maman|Tu as laissé les feuilles finir.</t>
         </is>
       </c>
     </row>
@@ -15763,12 +15763,12 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Derrière, pas trop près du vent. Derrière le tronc, la coupelle ne se plie plus. Nina se glisse derrière le tronc, tout bas. Rien ne claque, rien ne pousse plus. Le rond de savon attend, tout calme. Tu n'as pas couru. Tu es ronde, maintenant. Tu as préparé le chemin.</t>
+          <t>Derrière, pas trop près du vent. Derrière le tronc, la coupelle ne se plie plus. Nina se glisse derrière le tronc, tout bas. Rien ne claque, rien ne pousse plus. Le rond de savon attend, tout calme. Tu n'as pas couru. Tu es ronde, maintenant. Derrière, l'air était plus doux.</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>Derrière, pas trop près du vent. Derrière le tronc, la coupelle ne se plie plus. Nina se glisse derrière le tronc, tout bas. Rien ne claque, rien ne pousse plus. Le rond de savon attend, tout calme. Tu n'as pas couru. Tu es ronde, maintenant. Tu as préparé le chemin.</t>
+          <t>Derrière, pas trop près du vent. Derrière le tronc, la coupelle ne se plie plus. Nina se glisse derrière le tronc, tout bas. Rien ne claque, rien ne pousse plus. Le rond de savon attend, tout calme. Tu n'as pas couru. Tu es ronde, maintenant. Derrière, l'air était plus doux.</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -15910,7 +15910,7 @@
 narrateur|Le rond de savon attend, tout calme.
 papa|Tu n'as pas couru.
 enfant-f|Tu es ronde, maintenant.
-maman|Tu as préparé le chemin.</t>
+maman|Derrière, l'air était plus doux.</t>
         </is>
       </c>
     </row>
@@ -16109,12 +16109,12 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Tout petit, tout serré. Une toute petite bulle quitte la coupelle. Nina souffle à peine, sans prendre le vent. Le tilleul se tait, plus loin, tout seul. Plate, la coupelle attend, sans verser. Le petit rond n'a pas volé. Tu restes, bulle. Le petit tenait assez.</t>
+          <t>Tout petit, tout serré. Une toute petite bulle quitte la coupelle. Nina souffle à peine, sans prendre le vent. Le tilleul se tait, plus loin, tout seul. Le rond de savon attend, tout calme. Le petit rond n'a pas volé. Tu restes, bulle. Le petit rond a suffi.</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>Tout petit, tout serré. Une toute petite bulle quitte la coupelle. Nina souffle à peine, sans prendre le vent. Le tilleul se tait, plus loin, tout seul. Plate, la coupelle attend, sans verser. Le petit rond n'a pas volé. Tu restes, bulle. Le petit tenait assez.</t>
+          <t>Tout petit, tout serré. Une toute petite bulle quitte la coupelle. Nina souffle à peine, sans prendre le vent. Le tilleul se tait, plus loin, tout seul. Le rond de savon attend, tout calme. Le petit rond n'a pas volé. Tu restes, bulle. Le petit rond a suffi.</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -16253,10 +16253,10 @@
 narrateur|Une toute petite bulle quitte la coupelle.
 narrateur|Nina souffle à peine, sans prendre le vent.
 narrateur|Le tilleul se tait, plus loin, tout seul.
-narrateur|Plate, la coupelle attend, sans verser.
+narrateur|Le rond de savon attend, tout calme.
 papa|Le petit rond n'a pas volé.
 enfant-f|Tu restes, bulle.
-maman|Le petit tenait assez.</t>
+maman|Le petit rond a suffi.</t>
         </is>
       </c>
     </row>
@@ -16283,12 +16283,12 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Tout petit, le rond tient sur le nez, tout calme. On a soufflé à peine. Le petit rond n'a pas volé. Rentrez, le savon est déjà sec. La coupelle sèche près du gravier, un cercle de savon. Le tilleul se tait, plus loin, tout seul.</t>
+          <t>Tout petit, le rond tient sur le nez, tout calme. On a soufflé à peine. Le petit rond n'a pas volé. Le savon est déjà sec, on rentre. La coupelle sèche près du gravier, un cercle de savon. Le tilleul se tait, plus loin, tout seul.</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>Tout petit, le rond tient sur le nez, tout calme. On a soufflé à peine. Le petit rond n'a pas volé. Rentrez, le savon est déjà sec. La coupelle sèche près du gravier, un cercle de savon. Le tilleul se tait, plus loin, tout seul.</t>
+          <t>Tout petit, le rond tient sur le nez, tout calme. On a soufflé à peine. Le petit rond n'a pas volé. Le savon est déjà sec, on rentre. La coupelle sèche près du gravier, un cercle de savon. Le tilleul se tait, plus loin, tout seul.</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -16426,7 +16426,7 @@
           <t>narrateur|Tout petit, le rond tient sur le nez, tout calme.
 enfant-f|On a soufflé à peine.
 papa|Le petit rond n'a pas volé.
-maman|Rentrez, le savon est déjà sec.
+maman|Le savon est déjà sec, on rentre.
 narrateur|La coupelle sèche près du gravier, un cercle de savon.
 narrateur|Le tilleul se tait, plus loin, tout seul.</t>
         </is>
@@ -16449,7 +16449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -16548,6 +16548,20 @@
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>

<commit_message>
feat(F-NAR-019): TREE-DIF-056 polish La bulle de Nina, sur le nez de bronze
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-DIF-056.xlsx
+++ b/stories/arbres/TREE-DIF-056.xlsx
@@ -1197,17 +1197,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Dans le sac, le bâton cogne la coupelle. Une goutte de savon perle au poignet de Nina. Le parc sent le tilleul chaud, et le gravier. La statue de bronze tient un oiseau, trop petit. Tu as vu son nez, Nina ? Il a une larme de bronze, plus sombre. Elle n'est pas de l'eau. Le gravier chauffe sous ses sandales. En ce moment, Nina serre le sac contre elle. Je veux une bulle, collée sur la larme. La cloche va fermer le parc. On marche d'abord, non ? Non, la bulle, maintenant. Merci, tu as essuyé la goutte.</t>
+          <t>Dans le sac, le bâton cogne la coupelle. Une goutte de savon perle au poignet de Nina. Le parc sent le tilleul chaud, et le gravier. La statue de bronze tient un oiseau, trop petit. Tu as vu son nez, Nina ? Il a une larme de bronze, plus sombre. Elle n'est pas de l'eau. Le gravier chauffe sous ses sandales. Nina passe ici souvent, après l'école. Cette larme, elle ne l'avait pas vue. En ce moment, Nina serre le sac contre elle. Je veux une bulle, collée sur la larme. La cloche va fermer le parc. On marche d'abord, non ? Non, la bulle, maintenant. Merci, tu as essuyé la goutte. Le sac pend, trop plein pour courir.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Dans le sac, le bâton cogne la coupelle. Une goutte de savon perle au poignet de Nina. Le parc sent le tilleul chaud, et le gravier. La statue de bronze tient un oiseau, trop petit. Tu as vu son nez, Nina ? Il a une &lt;emphasis level="moderate"&gt;larme de bronze&lt;/emphasis&gt;, plus sombre. Elle n'est pas de l'eau. Le gravier chauffe sous ses sandales. En ce moment, Nina serre le sac contre elle. Je veux une bulle, collée sur la larme. La cloche va fermer le parc. On marche d'abord, non ? Non, la bulle, maintenant. Merci, tu as essuyé la goutte.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Dans le sac, le bâton cogne la coupelle. Une goutte de savon perle au poignet de Nina. Le parc sent le tilleul chaud, et le gravier. La statue de bronze tient un oiseau, trop petit. Tu as vu son nez, Nina ? Il a une &lt;emphasis level="moderate"&gt;larme de bronze&lt;/emphasis&gt;, plus sombre. Elle n'est pas de l'eau. Le gravier chauffe sous ses sandales. Nina passe ici souvent, après l'école. Cette larme, elle ne l'avait pas vue. En ce moment, Nina serre le sac contre elle. Je veux une bulle, collée sur la larme. La cloche va fermer le parc. On marche d'abord, non ? Non, la bulle, maintenant. Merci, tu as essuyé la goutte. Le sac pend, trop plein pour courir.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Dans le sac, le bâton cogne la coupelle. Une goutte de savon perle au poignet de Nina. Le parc sent le tilleul chaud, et le gravier. La statue de bronze tient un oiseau, trop petit. Tu as vu son nez, Nina ? Il a une &lt;emphasis&gt;larme de bronze&lt;/emphasis&gt;, plus sombre. Elle n'est pas de l'eau. Le gravier chauffe sous ses sandales. En ce moment, Nina serre le sac contre elle. Je veux une bulle, collée sur la larme. La cloche va fermer le parc. On marche d'abord, non ? Non, la bulle, maintenant. Merci, tu as essuyé la goutte. [pause]</t>
+          <t>Dans le sac, le bâton cogne la coupelle. Une goutte de savon perle au poignet de Nina. Le parc sent le tilleul chaud, et le gravier. La statue de bronze tient un oiseau, trop petit. Tu as vu son nez, Nina ? Il a une &lt;emphasis&gt;larme de bronze&lt;/emphasis&gt;, plus sombre. Elle n'est pas de l'eau. Le gravier chauffe sous ses sandales. Nina passe ici souvent, après l'école. Cette larme, elle ne l'avait pas vue. En ce moment, Nina serre le sac contre elle. Je veux une bulle, collée sur la larme. La cloche va fermer le parc. On marche d'abord, non ? Non, la bulle, maintenant. Merci, tu as essuyé la goutte. Le sac pend, trop plein pour courir. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1349,12 +1349,15 @@
 enfant-f|Il a une larme de bronze, plus sombre.
 maman|Elle n'est pas de l'eau.
 narrateur|Le gravier chauffe sous ses sandales.
+narrateur|Nina passe ici souvent, après l'école.
+narrateur|Cette larme, elle ne l'avait pas vue.
 narrateur|En ce moment, Nina serre le sac contre elle.
 enfant-f|Je veux une bulle, collée sur la larme.
 papa|La cloche va fermer le parc.
 maman|On marche d'abord, non ?
 enfant-f|Non, la bulle, maintenant.
-papa|Merci, tu as essuyé la goutte.</t>
+papa|Merci, tu as essuyé la goutte.
+narrateur|Le sac pend, trop plein pour courir.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1583,17 +1586,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Nina attrape d'abord le bâton, un peu humide. La bulle va s'y accrocher. Garde le cercle en l'air. Un film tremble au bout, puis tient. Elle lève le bois, trop vite. Pas si fort, le fil va casser. Nina baisse le cercle, les joues chaudes. Prends le savon, il est à tes pieds. La coupelle glisse sous son autre bras. Les trois partent, collés à Nina. Nez, j'arrive. Le bois sent le savon, un peu. Le bâton est à toi, là.</t>
+          <t>Nina attrape d'abord le bâton, un peu humide. La bulle va s'y accrocher. Garde le cercle en l'air. Un film tremble au bout, puis tient. Elle lève le bois, trop vite. Pas si fort, le fil va casser. Nina baisse le cercle, les joues chaudes. Prends le savon, il est à tes pieds. La coupelle glisse sous son autre bras. Les trois partent, collés à Nina. Nez, j'arrive. Le bois sent le savon, un peu. Le bâton est à toi, là. Elle veut souffler tout de suite, trop. Le bronze est loin, d'abord.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nina attrape d'abord le &lt;emphasis level="moderate"&gt;bâton&lt;/emphasis&gt;, un peu humide. La bulle va s'y accrocher. Garde le cercle en l'air. Un film tremble au bout, puis tient. Elle lève le bois, trop vite. Pas si fort, le fil va casser. Nina baisse le cercle, les joues chaudes. Prends le savon, il est à tes pieds. La coupelle glisse sous son autre bras. Les trois partent, collés à Nina. Nez, j'arrive. Le bois sent le savon, un peu. Le bâton est à toi, là.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nina attrape d'abord le &lt;emphasis level="moderate"&gt;bâton&lt;/emphasis&gt;, un peu humide. La bulle va s'y accrocher. Garde le cercle en l'air. Un film tremble au bout, puis tient. Elle lève le bois, trop vite. Pas si fort, le fil va casser. Nina baisse le cercle, les joues chaudes. Prends le savon, il est à tes pieds. La coupelle glisse sous son autre bras. Les trois partent, collés à Nina. Nez, j'arrive. Le bois sent le savon, un peu. Le bâton est à toi, là. Elle veut souffler tout de suite, trop. Le bronze est loin, d'abord.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Nina attrape d'abord le &lt;emphasis&gt;bâton&lt;/emphasis&gt;, un peu humide. La bulle va s'y accrocher. Garde le cercle en l'air. Un film tremble au bout, puis tient. Elle lève le bois, trop vite. Pas si fort, le fil va casser. Nina baisse le cercle, les joues chaudes. Prends le savon, il est à tes pieds. La coupelle glisse sous son autre bras. Les trois partent, collés à Nina. Nez, j'arrive. Le bois sent le savon, un peu. Le bâton est à toi, là. [pause]</t>
+          <t>Nina attrape d'abord le &lt;emphasis&gt;bâton&lt;/emphasis&gt;, un peu humide. La bulle va s'y accrocher. Garde le cercle en l'air. Un film tremble au bout, puis tient. Elle lève le bois, trop vite. Pas si fort, le fil va casser. Nina baisse le cercle, les joues chaudes. Prends le savon, il est à tes pieds. La coupelle glisse sous son autre bras. Les trois partent, collés à Nina. Nez, j'arrive. Le bois sent le savon, un peu. Le bâton est à toi, là. Elle veut souffler tout de suite, trop. Le bronze est loin, d'abord. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1739,7 +1742,9 @@
 narrateur|Les trois partent, collés à Nina.
 enfant-f|Nez, j'arrive.
 narrateur|Le bois sent le savon, un peu.
-papa|Le bâton est à toi, là.</t>
+papa|Le bâton est à toi, là.
+narrateur|Elle veut souffler tout de suite, trop.
+maman|Le bronze est loin, d'abord.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
@@ -1959,17 +1964,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le bâton reste contre elle, un peu humide. On va jusqu'au bronze. La cloche n'est pas loin. Tu tiens bien, Nina ? Oui, papa. Un fil de savon cherche l'air. On avance, sans courir.</t>
+          <t>Le bâton reste contre elle, un peu humide. On va jusqu'au bronze. La cloche n'est pas loin. Tu tiens bien, Nina ? Oui, papa. Un fil de savon cherche l'air. On avance, sans courir. Le cercle penche, puis se redresse. Le savon et la coupelle sont avec toi.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;bâton&lt;/emphasis&gt; reste contre elle, un peu humide. On va jusqu'au bronze. La cloche n'est pas loin. Tu tiens bien, Nina ? Oui, papa. Un fil de savon cherche l'air. On avance, sans courir.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;bâton&lt;/emphasis&gt; reste contre elle, un peu humide. On va jusqu'au bronze. La cloche n'est pas loin. Tu tiens bien, Nina ? Oui, papa. Un fil de savon cherche l'air. On avance, sans courir. Le cercle penche, puis se redresse. Le savon et la coupelle sont avec toi.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Le &lt;emphasis&gt;bâton&lt;/emphasis&gt; reste contre elle, un peu humide. On va jusqu'au bronze. La cloche n'est pas loin. Tu tiens bien, Nina ? Oui, papa. Un fil de savon cherche l'air. On avance, sans courir. [pause]</t>
+          <t>Le &lt;emphasis&gt;bâton&lt;/emphasis&gt; reste contre elle, un peu humide. On va jusqu'au bronze. La cloche n'est pas loin. Tu tiens bien, Nina ? Oui, papa. Un fil de savon cherche l'air. On avance, sans courir. Le cercle penche, puis se redresse. Le savon et la coupelle sont avec toi. [pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2109,7 +2114,9 @@
 papa|Tu tiens bien, Nina ?
 enfant-f|Oui, papa.
 narrateur|Un fil de savon cherche l'air.
-papa|On avance, sans courir.</t>
+papa|On avance, sans courir.
+narrateur|Le cercle penche, puis se redresse.
+maman|Le savon et la coupelle sont avec toi.</t>
         </is>
       </c>
       <c r="AX6" t="inlineStr">
@@ -2141,17 +2148,17 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Le bâton penche vers le bronze. Devant, l'allée soulève trop de poussière. Le socle, lui, brûle au soleil. Sous le tilleul, les feuilles claquent. Nina, tu vas où ?</t>
+          <t>Le bâton penche vers le bronze. Devant, l'allée soulève trop de poussière. Le socle, lui, brûle au soleil. Sous le tilleul, les feuilles claquent. Nina, tu vas où ? La larme attend, sur le nez.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Le bâton penche vers le bronze. Devant, l'allée soulève trop de poussière. Le socle, lui, brûle au soleil. Sous le tilleul, les feuilles claquent. Nina, tu vas où ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Le bâton penche vers le bronze. Devant, l'allée soulève trop de poussière. Le socle, lui, brûle au soleil. Sous le tilleul, les feuilles claquent. Nina, tu vas où ? La larme attend, sur le nez.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Le bâton penche vers le bronze. Devant, l'allée soulève trop de poussière. Le socle, lui, brûle au soleil. Sous le tilleul, les feuilles claquent. Nina, tu vas où ?&lt;/slow&gt; [long-pause]</t>
+          <t>&lt;slow&gt;Le bâton penche vers le bronze. Devant, l'allée soulève trop de poussière. Le socle, lui, brûle au soleil. Sous le tilleul, les feuilles claquent. Nina, tu vas où ? La larme attend, sur le nez.&lt;/slow&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr"/>
@@ -2313,7 +2320,8 @@
 narrateur|Devant, l'allée soulève trop de poussière.
 narrateur|Le socle, lui, brûle au soleil.
 narrateur|Sous le tilleul, les feuilles claquent.
-papa|Nina, tu vas où ?</t>
+papa|Nina, tu vas où ?
+maman|La larme attend, sur le nez.</t>
         </is>
       </c>
     </row>
@@ -2340,17 +2348,17 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Entre ses doigts, le bois du bâton est tiède. Le gravier de l'allée saute sous les pas. Un fil se casse, trop vite, trop fort. Ma bulle a crevé ! Le sourire de Nina disparaît. Dans sa poitrine, l'envie et la peur se bousculent. Ici, ça n'arrête pas. Papa s'accroupit, à la même hauteur. Elle lève le bâton, trop vite. Un pas tardif soulève la poussière, gris. Pas maintenant. La larme de bronze est grise, trop. Tu vois comment, Nina ?</t>
+          <t>Entre ses doigts, le bois du bâton est tiède. Le gravier de l'allée saute sous les pas. Un fil se casse, trop vite, trop fort. Ma bulle a crevé ! Le sourire de Nina disparaît. Dans sa poitrine, l'envie et la peur se bousculent. Ici, ça n'arrête pas. Papa s'accroupit, à la même hauteur. Elle lève le bâton, trop vite. Un pas tardif soulève la poussière, gris. Pas maintenant. La larme de bronze est grise, trop. Tu vois comment, Nina ? Nina serre le bâton, sans souffler. Alors on fait quoi ?</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Entre ses doigts, le bois du bâton est tiède. Le gravier de l'&lt;emphasis level="moderate"&gt;allée&lt;/emphasis&gt; saute sous les pas. Un fil se casse, trop vite, trop fort. Ma bulle a crevé ! Le sourire de Nina disparaît. Dans sa poitrine, l'envie et la peur se bousculent. Ici, ça n'arrête pas. Papa s'accroupit, à la même hauteur. Elle lève le bâton, trop vite. Un pas tardif soulève la poussière, gris. Pas maintenant. La larme de bronze est grise, trop. Tu vois comment, Nina ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Entre ses doigts, le bois du bâton est tiède. Le gravier de l'&lt;emphasis level="moderate"&gt;allée&lt;/emphasis&gt; saute sous les pas. Un fil se casse, trop vite, trop fort. Ma bulle a crevé ! Le sourire de Nina disparaît. Dans sa poitrine, l'envie et la peur se bousculent. Ici, ça n'arrête pas. Papa s'accroupit, à la même hauteur. Elle lève le bâton, trop vite. Un pas tardif soulève la poussière, gris. Pas maintenant. La larme de bronze est grise, trop. Tu vois comment, Nina ? Nina serre le bâton, sans souffler. Alors on fait quoi ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Entre ses doigts, le bois du bâton est tiède. Le gravier de l'&lt;emphasis&gt;allée&lt;/emphasis&gt; saute sous les pas. Un fil se casse, trop vite, trop fort. Ma bulle a crevé ! Le sourire de Nina disparaît. Dans sa poitrine, l'envie et la peur se bousculent. Ici, ça n'arrête pas. Papa s'accroupit, à la même hauteur. Elle lève le bâton, trop vite. Un pas tardif soulève la poussière, gris. Pas maintenant. La larme de bronze est grise, trop. Tu vois comment, Nina ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Entre ses doigts, le bois du bâton est tiède. Le gravier de l'&lt;emphasis&gt;allée&lt;/emphasis&gt; saute sous les pas. Un fil se casse, trop vite, trop fort. Ma bulle a crevé ! Le sourire de Nina disparaît. Dans sa poitrine, l'envie et la peur se bousculent. Ici, ça n'arrête pas. Papa s'accroupit, à la même hauteur. Elle lève le bâton, trop vite. Un pas tardif soulève la poussière, gris. Pas maintenant. La larme de bronze est grise, trop. Tu vois comment, Nina ? Nina serre le bâton, sans souffler. Alors on fait quoi ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr"/>
@@ -2500,7 +2508,9 @@
 narrateur|Un pas tardif soulève la poussière, gris.
 enfant-f|Pas maintenant.
 narrateur|La larme de bronze est grise, trop.
-maman|Tu vois comment, Nina ?</t>
+maman|Tu vois comment, Nina ?
+narrateur|Nina serre le bâton, sans souffler.
+enfant-f|Alors on fait quoi ?</t>
         </is>
       </c>
       <c r="AX8" t="inlineStr">
@@ -2728,17 +2738,17 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>On attend les pas. Nina tient le bâton, sans souffler. Le gravier se tait, une fois, puis plus. La larme de bronze redevient sombre, nette. Tu peux partir, maintenant. Pendant ce temps, le bâton reste droit. Les pas se sont tus, là. La bulle part, ronde, vers la larme. Tu as laissé le gravier se taire.</t>
+          <t>On attend les pas. Nina tient le bâton, sans souffler. Le gravier se tait, une fois, puis plus. La larme de bronze redevient sombre, nette. Tu peux partir, maintenant. Pendant ce temps, le bâton reste droit. Les pas se sont tus, là. La bulle part, ronde, vers la larme. Elle compte les pas, un, deux, trois. Je ne fonce pas. Tu as laissé le gravier se taire.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend les &lt;emphasis level="moderate"&gt;pas&lt;/emphasis&gt;. Nina tient le bâton, sans souffler. Le gravier se tait, une fois, puis plus. La larme de bronze redevient sombre, nette. Tu peux partir, maintenant. Pendant ce temps, le bâton reste droit. Les pas se sont tus, là. La bulle part, ronde, vers la larme. Tu as laissé le gravier se taire.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend les &lt;emphasis level="moderate"&gt;pas&lt;/emphasis&gt;. Nina tient le bâton, sans souffler. Le gravier se tait, une fois, puis plus. La larme de bronze redevient sombre, nette. Tu peux partir, maintenant. Pendant ce temps, le bâton reste droit. Les pas se sont tus, là. La bulle part, ronde, vers la larme. Elle compte les pas, un, deux, trois. Je ne fonce pas. Tu as laissé le gravier se taire.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>On attend les &lt;emphasis&gt;pas&lt;/emphasis&gt;. Nina tient le bâton, sans souffler. Le gravier se tait, une fois, puis plus. La larme de bronze redevient sombre, nette. Tu peux partir, maintenant. Pendant ce temps, le bâton reste droit. Les pas se sont tus, là. La bulle part, ronde, vers la larme. Tu as laissé le gravier se taire. [pause]</t>
+          <t>On attend les &lt;emphasis&gt;pas&lt;/emphasis&gt;. Nina tient le bâton, sans souffler. Le gravier se tait, une fois, puis plus. La larme de bronze redevient sombre, nette. Tu peux partir, maintenant. Pendant ce temps, le bâton reste droit. Les pas se sont tus, là. La bulle part, ronde, vers la larme. Elle compte les pas, un, deux, trois. Je ne fonce pas. Tu as laissé le gravier se taire. [pause]</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr"/>
@@ -2880,6 +2890,8 @@
 narrateur|Pendant ce temps, le bâton reste droit.
 papa|Les pas se sont tus, là.
 narrateur|La bulle part, ronde, vers la larme.
+narrateur|Elle compte les pas, un, deux, trois.
+enfant-f|Je ne fonce pas.
 maman|Tu as laissé le gravier se taire.</t>
         </is>
       </c>
@@ -3097,17 +3109,17 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Plus bas, d'abord. Elle baisse le bâton, loin de la poussière. Nina s'accroupit, les genoux au gravier. L'air est plus doux, près de l'herbe. La larme de bronze se voit d'en bas. Ici, tu ne crèves plus. Tu as vu l'herbe, avant. Un fil de savon cherche l'air, bas. Près du sol, ça tenait mieux.</t>
+          <t>Plus bas, d'abord. Elle baisse le bâton, loin de la poussière. Nina s'accroupit, les genoux au gravier. L'air est plus doux, près de l'herbe. La larme de bronze se voit d'en bas. Ici, tu ne crèves plus. Tu as vu l'herbe, avant. Un fil de savon cherche l'air, bas. Elle pose le cercle près de l'herbe. Je souffle d'en bas, vers la larme. Près du sol, ça tenait mieux.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Plus bas, d'abord. Elle baisse le bâton, loin de la poussière. Nina s'accroupit, les genoux au gravier. L'air est plus doux, près de l'herbe. La larme de bronze se voit d'en bas. Ici, tu ne crèves plus. Tu as vu l'herbe, avant. Un fil de savon cherche l'air, bas. Près du sol, ça tenait mieux.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Plus bas, d'abord. Elle baisse le bâton, loin de la poussière. Nina s'accroupit, les genoux au gravier. L'air est plus doux, près de l'herbe. La larme de bronze se voit d'en bas. Ici, tu ne crèves plus. Tu as vu l'herbe, avant. Un fil de savon cherche l'air, bas. Elle pose le cercle près de l'herbe. Je souffle d'en bas, vers la larme. Près du sol, ça tenait mieux.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Plus bas, d'abord. Elle baisse le bâton, loin de la poussière. Nina s'accroupit, les genoux au gravier. L'air est plus doux, près de l'herbe. La larme de bronze se voit d'en bas. Ici, tu ne crèves plus. Tu as vu l'herbe, avant. Un fil de savon cherche l'air, bas. Près du sol, ça tenait mieux. [pause]</t>
+          <t>Plus bas, d'abord. Elle baisse le bâton, loin de la poussière. Nina s'accroupit, les genoux au gravier. L'air est plus doux, près de l'herbe. La larme de bronze se voit d'en bas. Ici, tu ne crèves plus. Tu as vu l'herbe, avant. Un fil de savon cherche l'air, bas. Elle pose le cercle près de l'herbe. Je souffle d'en bas, vers la larme. Près du sol, ça tenait mieux. [pause]</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr"/>
@@ -3249,6 +3261,8 @@
 enfant-f|Ici, tu ne crèves plus.
 papa|Tu as vu l'herbe, avant.
 narrateur|Un fil de savon cherche l'air, bas.
+narrateur|Elle pose le cercle près de l'herbe.
+enfant-f|Je souffle d'en bas, vers la larme.
 maman|Près du sol, ça tenait mieux.</t>
         </is>
       </c>
@@ -3466,17 +3480,17 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Au bord, tout petit. Elle glisse le bâton vers le bord d'herbe. L'herbe tient, sans laisser la poussière. Nina souffle bas, une seule fois. La larme de bronze luit, hors de l'allée. Le bord n'a pas soulevé. Tu es à l'abri. Le rond monte, lent, jusqu'au nez. Tu as dit ça tout bas.</t>
+          <t>Au bord, tout petit. Elle glisse le bâton vers le bord d'herbe. L'herbe tient, sans laisser la poussière. Nina souffle bas, une seule fois. La larme de bronze luit, hors de l'allée. Le bord n'a pas soulevé. Tu es à l'abri. Le rond monte, lent, jusqu'au nez. Elle plante les pieds dans l'herbe. Le bord tient, pas l'allée. Tu as dit ça tout bas.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Au &lt;emphasis level="moderate"&gt;bord&lt;/emphasis&gt;, tout petit. Elle glisse le bâton vers le bord d'herbe. L'herbe tient, sans laisser la poussière. Nina souffle bas, une seule fois. La larme de bronze luit, hors de l'allée. Le bord n'a pas soulevé. Tu es à l'abri. Le rond monte, lent, jusqu'au nez. Tu as dit ça tout bas.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Au &lt;emphasis level="moderate"&gt;bord&lt;/emphasis&gt;, tout petit. Elle glisse le bâton vers le bord d'herbe. L'herbe tient, sans laisser la poussière. Nina souffle bas, une seule fois. La larme de bronze luit, hors de l'allée. Le bord n'a pas soulevé. Tu es à l'abri. Le rond monte, lent, jusqu'au nez. Elle plante les pieds dans l'herbe. Le bord tient, pas l'allée. Tu as dit ça tout bas.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Au &lt;emphasis&gt;bord&lt;/emphasis&gt;, tout petit. Elle glisse le bâton vers le bord d'herbe. L'herbe tient, sans laisser la poussière. Nina souffle bas, une seule fois. La larme de bronze luit, hors de l'allée. Le bord n'a pas soulevé. Tu es à l'abri. Le rond monte, lent, jusqu'au nez. Tu as dit ça tout bas. [pause]</t>
+          <t>Au &lt;emphasis&gt;bord&lt;/emphasis&gt;, tout petit. Elle glisse le bâton vers le bord d'herbe. L'herbe tient, sans laisser la poussière. Nina souffle bas, une seule fois. La larme de bronze luit, hors de l'allée. Le bord n'a pas soulevé. Tu es à l'abri. Le rond monte, lent, jusqu'au nez. Elle plante les pieds dans l'herbe. Le bord tient, pas l'allée. Tu as dit ça tout bas. [pause]</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr"/>
@@ -3618,6 +3632,8 @@
 papa|Le bord n'a pas soulevé.
 enfant-f|Tu es à l'abri.
 narrateur|Le rond monte, lent, jusqu'au nez.
+narrateur|Elle plante les pieds dans l'herbe.
+enfant-f|Le bord tient, pas l'allée.
 maman|Tu as dit ça tout bas.</t>
         </is>
       </c>
@@ -3835,17 +3851,17 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Entre ses doigts, le bois du bâton est tiède. Le bronze tient tout le soleil. Le fil fond, trop chaud, trop mince. Le nez brûle trop ! La bulle touche, puis crève tout de suite. Il ne reste rien sur le bronze. Ici, c'est trop chaud. Papa s'accroupit, à la même hauteur. Un nuage passe, et Nina lève le bois. Le soleil revient, net, sur la larme. Pas maintenant. La larme de bronze est sèche, trop pâle. Tu vois comment, Nina ?</t>
+          <t>Entre ses doigts, le bois du bâton est tiède. Le bronze tient tout le soleil. Le fil fond, trop chaud, trop mince. Le nez brûle trop ! La bulle touche, puis crève tout de suite. Il ne reste rien sur le bronze. Ici, c'est trop chaud. Papa s'accroupit, à la même hauteur. Un nuage passe, et Nina lève le bois. Le soleil revient, net, sur la larme. Pas maintenant. La larme de bronze est sèche, trop pâle. Tu vois comment, Nina ? Nina serre le bâton, sans souffler. Alors on fait quoi ?</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Entre ses doigts, le bois du bâton est tiède. Le bronze tient tout le soleil. Le fil fond, trop chaud, trop mince. Le nez brûle trop ! La bulle touche, puis crève tout de suite. Il ne reste rien sur le bronze. Ici, c'est trop chaud. Papa s'accroupit, à la même hauteur. Un nuage passe, et Nina lève le bois. Le soleil revient, net, sur la larme. Pas maintenant. La larme de bronze est sèche, trop pâle. Tu vois comment, Nina ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Entre ses doigts, le bois du bâton est tiède. Le bronze tient tout le soleil. Le fil fond, trop chaud, trop mince. Le nez brûle trop ! La bulle touche, puis crève tout de suite. Il ne reste rien sur le bronze. Ici, c'est trop chaud. Papa s'accroupit, à la même hauteur. Un nuage passe, et Nina lève le bois. Le soleil revient, net, sur la larme. Pas maintenant. La larme de bronze est sèche, trop pâle. Tu vois comment, Nina ? Nina serre le bâton, sans souffler. Alors on fait quoi ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Entre ses doigts, le bois du bâton est tiède. Le bronze tient tout le soleil. Le fil fond, trop chaud, trop mince. Le nez brûle trop ! La bulle touche, puis crève tout de suite. Il ne reste rien sur le bronze. Ici, c'est trop chaud. Papa s'accroupit, à la même hauteur. Un nuage passe, et Nina lève le bois. Le soleil revient, net, sur la larme. Pas maintenant. La larme de bronze est sèche, trop pâle. Tu vois comment, Nina ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Entre ses doigts, le bois du bâton est tiède. Le bronze tient tout le soleil. Le fil fond, trop chaud, trop mince. Le nez brûle trop ! La bulle touche, puis crève tout de suite. Il ne reste rien sur le bronze. Ici, c'est trop chaud. Papa s'accroupit, à la même hauteur. Un nuage passe, et Nina lève le bois. Le soleil revient, net, sur la larme. Pas maintenant. La larme de bronze est sèche, trop pâle. Tu vois comment, Nina ? Nina serre le bâton, sans souffler. Alors on fait quoi ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr"/>
@@ -3995,7 +4011,9 @@
 narrateur|Le soleil revient, net, sur la larme.
 enfant-f|Pas maintenant.
 narrateur|La larme de bronze est sèche, trop pâle.
-maman|Tu vois comment, Nina ?</t>
+maman|Tu vois comment, Nina ?
+narrateur|Nina serre le bâton, sans souffler.
+enfant-f|Alors on fait quoi ?</t>
         </is>
       </c>
       <c r="AX16" t="inlineStr">
@@ -4223,17 +4241,17 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>On attend l'ombre. Une ombre de tilleul glisse sur le nez. Sous l'ombre, le bâton ne fond plus. Le bronze se tait, puis se refroidit. La larme de bronze redevient sombre, froide. Le nez est redevenu doux. Maintenant, tu me vois. Pendant ce temps, le bâton reste droit. Tu as laissé l'ombre arriver.</t>
+          <t>On attend l'ombre. Une ombre de tilleul glisse sur le nez. Sous l'ombre, le bâton ne fond plus. Le bronze se tait, puis se refroidit. La larme de bronze redevient sombre, froide. Le nez est redevenu doux. Maintenant, tu me vois. Pendant ce temps, le bâton reste droit. Elle suit l'ombre, sans bouger le bois. Quand la larme est froide, je souffle. Tu as laissé l'ombre arriver.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend l'&lt;emphasis level="moderate"&gt;ombre&lt;/emphasis&gt;. Une ombre de tilleul glisse sur le nez. Sous l'ombre, le bâton ne fond plus. Le bronze se tait, puis se refroidit. La larme de bronze redevient sombre, froide. Le nez est redevenu doux. Maintenant, tu me vois. Pendant ce temps, le bâton reste droit. Tu as laissé l'ombre arriver.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend l'&lt;emphasis level="moderate"&gt;ombre&lt;/emphasis&gt;. Une ombre de tilleul glisse sur le nez. Sous l'ombre, le bâton ne fond plus. Le bronze se tait, puis se refroidit. La larme de bronze redevient sombre, froide. Le nez est redevenu doux. Maintenant, tu me vois. Pendant ce temps, le bâton reste droit. Elle suit l'ombre, sans bouger le bois. Quand la larme est froide, je souffle. Tu as laissé l'ombre arriver.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>On attend l'&lt;emphasis&gt;ombre&lt;/emphasis&gt;. Une ombre de tilleul glisse sur le nez. Sous l'ombre, le bâton ne fond plus. Le bronze se tait, puis se refroidit. La larme de bronze redevient sombre, froide. Le nez est redevenu doux. Maintenant, tu me vois. Pendant ce temps, le bâton reste droit. Tu as laissé l'ombre arriver. [pause]</t>
+          <t>On attend l'&lt;emphasis&gt;ombre&lt;/emphasis&gt;. Une ombre de tilleul glisse sur le nez. Sous l'ombre, le bâton ne fond plus. Le bronze se tait, puis se refroidit. La larme de bronze redevient sombre, froide. Le nez est redevenu doux. Maintenant, tu me vois. Pendant ce temps, le bâton reste droit. Elle suit l'ombre, sans bouger le bois. Quand la larme est froide, je souffle. Tu as laissé l'ombre arriver. [pause]</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr"/>
@@ -4375,6 +4393,8 @@
 maman|Le nez est redevenu doux.
 enfant-f|Maintenant, tu me vois.
 narrateur|Pendant ce temps, le bâton reste droit.
+narrateur|Elle suit l'ombre, sans bouger le bois.
+enfant-f|Quand la larme est froide, je souffle.
 papa|Tu as laissé l'ombre arriver.</t>
         </is>
       </c>
@@ -4592,17 +4612,17 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>L'oiseau, d'abord, il est plus frais. Elle pose d'abord le fil sur l'oiseau. L'oiseau de bronze est à l'ombre, lui. Le rond glisse, lent, vers la larme. Un fil de savon cherche l'air, court. Tu n'as pas soufflé trop fort. C'est pour toi. La larme de bronze reçoit le rond, entier. L'oiseau était plus frais, tu as vu.</t>
+          <t>L'oiseau, d'abord, il est plus frais. Elle pose d'abord le fil sur l'oiseau. L'oiseau de bronze est à l'ombre, lui. Le rond glisse, lent, vers la larme. Un fil de savon cherche l'air, court. Tu n'as pas soufflé trop fort. C'est pour toi. La larme de bronze reçoit le rond, entier. Elle trempe le cercle sur le bec. L'oiseau d'abord, la larme après. L'oiseau était plus frais, tu as vu.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;L'&lt;emphasis level="moderate"&gt;oiseau&lt;/emphasis&gt;, d'abord, il est plus frais. Elle pose d'abord le fil sur l'oiseau. L'oiseau de bronze est à l'ombre, lui. Le rond glisse, lent, vers la larme. Un fil de savon cherche l'air, court. Tu n'as pas soufflé trop fort. C'est pour toi. La larme de bronze reçoit le rond, entier. L'oiseau était plus frais, tu as vu.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;L'&lt;emphasis level="moderate"&gt;oiseau&lt;/emphasis&gt;, d'abord, il est plus frais. Elle pose d'abord le fil sur l'oiseau. L'oiseau de bronze est à l'ombre, lui. Le rond glisse, lent, vers la larme. Un fil de savon cherche l'air, court. Tu n'as pas soufflé trop fort. C'est pour toi. La larme de bronze reçoit le rond, entier. Elle trempe le cercle sur le bec. L'oiseau d'abord, la larme après. L'oiseau était plus frais, tu as vu.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>L'&lt;emphasis&gt;oiseau&lt;/emphasis&gt;, d'abord, il est plus frais. Elle pose d'abord le fil sur l'oiseau. L'oiseau de bronze est à l'ombre, lui. Le rond glisse, lent, vers la larme. Un fil de savon cherche l'air, court. Tu n'as pas soufflé trop fort. C'est pour toi. La larme de bronze reçoit le rond, entier. L'oiseau était plus frais, tu as vu. [pause]</t>
+          <t>L'&lt;emphasis&gt;oiseau&lt;/emphasis&gt;, d'abord, il est plus frais. Elle pose d'abord le fil sur l'oiseau. L'oiseau de bronze est à l'ombre, lui. Le rond glisse, lent, vers la larme. Un fil de savon cherche l'air, court. Tu n'as pas soufflé trop fort. C'est pour toi. La larme de bronze reçoit le rond, entier. Elle trempe le cercle sur le bec. L'oiseau d'abord, la larme après. L'oiseau était plus frais, tu as vu. [pause]</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr"/>
@@ -4744,6 +4764,8 @@
 papa|Tu n'as pas soufflé trop fort.
 enfant-f|C'est pour toi.
 narrateur|La larme de bronze reçoit le rond, entier.
+narrateur|Elle trempe le cercle sur le bec.
+enfant-f|L'oiseau d'abord, la larme après.
 maman|L'oiseau était plus frais, tu as vu.</t>
         </is>
       </c>
@@ -4961,17 +4983,17 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Tout près, contre le bronze. Nina se glisse contre le socle. Tout près, le bâton n'a plus d'air chaud. La bulle n'a plus à voyager trop loin. La larme de bronze est là, à un souffle. Tu t'es mise tout près, contre le nez. Le nez est là. Pendant ce temps, le bâton reste droit. Tu t'es mise tout contre.</t>
+          <t>Tout près, contre le bronze. Nina se glisse contre le socle. Tout près, le bâton n'a plus d'air chaud. La bulle n'a plus à voyager trop loin. La larme de bronze est là, à un souffle. Tu t'es mise tout près, contre le nez. Le nez est là. Pendant ce temps, le bâton reste droit. Elle avance le cercle, tout contre le nez. Un tout petit souffle, ici. Tu t'es mise tout contre.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Tout près, contre le bronze. Nina se glisse contre le socle. Tout près, le bâton n'a plus d'air chaud. La bulle n'a plus à voyager trop loin. La larme de bronze est là, à un souffle. Tu t'es mise &lt;emphasis level="moderate"&gt;tout près&lt;/emphasis&gt;, contre le nez. Le nez est là. Pendant ce temps, le bâton reste droit. Tu t'es mise tout contre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Tout près, contre le bronze. Nina se glisse contre le socle. Tout près, le bâton n'a plus d'air chaud. La bulle n'a plus à voyager trop loin. La larme de bronze est là, à un souffle. Tu t'es mise &lt;emphasis level="moderate"&gt;tout près&lt;/emphasis&gt;, contre le nez. Le nez est là. Pendant ce temps, le bâton reste droit. Elle avance le cercle, tout contre le nez. Un tout petit souffle, ici. Tu t'es mise tout contre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Tout près, contre le bronze. Nina se glisse contre le socle. Tout près, le bâton n'a plus d'air chaud. La bulle n'a plus à voyager trop loin. La larme de bronze est là, à un souffle. Tu t'es mise &lt;emphasis&gt;tout près&lt;/emphasis&gt;, contre le nez. Le nez est là. Pendant ce temps, le bâton reste droit. Tu t'es mise tout contre. [pause]</t>
+          <t>Tout près, contre le bronze. Nina se glisse contre le socle. Tout près, le bâton n'a plus d'air chaud. La bulle n'a plus à voyager trop loin. La larme de bronze est là, à un souffle. Tu t'es mise &lt;emphasis&gt;tout près&lt;/emphasis&gt;, contre le nez. Le nez est là. Pendant ce temps, le bâton reste droit. Elle avance le cercle, tout contre le nez. Un tout petit souffle, ici. Tu t'es mise tout contre. [pause]</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr"/>
@@ -5113,6 +5135,8 @@
 papa|Tu t'es mise tout près, contre le nez.
 enfant-f|Le nez est là.
 narrateur|Pendant ce temps, le bâton reste droit.
+narrateur|Elle avance le cercle, tout contre le nez.
+enfant-f|Un tout petit souffle, ici.
 maman|Tu t'es mise tout contre.</t>
         </is>
       </c>
@@ -5330,17 +5354,17 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Entre ses doigts, le bois du bâton est tiède. Le tilleul agite ses feuilles, trop vite. Le fil claque, trop léger dans l'air. Le vent prend tout ! Une feuille claque, puis une autre. La bulle part de travers, trop loin. Ici, ça souffle trop. Papa s'accroupit, à la même hauteur. Les feuilles se taisent, un instant. Nina lève le bâton, trop tôt. Un souffle tardif plie le fil. Pas maintenant. La larme de bronze reste nette, elle. Tu vois comment, Nina ?</t>
+          <t>Entre ses doigts, le bois du bâton est tiède. Le tilleul agite ses feuilles, trop vite. Le fil claque, trop léger dans l'air. Le vent prend tout ! Une feuille claque, puis une autre. La bulle part de travers, trop loin. Ici, ça souffle trop. Papa s'accroupit, à la même hauteur. Les feuilles se taisent, un instant. Nina lève le bâton, trop tôt. Un souffle tardif plie le fil. Pas maintenant. La larme de bronze reste nette, elle. Tu vois comment, Nina ? Nina serre le bâton, sans souffler. Alors on fait quoi ?</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Entre ses doigts, le bois du bâton est tiède. Le &lt;emphasis level="moderate"&gt;tilleul&lt;/emphasis&gt; agite ses feuilles, trop vite. Le fil claque, trop léger dans l'air. Le vent prend tout ! Une feuille claque, puis une autre. La bulle part de travers, trop loin. Ici, ça souffle trop. Papa s'accroupit, à la même hauteur. Les feuilles se taisent, un instant. Nina lève le bâton, trop tôt. Un souffle tardif plie le fil. Pas maintenant. La larme de bronze reste nette, elle. Tu vois comment, Nina ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Entre ses doigts, le bois du bâton est tiède. Le &lt;emphasis level="moderate"&gt;tilleul&lt;/emphasis&gt; agite ses feuilles, trop vite. Le fil claque, trop léger dans l'air. Le vent prend tout ! Une feuille claque, puis une autre. La bulle part de travers, trop loin. Ici, ça souffle trop. Papa s'accroupit, à la même hauteur. Les feuilles se taisent, un instant. Nina lève le bâton, trop tôt. Un souffle tardif plie le fil. Pas maintenant. La larme de bronze reste nette, elle. Tu vois comment, Nina ? Nina serre le bâton, sans souffler. Alors on fait quoi ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Entre ses doigts, le bois du bâton est tiède. Le &lt;emphasis&gt;tilleul&lt;/emphasis&gt; agite ses feuilles, trop vite. Le fil claque, trop léger dans l'air. Le vent prend tout ! Une feuille claque, puis une autre. La bulle part de travers, trop loin. Ici, ça souffle trop. Papa s'accroupit, à la même hauteur. Les feuilles se taisent, un instant. Nina lève le bâton, trop tôt. Un souffle tardif plie le fil. Pas maintenant. La larme de bronze reste nette, elle. Tu vois comment, Nina ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Entre ses doigts, le bois du bâton est tiède. Le &lt;emphasis&gt;tilleul&lt;/emphasis&gt; agite ses feuilles, trop vite. Le fil claque, trop léger dans l'air. Le vent prend tout ! Une feuille claque, puis une autre. La bulle part de travers, trop loin. Ici, ça souffle trop. Papa s'accroupit, à la même hauteur. Les feuilles se taisent, un instant. Nina lève le bâton, trop tôt. Un souffle tardif plie le fil. Pas maintenant. La larme de bronze reste nette, elle. Tu vois comment, Nina ? Nina serre le bâton, sans souffler. Alors on fait quoi ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr"/>
@@ -5491,7 +5515,9 @@
 narrateur|Un souffle tardif plie le fil.
 enfant-f|Pas maintenant.
 narrateur|La larme de bronze reste nette, elle.
-maman|Tu vois comment, Nina ?</t>
+maman|Tu vois comment, Nina ?
+narrateur|Nina serre le bâton, sans souffler.
+enfant-f|Alors on fait quoi ?</t>
         </is>
       </c>
       <c r="AX24" t="inlineStr">
@@ -5719,17 +5745,17 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>On attend les feuilles, d'abord. Elle tient le bâton, puis attend les feuilles. Les feuilles vont, reviennent, puis se taisent. L'air redevient un seul souffle, net. La larme de bronze ne bouge plus, du tout. Le tilleul n'a plus claqué. Maintenant, tu peux rester. Pendant ce temps, le bâton reste droit. Tu as laissé les feuilles finir.</t>
+          <t>On attend les feuilles, d'abord. Elle tient le bâton, puis attend les feuilles. Les feuilles vont, reviennent, puis se taisent. L'air redevient un seul souffle, net. La larme de bronze ne bouge plus, du tout. Le tilleul n'a plus claqué. Maintenant, tu peux rester. Pendant ce temps, le bâton reste droit. Elle ferme les yeux, et compte les claquements. Quand ça se tait, je souffle. Tu as laissé les feuilles finir.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend les &lt;emphasis level="moderate"&gt;feuilles&lt;/emphasis&gt;, d'abord. Elle tient le bâton, puis attend les feuilles. Les feuilles vont, reviennent, puis se taisent. L'air redevient un seul souffle, net. La larme de bronze ne bouge plus, du tout. Le tilleul n'a plus claqué. Maintenant, tu peux rester. Pendant ce temps, le bâton reste droit. Tu as laissé les feuilles finir.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend les &lt;emphasis level="moderate"&gt;feuilles&lt;/emphasis&gt;, d'abord. Elle tient le bâton, puis attend les feuilles. Les feuilles vont, reviennent, puis se taisent. L'air redevient un seul souffle, net. La larme de bronze ne bouge plus, du tout. Le tilleul n'a plus claqué. Maintenant, tu peux rester. Pendant ce temps, le bâton reste droit. Elle ferme les yeux, et compte les claquements. Quand ça se tait, je souffle. Tu as laissé les feuilles finir.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>On attend les &lt;emphasis&gt;feuilles&lt;/emphasis&gt;, d'abord. Elle tient le bâton, puis attend les feuilles. Les feuilles vont, reviennent, puis se taisent. L'air redevient un seul souffle, net. La larme de bronze ne bouge plus, du tout. Le tilleul n'a plus claqué. Maintenant, tu peux rester. Pendant ce temps, le bâton reste droit. Tu as laissé les feuilles finir. [pause]</t>
+          <t>On attend les &lt;emphasis&gt;feuilles&lt;/emphasis&gt;, d'abord. Elle tient le bâton, puis attend les feuilles. Les feuilles vont, reviennent, puis se taisent. L'air redevient un seul souffle, net. La larme de bronze ne bouge plus, du tout. Le tilleul n'a plus claqué. Maintenant, tu peux rester. Pendant ce temps, le bâton reste droit. Elle ferme les yeux, et compte les claquements. Quand ça se tait, je souffle. Tu as laissé les feuilles finir. [pause]</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr"/>
@@ -5871,6 +5897,8 @@
 papa|Le tilleul n'a plus claqué.
 enfant-f|Maintenant, tu peux rester.
 narrateur|Pendant ce temps, le bâton reste droit.
+narrateur|Elle ferme les yeux, et compte les claquements.
+enfant-f|Quand ça se tait, je souffle.
 maman|Tu as laissé les feuilles finir.</t>
         </is>
       </c>
@@ -6088,17 +6116,17 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Derrière, pas trop près du vent. Derrière le tronc, le bâton ne claque plus. Nina se glisse derrière le tronc, tout bas. Rien ne claque, rien ne pousse plus. La larme de bronze se voit entre deux branches. Tu n'as pas couru. Tu es ronde, maintenant. Un fil de savon cherche l'air, abrité. Derrière, l'air était plus doux.</t>
+          <t>Derrière, pas trop près du vent. Derrière le tronc, le bâton ne claque plus. Nina se glisse derrière le tronc, tout bas. Rien ne claque, rien ne pousse plus. La larme de bronze se voit entre deux branches. Tu n'as pas couru. Tu es ronde, maintenant. Un fil de savon cherche l'air, abrité. Elle s'appuie au tronc, le bois à l'abri. Derrière, le vent ne me prend pas. Derrière, l'air était plus doux.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Derrière, pas trop près du vent. Derrière le tronc, le bâton ne claque plus. Nina se glisse &lt;emphasis level="moderate"&gt;derrière&lt;/emphasis&gt; le tronc, tout bas. Rien ne claque, rien ne pousse plus. La larme de bronze se voit entre deux branches. Tu n'as pas couru. Tu es ronde, maintenant. Un fil de savon cherche l'air, abrité. Derrière, l'air était plus doux.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Derrière, pas trop près du vent. Derrière le tronc, le bâton ne claque plus. Nina se glisse &lt;emphasis level="moderate"&gt;derrière&lt;/emphasis&gt; le tronc, tout bas. Rien ne claque, rien ne pousse plus. La larme de bronze se voit entre deux branches. Tu n'as pas couru. Tu es ronde, maintenant. Un fil de savon cherche l'air, abrité. Elle s'appuie au tronc, le bois à l'abri. Derrière, le vent ne me prend pas. Derrière, l'air était plus doux.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Derrière, pas trop près du vent. Derrière le tronc, le bâton ne claque plus. Nina se glisse &lt;emphasis&gt;derrière&lt;/emphasis&gt; le tronc, tout bas. Rien ne claque, rien ne pousse plus. La larme de bronze se voit entre deux branches. Tu n'as pas couru. Tu es ronde, maintenant. Un fil de savon cherche l'air, abrité. Derrière, l'air était plus doux. [pause]</t>
+          <t>Derrière, pas trop près du vent. Derrière le tronc, le bâton ne claque plus. Nina se glisse &lt;emphasis&gt;derrière&lt;/emphasis&gt; le tronc, tout bas. Rien ne claque, rien ne pousse plus. La larme de bronze se voit entre deux branches. Tu n'as pas couru. Tu es ronde, maintenant. Un fil de savon cherche l'air, abrité. Elle s'appuie au tronc, le bois à l'abri. Derrière, le vent ne me prend pas. Derrière, l'air était plus doux. [pause]</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr"/>
@@ -6240,6 +6268,8 @@
 papa|Tu n'as pas couru.
 enfant-f|Tu es ronde, maintenant.
 narrateur|Un fil de savon cherche l'air, abrité.
+narrateur|Elle s'appuie au tronc, le bois à l'abri.
+enfant-f|Derrière, le vent ne me prend pas.
 maman|Derrière, l'air était plus doux.</t>
         </is>
       </c>
@@ -6457,17 +6487,17 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Tout petit, tout serré. Une toute petite bulle quitte le bâton. Nina souffle à peine, sans prendre le vent. Le tilleul se tait, plus loin, tout seul. La larme de bronze prend le petit rond. Le petit rond n'a pas volé. Tu restes, bulle. Un fil de savon cherche l'air, minuscule. Le petit rond a suffi.</t>
+          <t>Tout petit, tout serré. Une toute petite bulle quitte le bâton. Nina souffle à peine, sans prendre le vent. Le tilleul se tait, plus loin, tout seul. La larme de bronze prend le petit rond. Le petit rond n'a pas volé. Tu restes, bulle. Un fil de savon cherche l'air, minuscule. Elle pince le cercle, pour un tout petit trou. Une petite, pour la larme. Le petit rond a suffi.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Tout petit, tout serré. Une toute petite bulle quitte le bâton. Nina souffle à peine, sans prendre le vent. Le tilleul se tait, plus loin, tout seul. La larme de bronze prend le petit rond. Le petit rond n'a pas volé. Tu restes, bulle. Un fil de savon cherche l'air, minuscule. Le petit rond a suffi.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Tout petit, tout serré. Une toute petite bulle quitte le bâton. Nina souffle à peine, sans prendre le vent. Le tilleul se tait, plus loin, tout seul. La larme de bronze prend le petit rond. Le petit rond n'a pas volé. Tu restes, bulle. Un fil de savon cherche l'air, minuscule. Elle pince le cercle, pour un &lt;emphasis level="moderate"&gt;tout petit&lt;/emphasis&gt; trou. Une petite, pour la larme. Le petit rond a suffi.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Tout petit, tout serré. Une toute petite bulle quitte le bâton. Nina souffle à peine, sans prendre le vent. Le tilleul se tait, plus loin, tout seul. La larme de bronze prend le petit rond. Le petit rond n'a pas volé. Tu restes, bulle. Un fil de savon cherche l'air, minuscule. Le petit rond a suffi. [pause]</t>
+          <t>Tout petit, tout serré. Une toute petite bulle quitte le bâton. Nina souffle à peine, sans prendre le vent. Le tilleul se tait, plus loin, tout seul. La larme de bronze prend le petit rond. Le petit rond n'a pas volé. Tu restes, bulle. Un fil de savon cherche l'air, minuscule. Elle pince le cercle, pour un &lt;emphasis&gt;tout petit&lt;/emphasis&gt; trou. Une petite, pour la larme. Le petit rond a suffi. [pause]</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr"/>
@@ -6609,6 +6639,8 @@
 papa|Le petit rond n'a pas volé.
 enfant-f|Tu restes, bulle.
 narrateur|Un fil de savon cherche l'air, minuscule.
+narrateur|Elle pince le cercle, pour un tout petit trou.
+enfant-f|Une petite, pour la larme.
 maman|Le petit rond a suffi.</t>
         </is>
       </c>
@@ -6826,17 +6858,17 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Nina dévisse d'abord le savon, sans se presser. Il va donner la bulle. Une goutte, pas tout le flacon. La goutte reste au pouce, puis tombe. Elle veut souffler, tout de suite. Le bâton t'attend, près du sac. Papa pose la coupelle contre le gravier chaud. Nina serre les trois contre son ventre. Savon, tu restes avec moi. Le flacon colle un peu sa manche. Le savon est ouvert, tu peux y aller. Sans courir, Nina.</t>
+          <t>Nina dévisse d'abord le savon, sans se presser. Il va donner la bulle. Une goutte, pas tout le flacon. La goutte reste au pouce, puis tombe. Elle veut souffler, tout de suite. Le bâton t'attend, près du sac. Papa pose la coupelle contre le gravier chaud. Nina serre les trois contre son ventre. Savon, tu restes avec moi. Le flacon colle un peu sa manche. Le savon est ouvert, tu peux y aller. Sans courir, Nina. Elle essuie le pouce contre le bois. Vite, avant la cloche.</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nina dévisse d'abord le &lt;emphasis level="moderate"&gt;savon&lt;/emphasis&gt;, sans se presser. Il va donner la bulle. Une goutte, pas tout le flacon. La goutte reste au pouce, puis tombe. Elle veut souffler, tout de suite. Le bâton t'attend, près du sac. Papa pose la coupelle contre le gravier chaud. Nina serre les trois contre son ventre. Savon, tu restes avec moi. Le flacon colle un peu sa manche. Le savon est ouvert, tu peux y aller. Sans courir, Nina.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nina dévisse d'abord le &lt;emphasis level="moderate"&gt;savon&lt;/emphasis&gt;, sans se presser. Il va donner la bulle. Une goutte, pas tout le flacon. La goutte reste au pouce, puis tombe. Elle veut souffler, tout de suite. Le bâton t'attend, près du sac. Papa pose la coupelle contre le gravier chaud. Nina serre les trois contre son ventre. Savon, tu restes avec moi. Le flacon colle un peu sa manche. Le savon est ouvert, tu peux y aller. Sans courir, Nina. Elle essuie le pouce contre le bois. Vite, avant la cloche.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Nina dévisse d'abord le &lt;emphasis&gt;savon&lt;/emphasis&gt;, sans se presser. Il va donner la bulle. Une goutte, pas tout le flacon. La goutte reste au pouce, puis tombe. Elle veut souffler, tout de suite. Le bâton t'attend, près du sac. Papa pose la coupelle contre le gravier chaud. Nina serre les trois contre son ventre. Savon, tu restes avec moi. Le flacon colle un peu sa manche. Le savon est ouvert, tu peux y aller. Sans courir, Nina. [pause]</t>
+          <t>Nina dévisse d'abord le &lt;emphasis&gt;savon&lt;/emphasis&gt;, sans se presser. Il va donner la bulle. Une goutte, pas tout le flacon. La goutte reste au pouce, puis tombe. Elle veut souffler, tout de suite. Le bâton t'attend, près du sac. Papa pose la coupelle contre le gravier chaud. Nina serre les trois contre son ventre. Savon, tu restes avec moi. Le flacon colle un peu sa manche. Le savon est ouvert, tu peux y aller. Sans courir, Nina. Elle essuie le pouce contre le bois. Vite, avant la cloche. [pause]</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr"/>
@@ -6981,7 +7013,9 @@
 enfant-f|Savon, tu restes avec moi.
 narrateur|Le flacon colle un peu sa manche.
 maman|Le savon est ouvert, tu peux y aller.
-papa|Sans courir, Nina.</t>
+papa|Sans courir, Nina.
+narrateur|Elle essuie le pouce contre le bois.
+enfant-f|Vite, avant la cloche.</t>
         </is>
       </c>
       <c r="AX32" t="inlineStr">
@@ -7201,17 +7235,17 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Le savon pend au poignet, un peu lâche. Il va filer la bulle. Ça sent le savon, toi. Tes mains sont prêtes ? Oui, maman. Une goutte se tait, puis plus rien. On avance, sans se presser.</t>
+          <t>Le savon pend au poignet, un peu lâche. Il va filer la bulle. Ça sent le savon, toi. Tes mains sont prêtes ? Oui, maman. Une goutte se tait, puis plus rien. On avance, sans se presser. Le flacon tape son poignet, à chaque pas. Le bâton et la coupelle sont avec toi.</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;savon&lt;/emphasis&gt; pend au poignet, un peu lâche. Il va filer la bulle. Ça sent le savon, toi. Tes mains sont prêtes ? Oui, maman. Une goutte se tait, puis plus rien. On avance, sans se presser.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;savon&lt;/emphasis&gt; pend au poignet, un peu lâche. Il va filer la bulle. Ça sent le savon, toi. Tes mains sont prêtes ? Oui, maman. Une goutte se tait, puis plus rien. On avance, sans se presser. Le flacon tape son poignet, à chaque pas. Le bâton et la coupelle sont avec toi.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Le &lt;emphasis&gt;savon&lt;/emphasis&gt; pend au poignet, un peu lâche. Il va filer la bulle. Ça sent le savon, toi. Tes mains sont prêtes ? Oui, maman. Une goutte se tait, puis plus rien. On avance, sans se presser. [pause]</t>
+          <t>Le &lt;emphasis&gt;savon&lt;/emphasis&gt; pend au poignet, un peu lâche. Il va filer la bulle. Ça sent le savon, toi. Tes mains sont prêtes ? Oui, maman. Une goutte se tait, puis plus rien. On avance, sans se presser. Le flacon tape son poignet, à chaque pas. Le bâton et la coupelle sont avec toi. [pause]</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr"/>
@@ -7351,7 +7385,9 @@
 maman|Tes mains sont prêtes ?
 enfant-f|Oui, maman.
 narrateur|Une goutte se tait, puis plus rien.
-maman|On avance, sans se presser.</t>
+maman|On avance, sans se presser.
+narrateur|Le flacon tape son poignet, à chaque pas.
+papa|Le bâton et la coupelle sont avec toi.</t>
         </is>
       </c>
       <c r="AX34" t="inlineStr">
@@ -7383,17 +7419,17 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Le savon colle à sa manche. Devant, l'allée soulève trop de poussière. Le socle, lui, brûle au soleil. Sous le tilleul, les feuilles claquent. Nina, tu vas où ?</t>
+          <t>Le savon colle à sa manche. Devant, l'allée soulève trop de poussière. Le socle, lui, brûle au soleil. Sous le tilleul, les feuilles claquent. Nina, tu vas où ? La larme attend, sur le nez.</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Le savon colle à sa manche. Devant, l'allée soulève trop de poussière. Le socle, lui, brûle au soleil. Sous le tilleul, les feuilles claquent. Nina, tu vas où ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Le savon colle à sa manche. Devant, l'allée soulève trop de poussière. Le socle, lui, brûle au soleil. Sous le tilleul, les feuilles claquent. Nina, tu vas où ? La larme attend, sur le nez.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Le savon colle à sa manche. Devant, l'allée soulève trop de poussière. Le socle, lui, brûle au soleil. Sous le tilleul, les feuilles claquent. Nina, tu vas où ?&lt;/slow&gt; [long-pause]</t>
+          <t>&lt;slow&gt;Le savon colle à sa manche. Devant, l'allée soulève trop de poussière. Le socle, lui, brûle au soleil. Sous le tilleul, les feuilles claquent. Nina, tu vas où ? La larme attend, sur le nez.&lt;/slow&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr"/>
@@ -7555,7 +7591,8 @@
 narrateur|Devant, l'allée soulève trop de poussière.
 narrateur|Le socle, lui, brûle au soleil.
 narrateur|Sous le tilleul, les feuilles claquent.
-papa|Nina, tu vas où ?</t>
+papa|Nina, tu vas où ?
+maman|La larme attend, sur le nez.</t>
         </is>
       </c>
     </row>
@@ -7582,17 +7619,17 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Dans sa paume, le flacon de savon est tiède. Le gravier de l'allée saute sous les pas. La goutte saute, trop sèche, trop vite. Ma bulle a crevé ! Le sourire de Nina disparaît. Dans sa poitrine, l'envie et la peur se bousculent. Ici, ça n'arrête pas. Papa s'accroupit, à la même hauteur. Elle ouvre le flacon, trop vite. Un pas tardif soulève la poussière, gris. Pas maintenant. La larme de bronze est grise, trop. Tu vois comment, Nina ?</t>
+          <t>Dans sa paume, le flacon de savon est tiède. Le gravier de l'allée saute sous les pas. La goutte saute, trop sèche, trop vite. Ma bulle a crevé ! Le sourire de Nina disparaît. Dans sa poitrine, l'envie et la peur se bousculent. Ici, ça n'arrête pas. Papa s'accroupit, à la même hauteur. Elle ouvre le flacon, trop vite. Un pas tardif soulève la poussière, gris. Pas maintenant. La larme de bronze est grise, trop. Tu vois comment, Nina ? Nina serre le flacon, sans ouvrir. Alors on fait quoi ?</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Dans sa paume, le flacon de savon est tiède. Le gravier de l'&lt;emphasis level="moderate"&gt;allée&lt;/emphasis&gt; saute sous les pas. La goutte saute, trop sèche, trop vite. Ma bulle a crevé ! Le sourire de Nina disparaît. Dans sa poitrine, l'envie et la peur se bousculent. Ici, ça n'arrête pas. Papa s'accroupit, à la même hauteur. Elle ouvre le flacon, trop vite. Un pas tardif soulève la poussière, gris. Pas maintenant. La larme de bronze est grise, trop. Tu vois comment, Nina ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Dans sa paume, le flacon de savon est tiède. Le gravier de l'&lt;emphasis level="moderate"&gt;allée&lt;/emphasis&gt; saute sous les pas. La goutte saute, trop sèche, trop vite. Ma bulle a crevé ! Le sourire de Nina disparaît. Dans sa poitrine, l'envie et la peur se bousculent. Ici, ça n'arrête pas. Papa s'accroupit, à la même hauteur. Elle ouvre le flacon, trop vite. Un pas tardif soulève la poussière, gris. Pas maintenant. La larme de bronze est grise, trop. Tu vois comment, Nina ? Nina serre le flacon, sans ouvrir. Alors on fait quoi ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Dans sa paume, le flacon de savon est tiède. Le gravier de l'&lt;emphasis&gt;allée&lt;/emphasis&gt; saute sous les pas. La goutte saute, trop sèche, trop vite. Ma bulle a crevé ! Le sourire de Nina disparaît. Dans sa poitrine, l'envie et la peur se bousculent. Ici, ça n'arrête pas. Papa s'accroupit, à la même hauteur. Elle ouvre le flacon, trop vite. Un pas tardif soulève la poussière, gris. Pas maintenant. La larme de bronze est grise, trop. Tu vois comment, Nina ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Dans sa paume, le flacon de savon est tiède. Le gravier de l'&lt;emphasis&gt;allée&lt;/emphasis&gt; saute sous les pas. La goutte saute, trop sèche, trop vite. Ma bulle a crevé ! Le sourire de Nina disparaît. Dans sa poitrine, l'envie et la peur se bousculent. Ici, ça n'arrête pas. Papa s'accroupit, à la même hauteur. Elle ouvre le flacon, trop vite. Un pas tardif soulève la poussière, gris. Pas maintenant. La larme de bronze est grise, trop. Tu vois comment, Nina ? Nina serre le flacon, sans ouvrir. Alors on fait quoi ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr"/>
@@ -7742,7 +7779,9 @@
 narrateur|Un pas tardif soulève la poussière, gris.
 enfant-f|Pas maintenant.
 narrateur|La larme de bronze est grise, trop.
-maman|Tu vois comment, Nina ?</t>
+maman|Tu vois comment, Nina ?
+narrateur|Nina serre le flacon, sans ouvrir.
+enfant-f|Alors on fait quoi ?</t>
         </is>
       </c>
       <c r="AX36" t="inlineStr">
@@ -7970,17 +8009,17 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>On attend les pas. Nina tient le savon, sans ouvrir. Le gravier se tait, une fois, puis plus. La larme de bronze redevient sombre, nette. Tu peux partir, maintenant. Fermé, le savon attend contre son pouce. Les pas se sont tus, là. La goutte file, ronde, vers la larme. Tu as laissé le gravier se taire.</t>
+          <t>On attend les pas. Nina tient le savon, sans ouvrir. Le gravier se tait, une fois, puis plus. La larme de bronze redevient sombre, nette. Tu peux partir, maintenant. Fermé, le savon attend contre son pouce. Les pas se sont tus, là. La goutte file, ronde, vers la larme. Elle compte jusqu'à trois, bouchon fermé. Le flacon, je l'ouvre après. Tu as laissé le gravier se taire.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend les &lt;emphasis level="moderate"&gt;pas&lt;/emphasis&gt;. Nina tient le savon, sans ouvrir. Le gravier se tait, une fois, puis plus. La larme de bronze redevient sombre, nette. Tu peux partir, maintenant. Fermé, le savon attend contre son pouce. Les pas se sont tus, là. La goutte file, ronde, vers la larme. Tu as laissé le gravier se taire.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend les &lt;emphasis level="moderate"&gt;pas&lt;/emphasis&gt;. Nina tient le savon, sans ouvrir. Le gravier se tait, une fois, puis plus. La larme de bronze redevient sombre, nette. Tu peux partir, maintenant. Fermé, le savon attend contre son pouce. Les pas se sont tus, là. La goutte file, ronde, vers la larme. Elle compte jusqu'à trois, bouchon fermé. Le flacon, je l'ouvre après. Tu as laissé le gravier se taire.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>On attend les &lt;emphasis&gt;pas&lt;/emphasis&gt;. Nina tient le savon, sans ouvrir. Le gravier se tait, une fois, puis plus. La larme de bronze redevient sombre, nette. Tu peux partir, maintenant. Fermé, le savon attend contre son pouce. Les pas se sont tus, là. La goutte file, ronde, vers la larme. Tu as laissé le gravier se taire. [pause]</t>
+          <t>On attend les &lt;emphasis&gt;pas&lt;/emphasis&gt;. Nina tient le savon, sans ouvrir. Le gravier se tait, une fois, puis plus. La larme de bronze redevient sombre, nette. Tu peux partir, maintenant. Fermé, le savon attend contre son pouce. Les pas se sont tus, là. La goutte file, ronde, vers la larme. Elle compte jusqu'à trois, bouchon fermé. Le flacon, je l'ouvre après. Tu as laissé le gravier se taire. [pause]</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr"/>
@@ -8122,6 +8161,8 @@
 narrateur|Fermé, le savon attend contre son pouce.
 papa|Les pas se sont tus, là.
 narrateur|La goutte file, ronde, vers la larme.
+narrateur|Elle compte jusqu'à trois, bouchon fermé.
+enfant-f|Le flacon, je l'ouvre après.
 maman|Tu as laissé le gravier se taire.</t>
         </is>
       </c>
@@ -8339,17 +8380,17 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Plus bas, d'abord. Elle baisse le savon, loin de la poussière. Nina s'accroupit, les genoux au gravier. L'air est plus doux, près de l'herbe. La larme de bronze se voit d'en bas. Ici, tu ne crèves plus. Tu as vu l'herbe, avant. Une goutte de savon brille, prête à filer. Près du sol, ça tenait mieux.</t>
+          <t>Plus bas, d'abord. Elle baisse le savon, loin de la poussière. Nina s'accroupit, les genoux au gravier. L'air est plus doux, près de l'herbe. La larme de bronze se voit d'en bas. Ici, tu ne crèves plus. Tu as vu l'herbe, avant. Une goutte de savon brille, prête à filer. Elle pose le flacon dans l'herbe, droit. Une goutte, pas plus. Près du sol, ça tenait mieux.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Plus bas, d'abord. Elle baisse le savon, loin de la poussière. Nina s'accroupit, les genoux au gravier. L'air est plus doux, près de l'herbe. La larme de bronze se voit d'en bas. Ici, tu ne crèves plus. Tu as vu l'herbe, avant. Une goutte de savon brille, prête à filer. Près du sol, ça tenait mieux.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Plus bas, d'abord. Elle baisse le savon, loin de la poussière. Nina s'accroupit, les genoux au gravier. L'air est plus doux, près de l'herbe. La larme de bronze se voit d'en bas. Ici, tu ne crèves plus. Tu as vu l'herbe, avant. Une goutte de savon brille, prête à filer. Elle pose le flacon dans l'herbe, droit. Une goutte, pas plus. Près du sol, ça tenait mieux.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Plus bas, d'abord. Elle baisse le savon, loin de la poussière. Nina s'accroupit, les genoux au gravier. L'air est plus doux, près de l'herbe. La larme de bronze se voit d'en bas. Ici, tu ne crèves plus. Tu as vu l'herbe, avant. Une goutte de savon brille, prête à filer. Près du sol, ça tenait mieux. [pause]</t>
+          <t>Plus bas, d'abord. Elle baisse le savon, loin de la poussière. Nina s'accroupit, les genoux au gravier. L'air est plus doux, près de l'herbe. La larme de bronze se voit d'en bas. Ici, tu ne crèves plus. Tu as vu l'herbe, avant. Une goutte de savon brille, prête à filer. Elle pose le flacon dans l'herbe, droit. Une goutte, pas plus. Près du sol, ça tenait mieux. [pause]</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr"/>
@@ -8491,6 +8532,8 @@
 enfant-f|Ici, tu ne crèves plus.
 papa|Tu as vu l'herbe, avant.
 narrateur|Une goutte de savon brille, prête à filer.
+narrateur|Elle pose le flacon dans l'herbe, droit.
+enfant-f|Une goutte, pas plus.
 maman|Près du sol, ça tenait mieux.</t>
         </is>
       </c>
@@ -8708,17 +8751,17 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Au bord, tout petit. Elle glisse le savon vers le bord d'herbe. L'herbe tient, sans laisser la poussière. Nina ouvre le flacon, une seule goutte. La larme de bronze luit, hors de l'allée. Le bord n'a pas soulevé. Tu es à l'abri. Le rond monte, lent, jusqu'au nez. Tu as dit ça tout bas.</t>
+          <t>Au bord, tout petit. Elle glisse le savon vers le bord d'herbe. L'herbe tient, sans laisser la poussière. Nina ouvre le flacon, une seule goutte. La larme de bronze luit, hors de l'allée. Le bord n'a pas soulevé. Tu es à l'abri. Le rond monte, lent, jusqu'au nez. Elle mouille le cercle au bord, pas au milieu. Ici, la poussière ne vient pas. Tu as dit ça tout bas.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Au &lt;emphasis level="moderate"&gt;bord&lt;/emphasis&gt;, tout petit. Elle glisse le savon vers le bord d'herbe. L'herbe tient, sans laisser la poussière. Nina ouvre le flacon, une seule goutte. La larme de bronze luit, hors de l'allée. Le bord n'a pas soulevé. Tu es à l'abri. Le rond monte, lent, jusqu'au nez. Tu as dit ça tout bas.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Au &lt;emphasis level="moderate"&gt;bord&lt;/emphasis&gt;, tout petit. Elle glisse le savon vers le bord d'herbe. L'herbe tient, sans laisser la poussière. Nina ouvre le flacon, une seule goutte. La larme de bronze luit, hors de l'allée. Le bord n'a pas soulevé. Tu es à l'abri. Le rond monte, lent, jusqu'au nez. Elle mouille le cercle au bord, pas au milieu. Ici, la poussière ne vient pas. Tu as dit ça tout bas.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Au &lt;emphasis&gt;bord&lt;/emphasis&gt;, tout petit. Elle glisse le savon vers le bord d'herbe. L'herbe tient, sans laisser la poussière. Nina ouvre le flacon, une seule goutte. La larme de bronze luit, hors de l'allée. Le bord n'a pas soulevé. Tu es à l'abri. Le rond monte, lent, jusqu'au nez. Tu as dit ça tout bas. [pause]</t>
+          <t>Au &lt;emphasis&gt;bord&lt;/emphasis&gt;, tout petit. Elle glisse le savon vers le bord d'herbe. L'herbe tient, sans laisser la poussière. Nina ouvre le flacon, une seule goutte. La larme de bronze luit, hors de l'allée. Le bord n'a pas soulevé. Tu es à l'abri. Le rond monte, lent, jusqu'au nez. Elle mouille le cercle au bord, pas au milieu. Ici, la poussière ne vient pas. Tu as dit ça tout bas. [pause]</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr"/>
@@ -8860,6 +8903,8 @@
 papa|Le bord n'a pas soulevé.
 enfant-f|Tu es à l'abri.
 narrateur|Le rond monte, lent, jusqu'au nez.
+narrateur|Elle mouille le cercle au bord, pas au milieu.
+enfant-f|Ici, la poussière ne vient pas.
 maman|Tu as dit ça tout bas.</t>
         </is>
       </c>
@@ -9077,17 +9122,17 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Dans sa paume, le flacon de savon est tiède. Le bronze tient tout le soleil. La goutte sèche, trop vite, trop chaude. Le nez brûle trop ! La bulle touche, puis crève tout de suite. Il ne reste rien sur le bronze. Ici, c'est trop chaud. Papa s'accroupit, à la même hauteur. Un nuage passe, et Nina penche le flacon. Le soleil revient, net, sur la larme. Pas maintenant. La larme de bronze est sèche, trop pâle. Tu vois comment, Nina ?</t>
+          <t>Dans sa paume, le flacon de savon est tiède. Le bronze tient tout le soleil. La goutte sèche, trop vite, trop chaude. Le nez brûle trop ! La bulle touche, puis crève tout de suite. Il ne reste rien sur le bronze. Ici, c'est trop chaud. Papa s'accroupit, à la même hauteur. Un nuage passe, et Nina penche le flacon. Le soleil revient, net, sur la larme. Pas maintenant. La larme de bronze est sèche, trop pâle. Tu vois comment, Nina ? Nina serre le flacon, sans ouvrir. Alors on fait quoi ?</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Dans sa paume, le flacon de savon est tiède. Le bronze tient tout le soleil. La goutte sèche, trop vite, trop chaude. Le nez brûle trop ! La bulle touche, puis crève tout de suite. Il ne reste rien sur le bronze. Ici, c'est trop chaud. Papa s'accroupit, à la même hauteur. Un nuage passe, et Nina penche le flacon. Le soleil revient, net, sur la larme. Pas maintenant. La larme de bronze est sèche, trop pâle. Tu vois comment, Nina ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Dans sa paume, le flacon de savon est tiède. Le bronze tient tout le soleil. La goutte sèche, trop vite, trop chaude. Le nez brûle trop ! La bulle touche, puis crève tout de suite. Il ne reste rien sur le bronze. Ici, c'est trop chaud. Papa s'accroupit, à la même hauteur. Un nuage passe, et Nina penche le flacon. Le soleil revient, net, sur la larme. Pas maintenant. La larme de bronze est sèche, trop pâle. Tu vois comment, Nina ? Nina serre le flacon, sans ouvrir. Alors on fait quoi ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Dans sa paume, le flacon de savon est tiède. Le bronze tient tout le soleil. La goutte sèche, trop vite, trop chaude. Le nez brûle trop ! La bulle touche, puis crève tout de suite. Il ne reste rien sur le bronze. Ici, c'est trop chaud. Papa s'accroupit, à la même hauteur. Un nuage passe, et Nina penche le flacon. Le soleil revient, net, sur la larme. Pas maintenant. La larme de bronze est sèche, trop pâle. Tu vois comment, Nina ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Dans sa paume, le flacon de savon est tiède. Le bronze tient tout le soleil. La goutte sèche, trop vite, trop chaude. Le nez brûle trop ! La bulle touche, puis crève tout de suite. Il ne reste rien sur le bronze. Ici, c'est trop chaud. Papa s'accroupit, à la même hauteur. Un nuage passe, et Nina penche le flacon. Le soleil revient, net, sur la larme. Pas maintenant. La larme de bronze est sèche, trop pâle. Tu vois comment, Nina ? Nina serre le flacon, sans ouvrir. Alors on fait quoi ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr"/>
@@ -9237,7 +9282,9 @@
 narrateur|Le soleil revient, net, sur la larme.
 enfant-f|Pas maintenant.
 narrateur|La larme de bronze est sèche, trop pâle.
-maman|Tu vois comment, Nina ?</t>
+maman|Tu vois comment, Nina ?
+narrateur|Nina serre le flacon, sans ouvrir.
+enfant-f|Alors on fait quoi ?</t>
         </is>
       </c>
       <c r="AX44" t="inlineStr">
@@ -9465,17 +9512,17 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>On attend l'ombre. Une ombre de tilleul glisse sur le nez. Sous l'ombre, le savon ne sèche plus. Le bronze se tait, puis se refroidit. La larme de bronze redevient sombre, froide. Le nez est redevenu doux. Maintenant, tu me vois. Fermé, le savon attend contre son pouce. Tu as laissé l'ombre arriver.</t>
+          <t>On attend l'ombre. Une ombre de tilleul glisse sur le nez. Sous l'ombre, le savon ne sèche plus. Le bronze se tait, puis se refroidit. La larme de bronze redevient sombre, froide. Le nez est redevenu doux. Maintenant, tu me vois. Fermé, le savon attend contre son pouce. Elle cache le flacon sous l'ombre, d'abord. Le savon ne sèche plus, là. Tu as laissé l'ombre arriver.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend l'&lt;emphasis level="moderate"&gt;ombre&lt;/emphasis&gt;. Une ombre de tilleul glisse sur le nez. Sous l'ombre, le savon ne sèche plus. Le bronze se tait, puis se refroidit. La larme de bronze redevient sombre, froide. Le nez est redevenu doux. Maintenant, tu me vois. Fermé, le savon attend contre son pouce. Tu as laissé l'ombre arriver.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend l'&lt;emphasis level="moderate"&gt;ombre&lt;/emphasis&gt;. Une ombre de tilleul glisse sur le nez. Sous l'ombre, le savon ne sèche plus. Le bronze se tait, puis se refroidit. La larme de bronze redevient sombre, froide. Le nez est redevenu doux. Maintenant, tu me vois. Fermé, le savon attend contre son pouce. Elle cache le flacon sous l'ombre, d'abord. Le savon ne sèche plus, là. Tu as laissé l'ombre arriver.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>On attend l'&lt;emphasis&gt;ombre&lt;/emphasis&gt;. Une ombre de tilleul glisse sur le nez. Sous l'ombre, le savon ne sèche plus. Le bronze se tait, puis se refroidit. La larme de bronze redevient sombre, froide. Le nez est redevenu doux. Maintenant, tu me vois. Fermé, le savon attend contre son pouce. Tu as laissé l'ombre arriver. [pause]</t>
+          <t>On attend l'&lt;emphasis&gt;ombre&lt;/emphasis&gt;. Une ombre de tilleul glisse sur le nez. Sous l'ombre, le savon ne sèche plus. Le bronze se tait, puis se refroidit. La larme de bronze redevient sombre, froide. Le nez est redevenu doux. Maintenant, tu me vois. Fermé, le savon attend contre son pouce. Elle cache le flacon sous l'ombre, d'abord. Le savon ne sèche plus, là. Tu as laissé l'ombre arriver. [pause]</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr"/>
@@ -9617,6 +9664,8 @@
 maman|Le nez est redevenu doux.
 enfant-f|Maintenant, tu me vois.
 narrateur|Fermé, le savon attend contre son pouce.
+narrateur|Elle cache le flacon sous l'ombre, d'abord.
+enfant-f|Le savon ne sèche plus, là.
 papa|Tu as laissé l'ombre arriver.</t>
         </is>
       </c>
@@ -9834,17 +9883,17 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>L'oiseau, d'abord, il est plus frais. Elle pose d'abord la goutte sur l'oiseau. L'oiseau de bronze est à l'ombre, lui. Le rond glisse, lent, vers la larme. Une goutte de savon brille, courte. Tu n'as pas soufflé trop fort. C'est pour toi. La larme de bronze reçoit le rond, entier. L'oiseau était plus frais, tu as vu.</t>
+          <t>L'oiseau, d'abord, il est plus frais. Elle pose d'abord la goutte sur l'oiseau. L'oiseau de bronze est à l'ombre, lui. Le rond glisse, lent, vers la larme. Une goutte de savon brille, courte. Tu n'as pas soufflé trop fort. C'est pour toi. La larme de bronze reçoit le rond, entier. Elle pose une goutte sur le bec, d'abord. Le bec est frais, pas le nez. L'oiseau était plus frais, tu as vu.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;L'&lt;emphasis level="moderate"&gt;oiseau&lt;/emphasis&gt;, d'abord, il est plus frais. Elle pose d'abord la goutte sur l'oiseau. L'oiseau de bronze est à l'ombre, lui. Le rond glisse, lent, vers la larme. Une goutte de savon brille, courte. Tu n'as pas soufflé trop fort. C'est pour toi. La larme de bronze reçoit le rond, entier. L'oiseau était plus frais, tu as vu.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;L'&lt;emphasis level="moderate"&gt;oiseau&lt;/emphasis&gt;, d'abord, il est plus frais. Elle pose d'abord la goutte sur l'oiseau. L'oiseau de bronze est à l'ombre, lui. Le rond glisse, lent, vers la larme. Une goutte de savon brille, courte. Tu n'as pas soufflé trop fort. C'est pour toi. La larme de bronze reçoit le rond, entier. Elle pose une goutte sur le bec, d'abord. Le bec est frais, pas le nez. L'oiseau était plus frais, tu as vu.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>L'&lt;emphasis&gt;oiseau&lt;/emphasis&gt;, d'abord, il est plus frais. Elle pose d'abord la goutte sur l'oiseau. L'oiseau de bronze est à l'ombre, lui. Le rond glisse, lent, vers la larme. Une goutte de savon brille, courte. Tu n'as pas soufflé trop fort. C'est pour toi. La larme de bronze reçoit le rond, entier. L'oiseau était plus frais, tu as vu. [pause]</t>
+          <t>L'&lt;emphasis&gt;oiseau&lt;/emphasis&gt;, d'abord, il est plus frais. Elle pose d'abord la goutte sur l'oiseau. L'oiseau de bronze est à l'ombre, lui. Le rond glisse, lent, vers la larme. Une goutte de savon brille, courte. Tu n'as pas soufflé trop fort. C'est pour toi. La larme de bronze reçoit le rond, entier. Elle pose une goutte sur le bec, d'abord. Le bec est frais, pas le nez. L'oiseau était plus frais, tu as vu. [pause]</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr"/>
@@ -9986,6 +10035,8 @@
 papa|Tu n'as pas soufflé trop fort.
 enfant-f|C'est pour toi.
 narrateur|La larme de bronze reçoit le rond, entier.
+narrateur|Elle pose une goutte sur le bec, d'abord.
+enfant-f|Le bec est frais, pas le nez.
 maman|L'oiseau était plus frais, tu as vu.</t>
         </is>
       </c>
@@ -10203,17 +10254,17 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Tout près, contre le bronze. Nina se glisse contre le socle. Tout près, le savon n'a plus d'air chaud. La bulle n'a plus à voyager trop loin. La larme de bronze est là, à un souffle. Tu t'es mise tout près, contre le nez. Le nez est là. Fermé, le savon attend contre son pouce. Tu t'es mise tout contre.</t>
+          <t>Tout près, contre le bronze. Nina se glisse contre le socle. Tout près, le savon n'a plus d'air chaud. La bulle n'a plus à voyager trop loin. La larme de bronze est là, à un souffle. Tu t'es mise tout près, contre le nez. Le nez est là. Fermé, le savon attend contre son pouce. Elle met une goutte au pouce, tout près. Le pouce, puis la larme. Tu t'es mise tout contre.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Tout près, contre le bronze. Nina se glisse contre le socle. Tout près, le savon n'a plus d'air chaud. La bulle n'a plus à voyager trop loin. La larme de bronze est là, à un souffle. Tu t'es mise &lt;emphasis level="moderate"&gt;tout près&lt;/emphasis&gt;, contre le nez. Le nez est là. Fermé, le savon attend contre son pouce. Tu t'es mise tout contre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Tout près, contre le bronze. Nina se glisse contre le socle. Tout près, le savon n'a plus d'air chaud. La bulle n'a plus à voyager trop loin. La larme de bronze est là, à un souffle. Tu t'es mise &lt;emphasis level="moderate"&gt;tout près&lt;/emphasis&gt;, contre le nez. Le nez est là. Fermé, le savon attend contre son pouce. Elle met une goutte au pouce, tout près. Le pouce, puis la larme. Tu t'es mise tout contre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Tout près, contre le bronze. Nina se glisse contre le socle. Tout près, le savon n'a plus d'air chaud. La bulle n'a plus à voyager trop loin. La larme de bronze est là, à un souffle. Tu t'es mise &lt;emphasis&gt;tout près&lt;/emphasis&gt;, contre le nez. Le nez est là. Fermé, le savon attend contre son pouce. Tu t'es mise tout contre. [pause]</t>
+          <t>Tout près, contre le bronze. Nina se glisse contre le socle. Tout près, le savon n'a plus d'air chaud. La bulle n'a plus à voyager trop loin. La larme de bronze est là, à un souffle. Tu t'es mise &lt;emphasis&gt;tout près&lt;/emphasis&gt;, contre le nez. Le nez est là. Fermé, le savon attend contre son pouce. Elle met une goutte au pouce, tout près. Le pouce, puis la larme. Tu t'es mise tout contre. [pause]</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr"/>
@@ -10355,6 +10406,8 @@
 papa|Tu t'es mise tout près, contre le nez.
 enfant-f|Le nez est là.
 narrateur|Fermé, le savon attend contre son pouce.
+narrateur|Elle met une goutte au pouce, tout près.
+enfant-f|Le pouce, puis la larme.
 maman|Tu t'es mise tout contre.</t>
         </is>
       </c>
@@ -10572,17 +10625,17 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Dans sa paume, le flacon de savon est tiède. Le tilleul agite ses feuilles, trop vite. La goutte s'envole, trop prise par le vent. Le vent prend tout ! Une feuille claque, puis une autre. La bulle part de travers, trop loin. Ici, ça souffle trop. Papa s'accroupit, à la même hauteur. Les feuilles se taisent, un instant. Nina penche le flacon, trop tôt. Un souffle tardif emporte la goutte. Pas maintenant. La larme de bronze reste nette, elle. Tu vois comment, Nina ?</t>
+          <t>Dans sa paume, le flacon de savon est tiède. Le tilleul agite ses feuilles, trop vite. La goutte s'envole, trop prise par le vent. Le vent prend tout ! Une feuille claque, puis une autre. La bulle part de travers, trop loin. Ici, ça souffle trop. Papa s'accroupit, à la même hauteur. Les feuilles se taisent, un instant. Nina penche le flacon, trop tôt. Un souffle tardif emporte la goutte. Pas maintenant. La larme de bronze reste nette, elle. Tu vois comment, Nina ? Nina serre le flacon, sans ouvrir. Alors on fait quoi ?</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Dans sa paume, le flacon de savon est tiède. Le &lt;emphasis level="moderate"&gt;tilleul&lt;/emphasis&gt; agite ses feuilles, trop vite. La goutte s'envole, trop prise par le vent. Le vent prend tout ! Une feuille claque, puis une autre. La bulle part de travers, trop loin. Ici, ça souffle trop. Papa s'accroupit, à la même hauteur. Les feuilles se taisent, un instant. Nina penche le flacon, trop tôt. Un souffle tardif emporte la goutte. Pas maintenant. La larme de bronze reste nette, elle. Tu vois comment, Nina ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Dans sa paume, le flacon de savon est tiède. Le &lt;emphasis level="moderate"&gt;tilleul&lt;/emphasis&gt; agite ses feuilles, trop vite. La goutte s'envole, trop prise par le vent. Le vent prend tout ! Une feuille claque, puis une autre. La bulle part de travers, trop loin. Ici, ça souffle trop. Papa s'accroupit, à la même hauteur. Les feuilles se taisent, un instant. Nina penche le flacon, trop tôt. Un souffle tardif emporte la goutte. Pas maintenant. La larme de bronze reste nette, elle. Tu vois comment, Nina ? Nina serre le flacon, sans ouvrir. Alors on fait quoi ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Dans sa paume, le flacon de savon est tiède. Le &lt;emphasis&gt;tilleul&lt;/emphasis&gt; agite ses feuilles, trop vite. La goutte s'envole, trop prise par le vent. Le vent prend tout ! Une feuille claque, puis une autre. La bulle part de travers, trop loin. Ici, ça souffle trop. Papa s'accroupit, à la même hauteur. Les feuilles se taisent, un instant. Nina penche le flacon, trop tôt. Un souffle tardif emporte la goutte. Pas maintenant. La larme de bronze reste nette, elle. Tu vois comment, Nina ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Dans sa paume, le flacon de savon est tiède. Le &lt;emphasis&gt;tilleul&lt;/emphasis&gt; agite ses feuilles, trop vite. La goutte s'envole, trop prise par le vent. Le vent prend tout ! Une feuille claque, puis une autre. La bulle part de travers, trop loin. Ici, ça souffle trop. Papa s'accroupit, à la même hauteur. Les feuilles se taisent, un instant. Nina penche le flacon, trop tôt. Un souffle tardif emporte la goutte. Pas maintenant. La larme de bronze reste nette, elle. Tu vois comment, Nina ? Nina serre le flacon, sans ouvrir. Alors on fait quoi ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr"/>
@@ -10733,7 +10786,9 @@
 narrateur|Un souffle tardif emporte la goutte.
 enfant-f|Pas maintenant.
 narrateur|La larme de bronze reste nette, elle.
-maman|Tu vois comment, Nina ?</t>
+maman|Tu vois comment, Nina ?
+narrateur|Nina serre le flacon, sans ouvrir.
+enfant-f|Alors on fait quoi ?</t>
         </is>
       </c>
       <c r="AX52" t="inlineStr">
@@ -10961,17 +11016,17 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>On attend les feuilles, d'abord. Elle tient le savon, puis attend les feuilles. Les feuilles vont, reviennent, puis se taisent. L'air redevient un seul souffle, net. La larme de bronze ne bouge plus, du tout. Le tilleul n'a plus claqué. Maintenant, tu peux rester. Fermé, le savon attend contre son pouce. Tu as laissé les feuilles finir.</t>
+          <t>On attend les feuilles, d'abord. Elle tient le savon, puis attend les feuilles. Les feuilles vont, reviennent, puis se taisent. L'air redevient un seul souffle, net. La larme de bronze ne bouge plus, du tout. Le tilleul n'a plus claqué. Maintenant, tu peux rester. Fermé, le savon attend contre son pouce. Elle recapsule entre deux souffles. J'ouvre quand ça se tait. Tu as laissé les feuilles finir.</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend les &lt;emphasis level="moderate"&gt;feuilles&lt;/emphasis&gt;, d'abord. Elle tient le savon, puis attend les feuilles. Les feuilles vont, reviennent, puis se taisent. L'air redevient un seul souffle, net. La larme de bronze ne bouge plus, du tout. Le tilleul n'a plus claqué. Maintenant, tu peux rester. Fermé, le savon attend contre son pouce. Tu as laissé les feuilles finir.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend les &lt;emphasis level="moderate"&gt;feuilles&lt;/emphasis&gt;, d'abord. Elle tient le savon, puis attend les feuilles. Les feuilles vont, reviennent, puis se taisent. L'air redevient un seul souffle, net. La larme de bronze ne bouge plus, du tout. Le tilleul n'a plus claqué. Maintenant, tu peux rester. Fermé, le savon attend contre son pouce. Elle recapsule entre deux souffles. J'ouvre quand ça se tait. Tu as laissé les feuilles finir.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>On attend les &lt;emphasis&gt;feuilles&lt;/emphasis&gt;, d'abord. Elle tient le savon, puis attend les feuilles. Les feuilles vont, reviennent, puis se taisent. L'air redevient un seul souffle, net. La larme de bronze ne bouge plus, du tout. Le tilleul n'a plus claqué. Maintenant, tu peux rester. Fermé, le savon attend contre son pouce. Tu as laissé les feuilles finir. [pause]</t>
+          <t>On attend les &lt;emphasis&gt;feuilles&lt;/emphasis&gt;, d'abord. Elle tient le savon, puis attend les feuilles. Les feuilles vont, reviennent, puis se taisent. L'air redevient un seul souffle, net. La larme de bronze ne bouge plus, du tout. Le tilleul n'a plus claqué. Maintenant, tu peux rester. Fermé, le savon attend contre son pouce. Elle recapsule entre deux souffles. J'ouvre quand ça se tait. Tu as laissé les feuilles finir. [pause]</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr"/>
@@ -11113,6 +11168,8 @@
 papa|Le tilleul n'a plus claqué.
 enfant-f|Maintenant, tu peux rester.
 narrateur|Fermé, le savon attend contre son pouce.
+narrateur|Elle recapsule entre deux souffles.
+enfant-f|J'ouvre quand ça se tait.
 maman|Tu as laissé les feuilles finir.</t>
         </is>
       </c>
@@ -11330,17 +11387,17 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Derrière, pas trop près du vent. Derrière le tronc, le savon ne s'envole plus. Nina se glisse derrière le tronc, tout bas. Rien ne claque, rien ne pousse plus. La larme de bronze se voit entre deux branches. Tu n'as pas couru. Tu es ronde, maintenant. Une goutte de savon brille, abritée. Derrière, l'air était plus doux.</t>
+          <t>Derrière, pas trop près du vent. Derrière le tronc, le savon ne s'envole plus. Nina se glisse derrière le tronc, tout bas. Rien ne claque, rien ne pousse plus. La larme de bronze se voit entre deux branches. Tu n'as pas couru. Tu es ronde, maintenant. Une goutte de savon brille, abritée. Elle savonne le cercle derrière le tronc. Ici, ça ne s'envole pas. Derrière, l'air était plus doux.</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Derrière, pas trop près du vent. Derrière le tronc, le savon ne s'envole plus. Nina se glisse &lt;emphasis level="moderate"&gt;derrière&lt;/emphasis&gt; le tronc, tout bas. Rien ne claque, rien ne pousse plus. La larme de bronze se voit entre deux branches. Tu n'as pas couru. Tu es ronde, maintenant. Une goutte de savon brille, abritée. Derrière, l'air était plus doux.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Derrière, pas trop près du vent. Derrière le tronc, le savon ne s'envole plus. Nina se glisse &lt;emphasis level="moderate"&gt;derrière&lt;/emphasis&gt; le tronc, tout bas. Rien ne claque, rien ne pousse plus. La larme de bronze se voit entre deux branches. Tu n'as pas couru. Tu es ronde, maintenant. Une goutte de savon brille, abritée. Elle savonne le cercle derrière le tronc. Ici, ça ne s'envole pas. Derrière, l'air était plus doux.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Derrière, pas trop près du vent. Derrière le tronc, le savon ne s'envole plus. Nina se glisse &lt;emphasis&gt;derrière&lt;/emphasis&gt; le tronc, tout bas. Rien ne claque, rien ne pousse plus. La larme de bronze se voit entre deux branches. Tu n'as pas couru. Tu es ronde, maintenant. Une goutte de savon brille, abritée. Derrière, l'air était plus doux. [pause]</t>
+          <t>Derrière, pas trop près du vent. Derrière le tronc, le savon ne s'envole plus. Nina se glisse &lt;emphasis&gt;derrière&lt;/emphasis&gt; le tronc, tout bas. Rien ne claque, rien ne pousse plus. La larme de bronze se voit entre deux branches. Tu n'as pas couru. Tu es ronde, maintenant. Une goutte de savon brille, abritée. Elle savonne le cercle derrière le tronc. Ici, ça ne s'envole pas. Derrière, l'air était plus doux. [pause]</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr"/>
@@ -11482,6 +11539,8 @@
 papa|Tu n'as pas couru.
 enfant-f|Tu es ronde, maintenant.
 narrateur|Une goutte de savon brille, abritée.
+narrateur|Elle savonne le cercle derrière le tronc.
+enfant-f|Ici, ça ne s'envole pas.
 maman|Derrière, l'air était plus doux.</t>
         </is>
       </c>
@@ -11699,17 +11758,17 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Tout petit, tout serré. Une toute petite bulle quitte le savon. Nina souffle à peine, sans prendre le vent. Le tilleul se tait, plus loin, tout seul. La larme de bronze prend le petit rond. Le petit rond n'a pas volé. Tu restes, bulle. Une goutte de savon brille, minuscule. Le petit rond a suffi.</t>
+          <t>Tout petit, tout serré. Une toute petite bulle quitte le savon. Nina souffle à peine, sans prendre le vent. Le tilleul se tait, plus loin, tout seul. La larme de bronze prend le petit rond. Le petit rond n'a pas volé. Tu restes, bulle. Une goutte de savon brille, minuscule. Elle prend une seule goutte, pas deux. Une toute petite, pour la larme. Le petit rond a suffi.</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Tout petit, tout serré. Une toute petite bulle quitte le savon. Nina souffle à peine, sans prendre le vent. Le tilleul se tait, plus loin, tout seul. La larme de bronze prend le petit rond. Le petit rond n'a pas volé. Tu restes, bulle. Une goutte de savon brille, minuscule. Le petit rond a suffi.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Tout petit, tout serré. Une toute petite bulle quitte le savon. Nina souffle à peine, sans prendre le vent. Le tilleul se tait, plus loin, tout seul. La larme de bronze prend le petit rond. Le petit rond n'a pas volé. Tu restes, bulle. Une goutte de savon brille, minuscule. Elle prend une seule goutte, pas deux. Une toute petite, pour la larme. Le petit rond a suffi.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Tout petit, tout serré. Une toute petite bulle quitte le savon. Nina souffle à peine, sans prendre le vent. Le tilleul se tait, plus loin, tout seul. La larme de bronze prend le petit rond. Le petit rond n'a pas volé. Tu restes, bulle. Une goutte de savon brille, minuscule. Le petit rond a suffi. [pause]</t>
+          <t>Tout petit, tout serré. Une toute petite bulle quitte le savon. Nina souffle à peine, sans prendre le vent. Le tilleul se tait, plus loin, tout seul. La larme de bronze prend le petit rond. Le petit rond n'a pas volé. Tu restes, bulle. Une goutte de savon brille, minuscule. Elle prend une seule goutte, pas deux. Une toute petite, pour la larme. Le petit rond a suffi. [pause]</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr"/>
@@ -11851,6 +11910,8 @@
 papa|Le petit rond n'a pas volé.
 enfant-f|Tu restes, bulle.
 narrateur|Une goutte de savon brille, minuscule.
+narrateur|Elle prend une seule goutte, pas deux.
+enfant-f|Une toute petite, pour la larme.
 maman|Le petit rond a suffi.</t>
         </is>
       </c>
@@ -12068,17 +12129,17 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Nina lève d'abord la coupelle, bien à plat. Le savon va dormir dedans. Pas trop d'eau, juste un miroir. Le rond tremble, puis s'arrête. Elle penche le bol vers ses lèvres. Pas maintenant, le bronze est loin. Il glisse le bâton et le savon contre elle. Le gravier reste vide, derrière eux. Coupelle, je te porte. Un cercle de savon brille au fond. La coupelle est prête, on avance. Sans verser, tout droit.</t>
+          <t>Nina lève d'abord la coupelle, bien à plat. Le savon va dormir dedans. Pas trop d'eau, juste un miroir. Le rond tremble, puis s'arrête. Elle penche le bol vers ses lèvres. Pas maintenant, le bronze est loin. Il glisse le bâton et le savon contre elle. Le gravier reste vide, derrière eux. Coupelle, je te porte. Un cercle de savon brille au fond. La coupelle est prête, on avance. Sans verser, tout droit. Elle veut souffler dans le miroir, trop tôt. Le nez d'abord, pas le bol.</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nina lève d'abord la &lt;emphasis level="moderate"&gt;coupelle&lt;/emphasis&gt;, bien à plat. Le savon va dormir dedans. Pas trop d'eau, juste un miroir. Le rond tremble, puis s'arrête. Elle penche le bol vers ses lèvres. Pas maintenant, le bronze est loin. Il glisse le bâton et le savon contre elle. Le gravier reste vide, derrière eux. Coupelle, je te porte. Un cercle de savon brille au fond. La coupelle est prête, on avance. Sans verser, tout droit.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nina lève d'abord la &lt;emphasis level="moderate"&gt;coupelle&lt;/emphasis&gt;, bien à plat. Le savon va dormir dedans. Pas trop d'eau, juste un miroir. Le rond tremble, puis s'arrête. Elle penche le bol vers ses lèvres. Pas maintenant, le bronze est loin. Il glisse le bâton et le savon contre elle. Le gravier reste vide, derrière eux. Coupelle, je te porte. Un cercle de savon brille au fond. La coupelle est prête, on avance. Sans verser, tout droit. Elle veut souffler dans le miroir, trop tôt. Le nez d'abord, pas le bol.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Nina lève d'abord la &lt;emphasis&gt;coupelle&lt;/emphasis&gt;, bien à plat. Le savon va dormir dedans. Pas trop d'eau, juste un miroir. Le rond tremble, puis s'arrête. Elle penche le bol vers ses lèvres. Pas maintenant, le bronze est loin. Il glisse le bâton et le savon contre elle. Le gravier reste vide, derrière eux. Coupelle, je te porte. Un cercle de savon brille au fond. La coupelle est prête, on avance. Sans verser, tout droit. [pause]</t>
+          <t>Nina lève d'abord la &lt;emphasis&gt;coupelle&lt;/emphasis&gt;, bien à plat. Le savon va dormir dedans. Pas trop d'eau, juste un miroir. Le rond tremble, puis s'arrête. Elle penche le bol vers ses lèvres. Pas maintenant, le bronze est loin. Il glisse le bâton et le savon contre elle. Le gravier reste vide, derrière eux. Coupelle, je te porte. Un cercle de savon brille au fond. La coupelle est prête, on avance. Sans verser, tout droit. Elle veut souffler dans le miroir, trop tôt. Le nez d'abord, pas le bol. [pause]</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr"/>
@@ -12223,7 +12284,9 @@
 enfant-f|Coupelle, je te porte.
 narrateur|Un cercle de savon brille au fond.
 papa|La coupelle est prête, on avance.
-maman|Sans verser, tout droit.</t>
+maman|Sans verser, tout droit.
+narrateur|Elle veut souffler dans le miroir, trop tôt.
+papa|Le nez d'abord, pas le bol.</t>
         </is>
       </c>
       <c r="AX60" t="inlineStr">
@@ -12443,17 +12506,17 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>La coupelle reste plate, contre son ventre. Le savon ne verse pas. Le rond sent le tilleul, un peu. On avance, tous les trois ? Oui. Le miroir de savon attend, plat. On marche, sans se presser.</t>
+          <t>La coupelle reste plate, contre son ventre. Le savon ne verse pas. Le rond sent le tilleul, un peu. On avance, tous les trois ? Oui. Le miroir de savon attend, plat. On marche, sans se presser. Le bol chauffe un peu, contre le pull. Le bâton et le savon sont avec toi.</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;coupelle&lt;/emphasis&gt; reste plate, contre son ventre. Le savon ne verse pas. Le rond sent le tilleul, un peu. On avance, tous les trois ? Oui. Le miroir de savon attend, plat. On marche, sans se presser.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;coupelle&lt;/emphasis&gt; reste plate, contre son ventre. Le savon ne verse pas. Le rond sent le tilleul, un peu. On avance, tous les trois ? Oui. Le miroir de savon attend, plat. On marche, sans se presser. Le bol chauffe un peu, contre le pull. Le bâton et le savon sont avec toi.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>La &lt;emphasis&gt;coupelle&lt;/emphasis&gt; reste plate, contre son ventre. Le savon ne verse pas. Le rond sent le tilleul, un peu. On avance, tous les trois ? Oui. Le miroir de savon attend, plat. On marche, sans se presser. [pause]</t>
+          <t>La &lt;emphasis&gt;coupelle&lt;/emphasis&gt; reste plate, contre son ventre. Le savon ne verse pas. Le rond sent le tilleul, un peu. On avance, tous les trois ? Oui. Le miroir de savon attend, plat. On marche, sans se presser. Le bol chauffe un peu, contre le pull. Le bâton et le savon sont avec toi. [pause]</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr"/>
@@ -12593,7 +12656,9 @@
 papa|On avance, tous les trois ?
 enfant-f|Oui.
 narrateur|Le miroir de savon attend, plat.
-papa|On marche, sans se presser.</t>
+papa|On marche, sans se presser.
+narrateur|Le bol chauffe un peu, contre le pull.
+maman|Le bâton et le savon sont avec toi.</t>
         </is>
       </c>
       <c r="AX62" t="inlineStr">
@@ -12625,17 +12690,17 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>La coupelle appuie contre son ventre. Devant, l'allée soulève trop de poussière. Le socle, lui, brûle au soleil. Sous le tilleul, les feuilles claquent. Nina, tu vas où ?</t>
+          <t>La coupelle appuie contre son ventre. Devant, l'allée soulève trop de poussière. Le socle, lui, brûle au soleil. Sous le tilleul, les feuilles claquent. Nina, tu vas où ? La larme attend, sur le nez.</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;La coupelle appuie contre son ventre. Devant, l'allée soulève trop de poussière. Le socle, lui, brûle au soleil. Sous le tilleul, les feuilles claquent. Nina, tu vas où ?&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;La coupelle appuie contre son ventre. Devant, l'allée soulève trop de poussière. Le socle, lui, brûle au soleil. Sous le tilleul, les feuilles claquent. Nina, tu vas où ? La larme attend, sur le nez.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;La coupelle appuie contre son ventre. Devant, l'allée soulève trop de poussière. Le socle, lui, brûle au soleil. Sous le tilleul, les feuilles claquent. Nina, tu vas où ?&lt;/slow&gt; [long-pause]</t>
+          <t>&lt;slow&gt;La coupelle appuie contre son ventre. Devant, l'allée soulève trop de poussière. Le socle, lui, brûle au soleil. Sous le tilleul, les feuilles claquent. Nina, tu vas où ? La larme attend, sur le nez.&lt;/slow&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr"/>
@@ -12797,7 +12862,8 @@
 narrateur|Devant, l'allée soulève trop de poussière.
 narrateur|Le socle, lui, brûle au soleil.
 narrateur|Sous le tilleul, les feuilles claquent.
-papa|Nina, tu vas où ?</t>
+papa|Nina, tu vas où ?
+maman|La larme attend, sur le nez.</t>
         </is>
       </c>
     </row>
@@ -12824,17 +12890,17 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Contre son ventre, la coupelle reste bien plate. Le gravier de l'allée saute sous les pas. Le rond se plisse, trop agité, trop gris. Ma bulle a crevé ! Le sourire de Nina disparaît. Dans sa poitrine, l'envie et la peur se bousculent. Ici, ça n'arrête pas. Papa s'accroupit, à la même hauteur. Elle penche le bol, trop vite. Un pas tardif soulève la poussière, gris. Pas maintenant. La larme de bronze est grise, trop. Tu vois comment, Nina ?</t>
+          <t>Contre son ventre, la coupelle reste bien plate. Le gravier de l'allée saute sous les pas. Le rond se plisse, trop agité, trop gris. Ma bulle a crevé ! Le sourire de Nina disparaît. Dans sa poitrine, l'envie et la peur se bousculent. Ici, ça n'arrête pas. Papa s'accroupit, à la même hauteur. Elle penche le bol, trop vite. Un pas tardif soulève la poussière, gris. Pas maintenant. La larme de bronze est grise, trop. Tu vois comment, Nina ? Nina serre la coupelle, sans verser. Alors on fait quoi ?</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Contre son ventre, la coupelle reste bien plate. Le gravier de l'&lt;emphasis level="moderate"&gt;allée&lt;/emphasis&gt; saute sous les pas. Le rond se plisse, trop agité, trop gris. Ma bulle a crevé ! Le sourire de Nina disparaît. Dans sa poitrine, l'envie et la peur se bousculent. Ici, ça n'arrête pas. Papa s'accroupit, à la même hauteur. Elle penche le bol, trop vite. Un pas tardif soulève la poussière, gris. Pas maintenant. La larme de bronze est grise, trop. Tu vois comment, Nina ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Contre son ventre, la coupelle reste bien plate. Le gravier de l'&lt;emphasis level="moderate"&gt;allée&lt;/emphasis&gt; saute sous les pas. Le rond se plisse, trop agité, trop gris. Ma bulle a crevé ! Le sourire de Nina disparaît. Dans sa poitrine, l'envie et la peur se bousculent. Ici, ça n'arrête pas. Papa s'accroupit, à la même hauteur. Elle penche le bol, trop vite. Un pas tardif soulève la poussière, gris. Pas maintenant. La larme de bronze est grise, trop. Tu vois comment, Nina ? Nina serre la coupelle, sans verser. Alors on fait quoi ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Contre son ventre, la coupelle reste bien plate. Le gravier de l'&lt;emphasis&gt;allée&lt;/emphasis&gt; saute sous les pas. Le rond se plisse, trop agité, trop gris. Ma bulle a crevé ! Le sourire de Nina disparaît. Dans sa poitrine, l'envie et la peur se bousculent. Ici, ça n'arrête pas. Papa s'accroupit, à la même hauteur. Elle penche le bol, trop vite. Un pas tardif soulève la poussière, gris. Pas maintenant. La larme de bronze est grise, trop. Tu vois comment, Nina ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Contre son ventre, la coupelle reste bien plate. Le gravier de l'&lt;emphasis&gt;allée&lt;/emphasis&gt; saute sous les pas. Le rond se plisse, trop agité, trop gris. Ma bulle a crevé ! Le sourire de Nina disparaît. Dans sa poitrine, l'envie et la peur se bousculent. Ici, ça n'arrête pas. Papa s'accroupit, à la même hauteur. Elle penche le bol, trop vite. Un pas tardif soulève la poussière, gris. Pas maintenant. La larme de bronze est grise, trop. Tu vois comment, Nina ? Nina serre la coupelle, sans verser. Alors on fait quoi ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr"/>
@@ -12984,7 +13050,9 @@
 narrateur|Un pas tardif soulève la poussière, gris.
 enfant-f|Pas maintenant.
 narrateur|La larme de bronze est grise, trop.
-maman|Tu vois comment, Nina ?</t>
+maman|Tu vois comment, Nina ?
+narrateur|Nina serre la coupelle, sans verser.
+enfant-f|Alors on fait quoi ?</t>
         </is>
       </c>
       <c r="AX64" t="inlineStr">
@@ -13212,17 +13280,17 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>On attend les pas. Nina tient la coupelle, sans verser. Le gravier se tait, une fois, puis plus. La larme de bronze redevient sombre, nette. Tu peux partir, maintenant. Plate, la coupelle attend, sans verser. Les pas se sont tus, là. Le miroir file, rond, vers la larme. Tu as laissé le gravier se taire.</t>
+          <t>On attend les pas. Nina tient la coupelle, sans verser. Le gravier se tait, une fois, puis plus. La larme de bronze redevient sombre, nette. Tu peux partir, maintenant. Plate, la coupelle attend, sans verser. Les pas se sont tus, là. Le miroir file, rond, vers la larme. Elle garde le bol plat, sans le pencher. Le miroir, je le tiens droit. Tu as laissé le gravier se taire.</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend les &lt;emphasis level="moderate"&gt;pas&lt;/emphasis&gt;. Nina tient la coupelle, sans verser. Le gravier se tait, une fois, puis plus. La larme de bronze redevient sombre, nette. Tu peux partir, maintenant. Plate, la coupelle attend, sans verser. Les pas se sont tus, là. Le miroir file, rond, vers la larme. Tu as laissé le gravier se taire.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend les &lt;emphasis level="moderate"&gt;pas&lt;/emphasis&gt;. Nina tient la coupelle, sans verser. Le gravier se tait, une fois, puis plus. La larme de bronze redevient sombre, nette. Tu peux partir, maintenant. Plate, la coupelle attend, sans verser. Les pas se sont tus, là. Le miroir file, rond, vers la larme. Elle garde le bol plat, sans le pencher. Le miroir, je le tiens droit. Tu as laissé le gravier se taire.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>On attend les &lt;emphasis&gt;pas&lt;/emphasis&gt;. Nina tient la coupelle, sans verser. Le gravier se tait, une fois, puis plus. La larme de bronze redevient sombre, nette. Tu peux partir, maintenant. Plate, la coupelle attend, sans verser. Les pas se sont tus, là. Le miroir file, rond, vers la larme. Tu as laissé le gravier se taire. [pause]</t>
+          <t>On attend les &lt;emphasis&gt;pas&lt;/emphasis&gt;. Nina tient la coupelle, sans verser. Le gravier se tait, une fois, puis plus. La larme de bronze redevient sombre, nette. Tu peux partir, maintenant. Plate, la coupelle attend, sans verser. Les pas se sont tus, là. Le miroir file, rond, vers la larme. Elle garde le bol plat, sans le pencher. Le miroir, je le tiens droit. Tu as laissé le gravier se taire. [pause]</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr"/>
@@ -13364,6 +13432,8 @@
 narrateur|Plate, la coupelle attend, sans verser.
 papa|Les pas se sont tus, là.
 narrateur|Le miroir file, rond, vers la larme.
+narrateur|Elle garde le bol plat, sans le pencher.
+enfant-f|Le miroir, je le tiens droit.
 maman|Tu as laissé le gravier se taire.</t>
         </is>
       </c>
@@ -13581,17 +13651,17 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Plus bas, d'abord. Elle baisse la coupelle, loin de la poussière. Nina s'accroupit, les genoux au gravier. L'air est plus doux, près de l'herbe. La larme de bronze se voit d'en bas. Ici, tu ne crèves plus. Tu as vu l'herbe, avant. Le rond de savon attend, plat, bas. Près du sol, ça tenait mieux.</t>
+          <t>Plus bas, d'abord. Elle baisse la coupelle, loin de la poussière. Nina s'accroupit, les genoux au gravier. L'air est plus doux, près de l'herbe. La larme de bronze se voit d'en bas. Ici, tu ne crèves plus. Tu as vu l'herbe, avant. Le rond de savon attend, plat, bas. Elle pose le bol sur l'herbe, à plat. Le sol tient le miroir. Près du sol, ça tenait mieux.</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Plus bas, d'abord. Elle baisse la coupelle, loin de la poussière. Nina s'accroupit, les genoux au gravier. L'air est plus doux, près de l'herbe. La larme de bronze se voit d'en bas. Ici, tu ne crèves plus. Tu as vu l'herbe, avant. Le rond de savon attend, plat, bas. Près du sol, ça tenait mieux.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Plus bas, d'abord. Elle baisse la coupelle, loin de la poussière. Nina s'accroupit, les genoux au gravier. L'air est plus doux, près de l'herbe. La larme de bronze se voit d'en bas. Ici, tu ne crèves plus. Tu as vu l'herbe, avant. Le rond de savon attend, plat, bas. Elle pose le bol sur l'herbe, à plat. Le sol tient le miroir. Près du sol, ça tenait mieux.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Plus bas, d'abord. Elle baisse la coupelle, loin de la poussière. Nina s'accroupit, les genoux au gravier. L'air est plus doux, près de l'herbe. La larme de bronze se voit d'en bas. Ici, tu ne crèves plus. Tu as vu l'herbe, avant. Le rond de savon attend, plat, bas. Près du sol, ça tenait mieux. [pause]</t>
+          <t>Plus bas, d'abord. Elle baisse la coupelle, loin de la poussière. Nina s'accroupit, les genoux au gravier. L'air est plus doux, près de l'herbe. La larme de bronze se voit d'en bas. Ici, tu ne crèves plus. Tu as vu l'herbe, avant. Le rond de savon attend, plat, bas. Elle pose le bol sur l'herbe, à plat. Le sol tient le miroir. Près du sol, ça tenait mieux. [pause]</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr"/>
@@ -13733,6 +13803,8 @@
 enfant-f|Ici, tu ne crèves plus.
 papa|Tu as vu l'herbe, avant.
 narrateur|Le rond de savon attend, plat, bas.
+narrateur|Elle pose le bol sur l'herbe, à plat.
+enfant-f|Le sol tient le miroir.
 maman|Près du sol, ça tenait mieux.</t>
         </is>
       </c>
@@ -13950,17 +14022,17 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Au bord, tout petit. Elle glisse la coupelle vers le bord d'herbe. L'herbe tient, sans laisser la poussière. Nina penche le bol, une seule fois. La larme de bronze luit, hors de l'allée. Le bord n'a pas soulevé. Tu es à l'abri. Le rond monte, lent, jusqu'au nez. Tu as dit ça tout bas.</t>
+          <t>Au bord, tout petit. Elle glisse la coupelle vers le bord d'herbe. L'herbe tient, sans laisser la poussière. Nina penche le bol, une seule fois. La larme de bronze luit, hors de l'allée. Le bord n'a pas soulevé. Tu es à l'abri. Le rond monte, lent, jusqu'au nez. Elle glisse le bol sur l'herbe, hors du gris. L'herbe, pas le gravier. Tu as dit ça tout bas.</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Au &lt;emphasis level="moderate"&gt;bord&lt;/emphasis&gt;, tout petit. Elle glisse la coupelle vers le bord d'herbe. L'herbe tient, sans laisser la poussière. Nina penche le bol, une seule fois. La larme de bronze luit, hors de l'allée. Le bord n'a pas soulevé. Tu es à l'abri. Le rond monte, lent, jusqu'au nez. Tu as dit ça tout bas.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Au &lt;emphasis level="moderate"&gt;bord&lt;/emphasis&gt;, tout petit. Elle glisse la coupelle vers le bord d'herbe. L'herbe tient, sans laisser la poussière. Nina penche le bol, une seule fois. La larme de bronze luit, hors de l'allée. Le bord n'a pas soulevé. Tu es à l'abri. Le rond monte, lent, jusqu'au nez. Elle glisse le bol sur l'herbe, hors du gris. L'herbe, pas le gravier. Tu as dit ça tout bas.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>Au &lt;emphasis&gt;bord&lt;/emphasis&gt;, tout petit. Elle glisse la coupelle vers le bord d'herbe. L'herbe tient, sans laisser la poussière. Nina penche le bol, une seule fois. La larme de bronze luit, hors de l'allée. Le bord n'a pas soulevé. Tu es à l'abri. Le rond monte, lent, jusqu'au nez. Tu as dit ça tout bas. [pause]</t>
+          <t>Au &lt;emphasis&gt;bord&lt;/emphasis&gt;, tout petit. Elle glisse la coupelle vers le bord d'herbe. L'herbe tient, sans laisser la poussière. Nina penche le bol, une seule fois. La larme de bronze luit, hors de l'allée. Le bord n'a pas soulevé. Tu es à l'abri. Le rond monte, lent, jusqu'au nez. Elle glisse le bol sur l'herbe, hors du gris. L'herbe, pas le gravier. Tu as dit ça tout bas. [pause]</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr"/>
@@ -14102,6 +14174,8 @@
 papa|Le bord n'a pas soulevé.
 enfant-f|Tu es à l'abri.
 narrateur|Le rond monte, lent, jusqu'au nez.
+narrateur|Elle glisse le bol sur l'herbe, hors du gris.
+enfant-f|L'herbe, pas le gravier.
 maman|Tu as dit ça tout bas.</t>
         </is>
       </c>
@@ -14319,17 +14393,17 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Contre son ventre, la coupelle reste bien plate. Le bronze tient tout le soleil. Le rond tremble, trop chaud, trop mince. Le nez brûle trop ! La bulle touche, puis crève tout de suite. Il ne reste rien sur le bronze. Ici, c'est trop chaud. Papa s'accroupit, à la même hauteur. Un nuage passe, et Nina penche le bol. Le soleil revient, net, sur la larme. Pas maintenant. La larme de bronze est sèche, trop pâle. Tu vois comment, Nina ?</t>
+          <t>Contre son ventre, la coupelle reste bien plate. Le bronze tient tout le soleil. Le rond tremble, trop chaud, trop mince. Le nez brûle trop ! La bulle touche, puis crève tout de suite. Il ne reste rien sur le bronze. Ici, c'est trop chaud. Papa s'accroupit, à la même hauteur. Un nuage passe, et Nina penche le bol. Le soleil revient, net, sur la larme. Pas maintenant. La larme de bronze est sèche, trop pâle. Tu vois comment, Nina ? Nina serre la coupelle, sans verser. Alors on fait quoi ?</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Contre son ventre, la coupelle reste bien plate. Le bronze tient tout le soleil. Le rond tremble, trop chaud, trop mince. Le nez brûle trop ! La bulle touche, puis crève tout de suite. Il ne reste rien sur le bronze. Ici, c'est trop chaud. Papa s'accroupit, à la même hauteur. Un nuage passe, et Nina penche le bol. Le soleil revient, net, sur la larme. Pas maintenant. La larme de bronze est sèche, trop pâle. Tu vois comment, Nina ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Contre son ventre, la coupelle reste bien plate. Le bronze tient tout le soleil. Le rond tremble, trop chaud, trop mince. Le nez brûle trop ! La bulle touche, puis crève tout de suite. Il ne reste rien sur le bronze. Ici, c'est trop chaud. Papa s'accroupit, à la même hauteur. Un nuage passe, et Nina penche le bol. Le soleil revient, net, sur la larme. Pas maintenant. La larme de bronze est sèche, trop pâle. Tu vois comment, Nina ? Nina serre la coupelle, sans verser. Alors on fait quoi ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Contre son ventre, la coupelle reste bien plate. Le bronze tient tout le soleil. Le rond tremble, trop chaud, trop mince. Le nez brûle trop ! La bulle touche, puis crève tout de suite. Il ne reste rien sur le bronze. Ici, c'est trop chaud. Papa s'accroupit, à la même hauteur. Un nuage passe, et Nina penche le bol. Le soleil revient, net, sur la larme. Pas maintenant. La larme de bronze est sèche, trop pâle. Tu vois comment, Nina ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Contre son ventre, la coupelle reste bien plate. Le bronze tient tout le soleil. Le rond tremble, trop chaud, trop mince. Le nez brûle trop ! La bulle touche, puis crève tout de suite. Il ne reste rien sur le bronze. Ici, c'est trop chaud. Papa s'accroupit, à la même hauteur. Un nuage passe, et Nina penche le bol. Le soleil revient, net, sur la larme. Pas maintenant. La larme de bronze est sèche, trop pâle. Tu vois comment, Nina ? Nina serre la coupelle, sans verser. Alors on fait quoi ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr"/>
@@ -14479,7 +14553,9 @@
 narrateur|Le soleil revient, net, sur la larme.
 enfant-f|Pas maintenant.
 narrateur|La larme de bronze est sèche, trop pâle.
-maman|Tu vois comment, Nina ?</t>
+maman|Tu vois comment, Nina ?
+narrateur|Nina serre la coupelle, sans verser.
+enfant-f|Alors on fait quoi ?</t>
         </is>
       </c>
       <c r="AX72" t="inlineStr">
@@ -14707,17 +14783,17 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>On attend l'ombre. Une ombre de tilleul glisse sur le nez. Sous l'ombre, la coupelle ne fume plus. Le bronze se tait, puis se refroidit. La larme de bronze redevient sombre, froide. Le nez est redevenu doux. Maintenant, tu me vois. Plate, la coupelle attend, sans verser. Tu as laissé l'ombre arriver.</t>
+          <t>On attend l'ombre. Une ombre de tilleul glisse sur le nez. Sous l'ombre, la coupelle ne fume plus. Le bronze se tait, puis se refroidit. La larme de bronze redevient sombre, froide. Le nez est redevenu doux. Maintenant, tu me vois. Plate, la coupelle attend, sans verser. Elle attend que le bol ne fume plus. Le miroir est froid, maintenant. Tu as laissé l'ombre arriver.</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend l'&lt;emphasis level="moderate"&gt;ombre&lt;/emphasis&gt;. Une ombre de tilleul glisse sur le nez. Sous l'ombre, la coupelle ne fume plus. Le bronze se tait, puis se refroidit. La larme de bronze redevient sombre, froide. Le nez est redevenu doux. Maintenant, tu me vois. Plate, la coupelle attend, sans verser. Tu as laissé l'ombre arriver.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend l'&lt;emphasis level="moderate"&gt;ombre&lt;/emphasis&gt;. Une ombre de tilleul glisse sur le nez. Sous l'ombre, la coupelle ne fume plus. Le bronze se tait, puis se refroidit. La larme de bronze redevient sombre, froide. Le nez est redevenu doux. Maintenant, tu me vois. Plate, la coupelle attend, sans verser. Elle attend que le bol ne fume plus. Le miroir est froid, maintenant. Tu as laissé l'ombre arriver.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>On attend l'&lt;emphasis&gt;ombre&lt;/emphasis&gt;. Une ombre de tilleul glisse sur le nez. Sous l'ombre, la coupelle ne fume plus. Le bronze se tait, puis se refroidit. La larme de bronze redevient sombre, froide. Le nez est redevenu doux. Maintenant, tu me vois. Plate, la coupelle attend, sans verser. Tu as laissé l'ombre arriver. [pause]</t>
+          <t>On attend l'&lt;emphasis&gt;ombre&lt;/emphasis&gt;. Une ombre de tilleul glisse sur le nez. Sous l'ombre, la coupelle ne fume plus. Le bronze se tait, puis se refroidit. La larme de bronze redevient sombre, froide. Le nez est redevenu doux. Maintenant, tu me vois. Plate, la coupelle attend, sans verser. Elle attend que le bol ne fume plus. Le miroir est froid, maintenant. Tu as laissé l'ombre arriver. [pause]</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr"/>
@@ -14859,6 +14935,8 @@
 maman|Le nez est redevenu doux.
 enfant-f|Maintenant, tu me vois.
 narrateur|Plate, la coupelle attend, sans verser.
+narrateur|Elle attend que le bol ne fume plus.
+enfant-f|Le miroir est froid, maintenant.
 papa|Tu as laissé l'ombre arriver.</t>
         </is>
       </c>
@@ -15076,17 +15154,17 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>L'oiseau, d'abord, il est plus frais. Elle pose d'abord le rond sur l'oiseau. L'oiseau de bronze est à l'ombre, lui. Le rond glisse, lent, vers la larme. Le rond de savon attend, court. Tu n'as pas soufflé trop fort. C'est pour toi. La larme de bronze reçoit le rond, entier. L'oiseau était plus frais, tu as vu.</t>
+          <t>L'oiseau, d'abord, il est plus frais. Elle pose d'abord le rond sur l'oiseau. L'oiseau de bronze est à l'ombre, lui. Le rond glisse, lent, vers la larme. Le rond de savon attend, court. Tu n'as pas soufflé trop fort. C'est pour toi. La larme de bronze reçoit le rond, entier. Elle penche le bol vers le bec, d'abord. Le bec, puis la larme. L'oiseau était plus frais, tu as vu.</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;L'&lt;emphasis level="moderate"&gt;oiseau&lt;/emphasis&gt;, d'abord, il est plus frais. Elle pose d'abord le rond sur l'oiseau. L'oiseau de bronze est à l'ombre, lui. Le rond glisse, lent, vers la larme. Le rond de savon attend, court. Tu n'as pas soufflé trop fort. C'est pour toi. La larme de bronze reçoit le rond, entier. L'oiseau était plus frais, tu as vu.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;L'&lt;emphasis level="moderate"&gt;oiseau&lt;/emphasis&gt;, d'abord, il est plus frais. Elle pose d'abord le rond sur l'oiseau. L'oiseau de bronze est à l'ombre, lui. Le rond glisse, lent, vers la larme. Le rond de savon attend, court. Tu n'as pas soufflé trop fort. C'est pour toi. La larme de bronze reçoit le rond, entier. Elle penche le bol vers le bec, d'abord. Le bec, puis la larme. L'oiseau était plus frais, tu as vu.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>L'&lt;emphasis&gt;oiseau&lt;/emphasis&gt;, d'abord, il est plus frais. Elle pose d'abord le rond sur l'oiseau. L'oiseau de bronze est à l'ombre, lui. Le rond glisse, lent, vers la larme. Le rond de savon attend, court. Tu n'as pas soufflé trop fort. C'est pour toi. La larme de bronze reçoit le rond, entier. L'oiseau était plus frais, tu as vu. [pause]</t>
+          <t>L'&lt;emphasis&gt;oiseau&lt;/emphasis&gt;, d'abord, il est plus frais. Elle pose d'abord le rond sur l'oiseau. L'oiseau de bronze est à l'ombre, lui. Le rond glisse, lent, vers la larme. Le rond de savon attend, court. Tu n'as pas soufflé trop fort. C'est pour toi. La larme de bronze reçoit le rond, entier. Elle penche le bol vers le bec, d'abord. Le bec, puis la larme. L'oiseau était plus frais, tu as vu. [pause]</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr"/>
@@ -15228,6 +15306,8 @@
 papa|Tu n'as pas soufflé trop fort.
 enfant-f|C'est pour toi.
 narrateur|La larme de bronze reçoit le rond, entier.
+narrateur|Elle penche le bol vers le bec, d'abord.
+enfant-f|Le bec, puis la larme.
 maman|L'oiseau était plus frais, tu as vu.</t>
         </is>
       </c>
@@ -15445,17 +15525,17 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Tout près, contre le bronze. Nina se glisse contre le socle. Tout près, la coupelle n'a plus d'air chaud. La bulle n'a plus à voyager trop loin. La larme de bronze est là, à un souffle. Tu t'es mise tout près, contre le nez. Le nez est là. Plate, la coupelle attend, sans verser. Tu t'es mise tout contre.</t>
+          <t>Tout près, contre le bronze. Nina se glisse contre le socle. Tout près, la coupelle n'a plus d'air chaud. La bulle n'a plus à voyager trop loin. La larme de bronze est là, à un souffle. Tu t'es mise tout près, contre le nez. Le nez est là. Plate, la coupelle attend, sans verser. Elle lève le bol jusqu'au nez, tout près. Le miroir touche presque. Tu t'es mise tout contre.</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Tout près, contre le bronze. Nina se glisse contre le socle. Tout près, la coupelle n'a plus d'air chaud. La bulle n'a plus à voyager trop loin. La larme de bronze est là, à un souffle. Tu t'es mise &lt;emphasis level="moderate"&gt;tout près&lt;/emphasis&gt;, contre le nez. Le nez est là. Plate, la coupelle attend, sans verser. Tu t'es mise tout contre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Tout près, contre le bronze. Nina se glisse contre le socle. Tout près, la coupelle n'a plus d'air chaud. La bulle n'a plus à voyager trop loin. La larme de bronze est là, à un souffle. Tu t'es mise &lt;emphasis level="moderate"&gt;tout près&lt;/emphasis&gt;, contre le nez. Le nez est là. Plate, la coupelle attend, sans verser. Elle lève le bol jusqu'au nez, tout près. Le miroir touche presque. Tu t'es mise tout contre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>Tout près, contre le bronze. Nina se glisse contre le socle. Tout près, la coupelle n'a plus d'air chaud. La bulle n'a plus à voyager trop loin. La larme de bronze est là, à un souffle. Tu t'es mise &lt;emphasis&gt;tout près&lt;/emphasis&gt;, contre le nez. Le nez est là. Plate, la coupelle attend, sans verser. Tu t'es mise tout contre. [pause]</t>
+          <t>Tout près, contre le bronze. Nina se glisse contre le socle. Tout près, la coupelle n'a plus d'air chaud. La bulle n'a plus à voyager trop loin. La larme de bronze est là, à un souffle. Tu t'es mise &lt;emphasis&gt;tout près&lt;/emphasis&gt;, contre le nez. Le nez est là. Plate, la coupelle attend, sans verser. Elle lève le bol jusqu'au nez, tout près. Le miroir touche presque. Tu t'es mise tout contre. [pause]</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr"/>
@@ -15597,6 +15677,8 @@
 papa|Tu t'es mise tout près, contre le nez.
 enfant-f|Le nez est là.
 narrateur|Plate, la coupelle attend, sans verser.
+narrateur|Elle lève le bol jusqu'au nez, tout près.
+enfant-f|Le miroir touche presque.
 maman|Tu t'es mise tout contre.</t>
         </is>
       </c>
@@ -15814,17 +15896,17 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Contre son ventre, la coupelle reste bien plate. Le tilleul agite ses feuilles, trop vite. Le rond se plie, trop poussé par les feuilles. Le vent prend tout ! Une feuille claque, puis une autre. La bulle part de travers, trop loin. Ici, ça souffle trop. Papa s'accroupit, à la même hauteur. Les feuilles se taisent, un instant. Nina penche le bol, trop tôt. Un souffle tardif plie le miroir. Pas maintenant. La larme de bronze reste nette, elle. Tu vois comment, Nina ?</t>
+          <t>Contre son ventre, la coupelle reste bien plate. Le tilleul agite ses feuilles, trop vite. Le rond se plie, trop poussé par les feuilles. Le vent prend tout ! Une feuille claque, puis une autre. La bulle part de travers, trop loin. Ici, ça souffle trop. Papa s'accroupit, à la même hauteur. Les feuilles se taisent, un instant. Nina penche le bol, trop tôt. Un souffle tardif plie le miroir. Pas maintenant. La larme de bronze reste nette, elle. Tu vois comment, Nina ? Nina serre la coupelle, sans verser. Alors on fait quoi ?</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Contre son ventre, la coupelle reste bien plate. Le &lt;emphasis level="moderate"&gt;tilleul&lt;/emphasis&gt; agite ses feuilles, trop vite. Le rond se plie, trop poussé par les feuilles. Le vent prend tout ! Une feuille claque, puis une autre. La bulle part de travers, trop loin. Ici, ça souffle trop. Papa s'accroupit, à la même hauteur. Les feuilles se taisent, un instant. Nina penche le bol, trop tôt. Un souffle tardif plie le miroir. Pas maintenant. La larme de bronze reste nette, elle. Tu vois comment, Nina ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Contre son ventre, la coupelle reste bien plate. Le &lt;emphasis level="moderate"&gt;tilleul&lt;/emphasis&gt; agite ses feuilles, trop vite. Le rond se plie, trop poussé par les feuilles. Le vent prend tout ! Une feuille claque, puis une autre. La bulle part de travers, trop loin. Ici, ça souffle trop. Papa s'accroupit, à la même hauteur. Les feuilles se taisent, un instant. Nina penche le bol, trop tôt. Un souffle tardif plie le miroir. Pas maintenant. La larme de bronze reste nette, elle. Tu vois comment, Nina ? Nina serre la coupelle, sans verser. Alors on fait quoi ?&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Contre son ventre, la coupelle reste bien plate. Le &lt;emphasis&gt;tilleul&lt;/emphasis&gt; agite ses feuilles, trop vite. Le rond se plie, trop poussé par les feuilles. Le vent prend tout ! Une feuille claque, puis une autre. La bulle part de travers, trop loin. Ici, ça souffle trop. Papa s'accroupit, à la même hauteur. Les feuilles se taisent, un instant. Nina penche le bol, trop tôt. Un souffle tardif plie le miroir. Pas maintenant. La larme de bronze reste nette, elle. Tu vois comment, Nina ?&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Contre son ventre, la coupelle reste bien plate. Le &lt;emphasis&gt;tilleul&lt;/emphasis&gt; agite ses feuilles, trop vite. Le rond se plie, trop poussé par les feuilles. Le vent prend tout ! Une feuille claque, puis une autre. La bulle part de travers, trop loin. Ici, ça souffle trop. Papa s'accroupit, à la même hauteur. Les feuilles se taisent, un instant. Nina penche le bol, trop tôt. Un souffle tardif plie le miroir. Pas maintenant. La larme de bronze reste nette, elle. Tu vois comment, Nina ? Nina serre la coupelle, sans verser. Alors on fait quoi ?&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr"/>
@@ -15975,7 +16057,9 @@
 narrateur|Un souffle tardif plie le miroir.
 enfant-f|Pas maintenant.
 narrateur|La larme de bronze reste nette, elle.
-maman|Tu vois comment, Nina ?</t>
+maman|Tu vois comment, Nina ?
+narrateur|Nina serre la coupelle, sans verser.
+enfant-f|Alors on fait quoi ?</t>
         </is>
       </c>
       <c r="AX80" t="inlineStr">
@@ -16203,17 +16287,17 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>On attend les feuilles, d'abord. Elle tient la coupelle, puis attend les feuilles. Les feuilles vont, reviennent, puis se taisent. L'air redevient un seul souffle, net. La larme de bronze ne bouge plus, du tout. Le tilleul n'a plus claqué. Maintenant, tu peux rester. Plate, la coupelle attend, sans verser. Tu as laissé les feuilles finir.</t>
+          <t>On attend les feuilles, d'abord. Elle tient la coupelle, puis attend les feuilles. Les feuilles vont, reviennent, puis se taisent. L'air redevient un seul souffle, net. La larme de bronze ne bouge plus, du tout. Le tilleul n'a plus claqué. Maintenant, tu peux rester. Plate, la coupelle attend, sans verser. Elle couvre le bol avec sa paume. Ma main garde le miroir. Tu as laissé les feuilles finir.</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend les &lt;emphasis level="moderate"&gt;feuilles&lt;/emphasis&gt;, d'abord. Elle tient la coupelle, puis attend les feuilles. Les feuilles vont, reviennent, puis se taisent. L'air redevient un seul souffle, net. La larme de bronze ne bouge plus, du tout. Le tilleul n'a plus claqué. Maintenant, tu peux rester. Plate, la coupelle attend, sans verser. Tu as laissé les feuilles finir.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;On attend les &lt;emphasis level="moderate"&gt;feuilles&lt;/emphasis&gt;, d'abord. Elle tient la coupelle, puis attend les feuilles. Les feuilles vont, reviennent, puis se taisent. L'air redevient un seul souffle, net. La larme de bronze ne bouge plus, du tout. Le tilleul n'a plus claqué. Maintenant, tu peux rester. Plate, la coupelle attend, sans verser. Elle couvre le bol avec sa paume. Ma main garde le miroir. Tu as laissé les feuilles finir.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>On attend les &lt;emphasis&gt;feuilles&lt;/emphasis&gt;, d'abord. Elle tient la coupelle, puis attend les feuilles. Les feuilles vont, reviennent, puis se taisent. L'air redevient un seul souffle, net. La larme de bronze ne bouge plus, du tout. Le tilleul n'a plus claqué. Maintenant, tu peux rester. Plate, la coupelle attend, sans verser. Tu as laissé les feuilles finir. [pause]</t>
+          <t>On attend les &lt;emphasis&gt;feuilles&lt;/emphasis&gt;, d'abord. Elle tient la coupelle, puis attend les feuilles. Les feuilles vont, reviennent, puis se taisent. L'air redevient un seul souffle, net. La larme de bronze ne bouge plus, du tout. Le tilleul n'a plus claqué. Maintenant, tu peux rester. Plate, la coupelle attend, sans verser. Elle couvre le bol avec sa paume. Ma main garde le miroir. Tu as laissé les feuilles finir. [pause]</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr"/>
@@ -16355,6 +16439,8 @@
 papa|Le tilleul n'a plus claqué.
 enfant-f|Maintenant, tu peux rester.
 narrateur|Plate, la coupelle attend, sans verser.
+narrateur|Elle couvre le bol avec sa paume.
+enfant-f|Ma main garde le miroir.
 maman|Tu as laissé les feuilles finir.</t>
         </is>
       </c>
@@ -16572,17 +16658,17 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Derrière, pas trop près du vent. Derrière le tronc, la coupelle ne se plie plus. Nina se glisse derrière le tronc, tout bas. Rien ne claque, rien ne pousse plus. La larme de bronze se voit entre deux branches. Tu n'as pas couru. Tu es ronde, maintenant. Le rond de savon attend, abrité. Derrière, l'air était plus doux.</t>
+          <t>Derrière, pas trop près du vent. Derrière le tronc, la coupelle ne se plie plus. Nina se glisse derrière le tronc, tout bas. Rien ne claque, rien ne pousse plus. La larme de bronze se voit entre deux branches. Tu n'as pas couru. Tu es ronde, maintenant. Le rond de savon attend, abrité. Elle pose le bol au pied du tronc. Le tronc garde le miroir. Derrière, l'air était plus doux.</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Derrière, pas trop près du vent. Derrière le tronc, la coupelle ne se plie plus. Nina se glisse &lt;emphasis level="moderate"&gt;derrière&lt;/emphasis&gt; le tronc, tout bas. Rien ne claque, rien ne pousse plus. La larme de bronze se voit entre deux branches. Tu n'as pas couru. Tu es ronde, maintenant. Le rond de savon attend, abrité. Derrière, l'air était plus doux.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Derrière, pas trop près du vent. Derrière le tronc, la coupelle ne se plie plus. Nina se glisse &lt;emphasis level="moderate"&gt;derrière&lt;/emphasis&gt; le tronc, tout bas. Rien ne claque, rien ne pousse plus. La larme de bronze se voit entre deux branches. Tu n'as pas couru. Tu es ronde, maintenant. Le rond de savon attend, abrité. Elle pose le bol au pied du tronc. Le tronc garde le miroir. Derrière, l'air était plus doux.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>Derrière, pas trop près du vent. Derrière le tronc, la coupelle ne se plie plus. Nina se glisse &lt;emphasis&gt;derrière&lt;/emphasis&gt; le tronc, tout bas. Rien ne claque, rien ne pousse plus. La larme de bronze se voit entre deux branches. Tu n'as pas couru. Tu es ronde, maintenant. Le rond de savon attend, abrité. Derrière, l'air était plus doux. [pause]</t>
+          <t>Derrière, pas trop près du vent. Derrière le tronc, la coupelle ne se plie plus. Nina se glisse &lt;emphasis&gt;derrière&lt;/emphasis&gt; le tronc, tout bas. Rien ne claque, rien ne pousse plus. La larme de bronze se voit entre deux branches. Tu n'as pas couru. Tu es ronde, maintenant. Le rond de savon attend, abrité. Elle pose le bol au pied du tronc. Le tronc garde le miroir. Derrière, l'air était plus doux. [pause]</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr"/>
@@ -16724,6 +16810,8 @@
 papa|Tu n'as pas couru.
 enfant-f|Tu es ronde, maintenant.
 narrateur|Le rond de savon attend, abrité.
+narrateur|Elle pose le bol au pied du tronc.
+enfant-f|Le tronc garde le miroir.
 maman|Derrière, l'air était plus doux.</t>
         </is>
       </c>
@@ -16941,17 +17029,17 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Tout petit, tout serré. Une toute petite bulle quitte la coupelle. Nina souffle à peine, sans prendre le vent. Le tilleul se tait, plus loin, tout seul. La larme de bronze prend le petit rond. Le petit rond n'a pas volé. Tu restes, bulle. Le rond de savon attend, minuscule. Le petit rond a suffi.</t>
+          <t>Tout petit, tout serré. Une toute petite bulle quitte la coupelle. Nina souffle à peine, sans prendre le vent. Le tilleul se tait, plus loin, tout seul. La larme de bronze prend le petit rond. Le petit rond n'a pas volé. Tu restes, bulle. Le rond de savon attend, minuscule. Elle prend un tout petit cercle, au bord. Un petit miroir, pour la larme. Le petit rond a suffi.</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Tout petit, tout serré. Une toute petite bulle quitte la coupelle. Nina souffle à peine, sans prendre le vent. Le tilleul se tait, plus loin, tout seul. La larme de bronze prend le petit rond. Le petit rond n'a pas volé. Tu restes, bulle. Le rond de savon attend, minuscule. Le petit rond a suffi.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Tout petit, tout serré. Une toute petite bulle quitte la coupelle. Nina souffle à peine, sans prendre le vent. Le tilleul se tait, plus loin, tout seul. La larme de bronze prend le petit rond. Le petit rond n'a pas volé. Tu restes, bulle. Le rond de savon attend, minuscule. Elle prend un &lt;emphasis level="moderate"&gt;tout petit&lt;/emphasis&gt; cercle, au bord. Un petit miroir, pour la larme. Le petit rond a suffi.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>Tout petit, tout serré. Une toute petite bulle quitte la coupelle. Nina souffle à peine, sans prendre le vent. Le tilleul se tait, plus loin, tout seul. La larme de bronze prend le petit rond. Le petit rond n'a pas volé. Tu restes, bulle. Le rond de savon attend, minuscule. Le petit rond a suffi. [pause]</t>
+          <t>Tout petit, tout serré. Une toute petite bulle quitte la coupelle. Nina souffle à peine, sans prendre le vent. Le tilleul se tait, plus loin, tout seul. La larme de bronze prend le petit rond. Le petit rond n'a pas volé. Tu restes, bulle. Le rond de savon attend, minuscule. Elle prend un &lt;emphasis&gt;tout petit&lt;/emphasis&gt; cercle, au bord. Un petit miroir, pour la larme. Le petit rond a suffi. [pause]</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr"/>
@@ -17093,6 +17181,8 @@
 papa|Le petit rond n'a pas volé.
 enfant-f|Tu restes, bulle.
 narrateur|Le rond de savon attend, minuscule.
+narrateur|Elle prend un tout petit cercle, au bord.
+enfant-f|Un petit miroir, pour la larme.
 maman|Le petit rond a suffi.</t>
         </is>
       </c>
@@ -17304,7 +17394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17424,6 +17514,13 @@
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>